<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 6, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1316,8 +1316,664 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1168692108</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>【正規品】松の木 鎮静 シカ クレンザー 150ml</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="b">
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168692108</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1164469069</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>【正規品】グリーンシカ コラーゲン クリアフォーム 2.0 300ml</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>3690</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="b">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164469069</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1163729695</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>【正規品】ディープポア クレンジング ソーダフォーム 150ml</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>3590</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="b">
+        <v>0</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163729695</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1205554253</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>【正規品】トラネキサム酸スキンブースタークリーム 100ml</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>メディテラピー</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>4990</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205554253</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1193459511</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>【正規品】レチノコラーゲン低分子300ネックカッサクリーム 50ml (2個)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>CKD_GUARANTEED</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>6490</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="b">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193459511</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1210771223</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PLUS82</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>マデカクリーム イン バブルセラム 100ml+100ml（+マデカパウダー ビタグルシ 6g）</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>6273</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="b">
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210771223</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1206008325</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>DreamWish</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ペプチドショット2X 弾力アンプル 30ml（ハリ感ケア／保湿／弾力サポート美容液）</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>アンプルエヌ</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>2122</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="b">
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206008325</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1206008294</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DreamWish</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ウォーターフィット リカバー BBクリーム 30ml #SPF40 PA+++ #保湿密着</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>セルフュージョンC</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>2927</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="b">
+        <v>0</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206008294</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1205912921</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>DreamWish</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>レチンアルブースターショット 30ml+30ml #レチナール2.0% #セラミド #エクトイン #カフェイン #ペプチド</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>アレンシア</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>4046</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" t="b">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205912921</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1205483331</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>COCOAN</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>【1+1セット】成分エディターグリーントマト NMN フォアリフティングアンプル 40ml+40ml / 毛穴のしわ 弾力 エッセンス 美容液 グリーントマト</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>グリーントマト</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="b">
+        <v>0</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205483331</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1205132300</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>COCOAN</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>[1個]ダークスポットセラム30ml (ナイアシンアミド10%, トラネキサム酸 4%)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>2350</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205132300</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1107510664</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>KSB</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>[新作]ムード レイヤー スティック クレヨン 5color 00 milky syrup 01 caramel drizzle 02 rose milk tea 03 mauve latte</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>alternative stereo</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>2405</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" t="b">
+        <v>0</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1107510664</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>1154233546</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>jullyland</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ダークスポットセラム (ナイアシンアミド10%, トラネキサム酸 4%) 30ml/韓国コスメ/アンプル</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>2580</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="b">
+        <v>0</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154233546</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1188839770</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>[保湿 保水 栄養 シートマスク 10枚 5種類から選択] 高保湿 まとめ買い 夜用 デイリー スキンケア</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1709</v>
+      </c>
+      <c r="G35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" t="b">
+        <v>0</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188839770</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>1197460025</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>【1+1 クリームミスト 120ml】保湿ミスト 化粧水ミスト うるおいケア 整肌ケア スプレー 韓国スキンケア デイリーケア</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>3899</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="b">
+        <v>0</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197460025</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>1188077394</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>[秀麗な本超保湿クリーム 50ml] 韓国漢方 高保湿 エイジングケア シワ/改/善 /弾力アップ しっとり濃密テクスチャー</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>秀麗韓</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>4427</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="b">
+        <v>0</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188077394</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J21"/>
+  <autoFilter ref="A1:J37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 9, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1972,8 +1972,623 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>1147146315</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>jinytrading</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>PDRN ピンク グルタチオン セラム ミスト 100ml 水分 保湿 弾力 韓国化粧品 韓国美容ギフト</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>2961</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="b">
+        <v>0</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1147146315</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>1159784308</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>jinytrading</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ビタCプラス アスコルビン酸 クリアコンプレクション フォーミングクレンザー 120ml 高濃度ビタミンC フォームクレンジング 水分 保湿 韓国化粧品 韓国美容ギフト</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>1971</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="b">
+        <v>0</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159784308</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>1198095545</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>leekorea</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>【GIFT】洗顔/ゼロ 毛穴 ブラックヘッド ディープ クレンジングオイル 205ml/毛穴ケア/毛穴 黒ずみ/ブラックヘッド/韓国コスメ 毛穴</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="b">
+        <v>0</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198095545</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>1209903581</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>leekorea</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>【ニキビケア】1番 パントテン酸アクティブスージングクリーム 80ml/ニキビ</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="b">
+        <v>0</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209903581</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>1110469138</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>leekorea</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>【5種沢1】CICA/PDRN/毛穴/ニキビケア/保湿／トナーパット／鎮静／トナー／化粧水/毛穴ケア/ふき取り化粧水/メが割/美容液</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>2995</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="b">
+        <v>0</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1110469138</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>1203205247</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>vanguardvista</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>[正規品] 人気 おすすめ 韓国 クリーム Rx 30ml+7ml セット スキンケア クリーム ギフト</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ドミナス</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>5820</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="b">
+        <v>0</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203205247</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>1207091863</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>リードルショット フォーメン オールインワン100 Mプラス 150ml＋30ml 企画セット メンズスキンケア 韓国コスメ 化粧水 乳液 美容液</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>3855</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="b">
+        <v>0</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207091863</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>1174137858</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ローズマリー &amp;amp; シーソルト &amp;amp; AHA シャンプー 500ml × 2本セット 韓国シャンプー スカルプケア 頭皮クレンジング ボリュームケア</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>オーガニスト</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>2899</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="b">
+        <v>0</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174137858</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>1024539184</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>[1+1]ハニーアンドマカデミア ネイチャーシャンプー 500ml+プロテイントリートメント 500mlホワイトムスクの香り</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>3480</v>
+      </c>
+      <c r="G46" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" t="b">
+        <v>0</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1024539184</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>1207091851</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>3番 ノーファンデ陶器肌トーンアップUVクリーム 50ml (SPF50+ PA++++) / トーンケアクリーム 保湿ベース 水分クリーム 化粧下地 ナチュラルトーンアップ</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>3995</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="b">
+        <v>0</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207091851</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>1174312286</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>sinature23</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>【1+1】【韓国コスメ】【正規品扱い店】[病院専用] ラポラピルナトックス 50ml - シミ改善＆肌トーンアップの機能性クリーム！</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Dermagen</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>7128</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="b">
+        <v>0</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174312286</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>1146499682</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>sinature23</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【正規品扱い店】タイムエナジーリセッティングエマルジョン 120ml - 時間を超える美肌の秘訣！</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>sum37</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>4781</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="b">
+        <v>0</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146499682</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>1146499598</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>sinature23</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【正規品扱い店】[5番企画セット] 白玉リンガーグルタチオンCトナー200ML ＋ 白玉グルタチオンC美容液30ML - 輝く美肌へ導く！</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>7013</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" t="b">
+        <v>0</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146499598</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>1145594895</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>sinature22</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>【正規品扱い店】【1+1】【本品+レフィル】ダイブイン低分子ヒアルロン酸セラム, 50mL*2</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>4879</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" t="b">
+        <v>0</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145594895</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>1145594718</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>sinature22</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【正規品扱い店】シルクペプチドインテンシブリフティングアンプル35ML</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Sung Boon Editor</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>2407</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" t="b">
+        <v>0</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145594718</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J37"/>
+  <autoFilter ref="A1:J52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 12, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2587,8 +2587,705 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>1165444330</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>saleb</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>アヌカチン シャンプー 525ml</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>moev</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>5150</v>
+      </c>
+      <c r="G53" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" t="b">
+        <v>0</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165444330</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>1179699936</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>saleb</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>[輪郭アンプル] コアタイムアンプル 15ml (+7ml)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>NEURADERM</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>4340</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" t="b">
+        <v>0</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179699936</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>1165596313</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>saleb</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>[1+1] 黒雲 毛根強化アンドボリュームケアシャンプー 500ml</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>呂</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>3470</v>
+      </c>
+      <c r="G55" t="n">
+        <v>3</v>
+      </c>
+      <c r="H55" t="b">
+        <v>0</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165596313</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>1165513951</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>saleb</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>マダガスカル センテラ クイック カーミングパッド 70枚</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>3750</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" t="b">
+        <v>0</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165513951</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>1165361801</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>saleb</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>[1+1] コルツフート アンチダンドラフ シャンプー 200ml</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>ラウシュ</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>6570</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" t="b">
+        <v>0</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165361801</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>1207091316</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>manmulsang</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>レチノールスーパーバウンスセラム 20ml＋15ml 企画セット 初めてのレチノールケア 昼夜使いやすい 美容液 メイク前 なめらか肌印象 韓国コスメ スポイトタイプ 水分感 クリーム前 スキンケア</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>アイオペ</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>5324</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="b">
+        <v>0</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207091316</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>1210932470</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>refill</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>ブルー EGF カーミングミスト 100ml 韓国フェイスミスト 化粧水ミスト うるおいケア 肌コンディションケア</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>dear,Klairs</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>3599</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="b">
+        <v>0</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210932470</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>1198423707</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>refill</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>ポリジェン シークニング スカルプ コンディショニングマスク 200ml / 頭皮ケア ボリュームアップケア ハリコシ ダメージケア 保湿 しっとり サロンケア ヘアパック スカルプパック</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>3296</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="b">
+        <v>0</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198423707</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>1211212429</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>refill</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>セルアップ マイクロ フォームクレンザー 120ml 2個＋クレンジングミルク20ml 韓国洗顔フォーム 洗顔料 毛穴汚れケア うるおい洗顔</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ラゴム</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>3899</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="b">
+        <v>0</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211212429</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>1196826611</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>OliveYouth</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>ブルービーン B5-PDRN マイルドローション 230ml / 保湿乳液 敏感肌対応 うるおいケア スキンケアローション 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>2999</v>
+      </c>
+      <c r="G62" t="n">
+        <v>3</v>
+      </c>
+      <c r="H62" t="b">
+        <v>0</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196826611</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>1164705875</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>OliveYouth</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>ウォータープルーフプロ日焼け止め 50g+サンスティック 20g / アウトドア スポーツ対応UVクリーム 汗・水に強いスティックタイプ 手を汚さない</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>5499</v>
+      </c>
+      <c r="G63" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" t="b">
+        <v>0</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164705875</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>1187759601</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>joungho</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>【韓国旅行の定番】垢すり石鹸＆グローブ6個セットまるで韓国エステ！自宅で叶う極上のツルツル美肌体験</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ダイソー</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G64" t="n">
+        <v>2</v>
+      </c>
+      <c r="H64" t="b">
+        <v>0</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187759601</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>1194068552</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>joungho</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>韓国国民アイテム キュアアルファカーミングアロエクリーム 50g 2個</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>CURE</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="b">
+        <v>0</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194068552</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>1183178551</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Starlit</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>TN トラネキサミン5%＋ナイアシンアミド5% ブライトニング セラム60ml</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>コスデバハ</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>3880</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="b">
+        <v>0</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183178551</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>1188405527</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Starlit</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>ゆずグレープフルーツ ビーガン パッククレンザー 80g+毛穴ブラシ [毛穴ケア+洗顔+すっきり]</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ホイップド</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>3680</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="b">
+        <v>0</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188405527</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>1080770379</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>NARShA</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>ライトオンインシャワーボディトーンアップボディローション ベビーパウダーの香り290ml</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>4720</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="b">
+        <v>0</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1080770379</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>1206876054</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>NARShA</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>[ブラシ元祖] グロウターンエクソソームブラシアンプル130ml企画(+30ml)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>lily eve</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>5950</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="b">
+        <v>0</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206876054</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J52"/>
+  <autoFilter ref="A1:J69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 15, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3284,8 +3284,664 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1206207561</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>durudurupanda</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>[1+1] トーンアップ パールクリーム 本体30g+30g スキンケア / 保湿 / ベースメイク韓国コスメ 並行輸入</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>MAY ISLAND</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>3530</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="b">
+        <v>0</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206207561</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>1205776987</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>durudurupanda</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>AGE-R グルタチオン グロウ カプセル クリーム 50ml 保湿 スキンケア 並行輸入</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>3530</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="b">
+        <v>0</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205776987</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>1199084782</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>durudurupanda</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ヴィーガンコンブチャ ティー エッセンス 150ml 保湿 しっとり エッセンス 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Dr.Ceuracle</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>3380</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" t="b">
+        <v>0</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199084782</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>1198940759</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>durudurupanda</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Relief Sun Aqua-Fresh : Rice + B5 アクアフレッシュ UVクリーム 50ml 米 うるおい 日焼け止め</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>2240</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" t="b">
+        <v>0</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198940759</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>1195384789</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>durudurupanda</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>24K ゴールド トナー 保湿 化粧水 120ml 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>アンジョ</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>1570</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" t="b">
+        <v>0</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195384789</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>1172312020</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>hokkorikorea</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>【SALE】【毛穴ケア】PDRN毛穴弾力パッド 100枚 ハリ感 キメ整う エイジングケア ツヤ肌 角質ケア うるおい 人気 韓国コスメ 大容量 毎日ケア 時短 敏感肌OK 透明感 キメケア 保湿</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>3006</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" t="b">
+        <v>0</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172312020</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>1193625970</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>glowbox</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>【公式】 グロウオイルミスト 50ml うるおい×ツヤ肌キープ</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>5990</v>
+      </c>
+      <c r="G76" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" t="b">
+        <v>0</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193625970</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>1206859281</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>hikoreashop</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ポアブライトニングシミケアクリームマスク, 4枚 /ブライトニング/韓国マスクパック/ナイアシンアミド/保湿/水分/肌トーン改善/顔の頬リフ</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>2780</v>
+      </c>
+      <c r="G77" t="n">
+        <v>1</v>
+      </c>
+      <c r="H77" t="b">
+        <v>0</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206859281</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>1203000979</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>hikoreashop</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>大豆エッセンス, 50ml</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ミクスン</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G78" t="n">
+        <v>1</v>
+      </c>
+      <c r="H78" t="b">
+        <v>0</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203000979</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>1198208356</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>hikoreashop</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>アヌカチンシャンプー, 300ml</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>moev</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1775</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" t="b">
+        <v>0</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198208356</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>1117793591</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>OLIVIASHOP</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>【正規品/ PDRNスペシャル 3種 鎮静 セット】PDRNリジュビネイティングトナー 300ml+ビタトーニングアンプル 30ml+ジュビネイティングクリーム 70ml/鎮静/保湿/回復/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ジェナベール</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>11749</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" t="b">
+        <v>0</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1117793591</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>1138030129</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>OLIVIASHOP</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>【正規品】345リリーフクリーム, 50mlニキビ肌鎮静デイリークリーム relief cream</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ドクターエルシア</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>2680</v>
+      </c>
+      <c r="G81" t="n">
+        <v>2</v>
+      </c>
+      <c r="H81" t="b">
+        <v>0</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138030129</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>1210577063</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>wingkone</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>【正規品】【NEW】【脱色/染め】 眉毛脱色 イージーブロウトーンチェンジャー 5回分 / イージーブロウムードチェンジャー 5回分 / アイブロウ / 韓国コスメ / 眉毛</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>コスノリ</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>1810</v>
+      </c>
+      <c r="G82" t="n">
+        <v>3</v>
+      </c>
+      <c r="H82" t="b">
+        <v>0</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210577063</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>1202057165</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>thenido</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>[1+1] インフューズド コラーゲン コンセントレート フルイド 50ml 2件</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>BEAUDIANI</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>4428</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" t="b">
+        <v>0</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202057165</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>1202051148</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>thenido</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>インフュージングコラーゲンパウダー, 1.5g</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>BEAUDIANI</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>3258</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" t="b">
+        <v>0</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202051148</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>1202043668</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>thenido</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>[1+1] インフュージングコラーゲンミスト 50ml 2件</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>BEAUDIANI</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>4473</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="b">
+        <v>0</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202043668</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J69"/>
+  <autoFilter ref="A1:J85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 18, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3940,8 +3940,664 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>1206008183</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>247GOODLUCK</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>ナイアシン トラネキサム酸13% セラム 30ml／トーンアップケア／肌荒れケア</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>1565</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" t="b">
+        <v>0</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206008183</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>1203846979</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>247GOODLUCK</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>PDRN エアクラウド メラケア サンスクリーン 50ml #SPF50+ PA++++ #アルブチン #トラネクサン酸 #ナイアシンアミド #エラスチン #コラーゲン</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>3480</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" t="b">
+        <v>0</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203846979</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>1157418989</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>busanjin</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>ゼロ毛穴 黒ずみ マッドパック 100g #AHA+BHA+PHA</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" t="b">
+        <v>0</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157418989</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>1205905548</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>FROM051</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>メラレイジングアンプルクリーム 56g #シミケア #ナイアシンアミド #トラネキサム酸 #8種ヒアルロン酸</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>シャルド</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>5883</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" t="b">
+        <v>0</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205905548</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>1205520797</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>siriya</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>ポアコントロール131 クレンジングオイル200ml／毛穴ケア／皮脂バランス</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>3153</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" t="b">
+        <v>0</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205520797</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>1204558349</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>siriya</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>リポソームバブルブースター 95ml 2種（コラーゲン／キャビア PDRN）から1つ選択</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>3498</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" t="b">
+        <v>0</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204558349</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>1208085435</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>VividgrowMAN</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>[26SS/New]クリアライスサンスクリーン 50ml（+20ml＋チュンシキキーホルダー）</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" t="b">
+        <v>0</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208085435</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>1208085817</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>VividgrowMAN</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>(ポケモンエディション)体臭ソリューション デオドラント ボディウォッシュ 720ml 2種から1つ選択</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>46CM</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>2889</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" t="b">
+        <v>0</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208085817</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>1199735232</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>VividgrowMAN</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>PDRNピンクエクソソームショット2000, 30ml</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" t="b">
+        <v>0</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199735232</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>1191662969</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>bloomingseoul</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>ブルービーン B5-PDRN マイルドローション 230ml(+ブルービーンクリーム7ml)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>2374</v>
+      </c>
+      <c r="G95" t="n">
+        <v>3</v>
+      </c>
+      <c r="H95" t="b">
+        <v>0</v>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191662969</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>1209320737</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>FaceiD</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>[2PACK] クリーンイットゼロ 抹茶クレンジングバーム 100ml</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>バニラコ</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>4555</v>
+      </c>
+      <c r="G96" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" t="b">
+        <v>0</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209320737</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>1201575924</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>FaceiD</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>[26SS/New]ピーチフェア ビーガン トーンアップ カプセルサンスクリーン 50ml #SPF50+ PA++++ #グルタチオン #ナイアシンアミド</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>ホイップド</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>3353</v>
+      </c>
+      <c r="G97" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" t="b">
+        <v>0</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201575924</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>1201571343</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>FaceiD</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>[25SS/新作]4GF ザマ リペア ハイドロ セラム 30ml #エクソソーム #ナイアシンアミド #ペプチド #ノンコメドジェニック</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>CELORABY</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>5397</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" t="b">
+        <v>0</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201571343</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>1190875712</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>DEdge</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>[26SS/New]セビウム セラム 30ml（+センシビオ H2O 5ml×2）</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>ビオデルマ</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>6600</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" t="b">
+        <v>0</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190875712</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>1190240492</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>DEdge</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>アップルタチオン トニング トナー パッド 60枚 #独自特許原料アップルタチオン #リンゴエキス+アロエ+高純度グルタチオン #鎮静</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>farmic</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>5168</v>
+      </c>
+      <c r="G100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" t="b">
+        <v>0</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190240492</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>1152717704</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>DEdge</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>[26SS/New]ボディタミン アルファ ブライトニング スポット ボディセラム 80ml #ナイアシンアミド10%</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>ビヨンド</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>2948</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" t="b">
+        <v>0</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152717704</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J85"/>
+  <autoFilter ref="A1:J101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 21, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$117</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:J117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4596,8 +4596,664 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>1125754461</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>[1+1]レッドブレミッシュクリアスージングクリーム 50ml 2個+10ml 2個/正規品</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>3469</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" t="b">
+        <v>0</v>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1125754461</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>1212553298</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>【正規品+GIFT付き】リードルショット コラーゲンクリーム 50ml＋スティックパウチ 3個</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>3021</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" t="b">
+        <v>0</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212553298</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>1212350487</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>[1+1]MEDI AHAイボ取りクリーム25ml 2個&amp;nbsp; / メディオルガ稗粒腫スポットクリーム/ポツポツちびイボ</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>3666</v>
+      </c>
+      <c r="G104" t="n">
+        <v>0</v>
+      </c>
+      <c r="H104" t="b">
+        <v>0</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350487</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>1212350471</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>[1+1]メディオルガブライトニングクリーム30ml 2個/しみ取りクリーム お肌のトーンアップ</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>3055</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" t="b">
+        <v>0</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350471</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>1212350473</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>MEDI AHAイボ取りクリーム25ml/ メディオルガ稗粒腫スポットクリーム/ポツポツちびイボ</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>2331</v>
+      </c>
+      <c r="G106" t="n">
+        <v>1</v>
+      </c>
+      <c r="H106" t="b">
+        <v>0</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350473</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>1172083985</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>KBEAT</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>【公式】ティーツリー グリーン ボディウォッシュ 500ml</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>原料工房</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>3739</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" t="b">
+        <v>0</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172083985</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>1194074735</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>octaglobal</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>PDRN ヒアルロン酸カプセル100 セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" t="b">
+        <v>0</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194074735</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>1213314755</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>cosone</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>[1+1] エアリーフィットサンスティック　/　2個入り</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>KAHI</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>3801</v>
+      </c>
+      <c r="G109" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" t="b">
+        <v>0</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213314755</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>1213007507</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>cosone</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>エアリーフィットサンスティック</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>KAHI</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>2077</v>
+      </c>
+      <c r="G110" t="n">
+        <v>0</v>
+      </c>
+      <c r="H110" t="b">
+        <v>0</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213007507</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>1208546349</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>cosone</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>[1+1] ピュアクレンジングオイル 200ml　/　2個入り</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>3400</v>
+      </c>
+      <c r="G111" t="n">
+        <v>0</v>
+      </c>
+      <c r="H111" t="b">
+        <v>0</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208546349</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>1204555836</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>cosone</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>PDRNビタペプチド毛穴リペアセラム, 35ml</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>dear,Klairs</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G112" t="n">
+        <v>2</v>
+      </c>
+      <c r="H112" t="b">
+        <v>0</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204555836</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>1201560856</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>[NEW] PDRN カフェイン 1000 オーバーナイト ラッピング マスク 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>P.CALM</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>4100</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" t="b">
+        <v>0</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201560856</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>1208992240</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>[NEW] マイルド ヴィーガン トーンアップ 日焼け止め 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>コスノリ</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" t="b">
+        <v>0</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208992240</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>1191141866</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>[NEW] スーパー コラーゲン バブル セラム マスク 90g 1個</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>AROCELL</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>5550</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" t="b">
+        <v>0</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191141866</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>1168717728</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>[新商品] キャロット カロチン モイスト エフェクター 55ml 1個</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>4900</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" t="b">
+        <v>0</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168717728</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>1146804177</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>[正品] ゼロ 毛穴 ブラックヘッド ディープ クレンジングオイル 205ml 1個</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G117" t="n">
+        <v>0</v>
+      </c>
+      <c r="H117" t="b">
+        <v>0</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146804177</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J101"/>
+  <autoFilter ref="A1:J117"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 24, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$126</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J117"/>
+  <dimension ref="A1:J126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5252,8 +5252,377 @@
         </is>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>1160418590</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>julynana</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>[2種セット]ブリングリーン ティーツリー シカスージングトナー 250ml + クリーム100ml</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>3510</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0</v>
+      </c>
+      <c r="H118" t="b">
+        <v>0</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160418590</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>1152030824</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>julynana</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>[人気2種セット]ホワイトトリュフファーストスプレーセラム 100ml +ウォータフルトーンアップサンクリーム50ml</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>5640</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0</v>
+      </c>
+      <c r="H119" t="b">
+        <v>0</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152030824</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>1211694332</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>blanc-lapin</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>ジュリーク JURLIQUE RO バランシングミスト 100ml 化粧水 [169628]</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>ジュリーク</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>4460</v>
+      </c>
+      <c r="G120" t="n">
+        <v>0</v>
+      </c>
+      <c r="H120" t="b">
+        <v>0</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211694332</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>1205909859</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>blanc-lapin</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>【本体フィルム剥がれあり】クラランス CLARINS グランアイセラムV 15ml [448368]</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>クラランス</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>5580</v>
+      </c>
+      <c r="G121" t="n">
+        <v>0</v>
+      </c>
+      <c r="H121" t="b">
+        <v>0</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205909859</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>1191657535</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>seoulglowpick</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>シカケア クリア アンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>ロベクチン</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" t="b">
+        <v>0</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191657535</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>1191655869</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>seoulglowpick</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>[新作]オールデイ ノーセバム トーンアップ サンクッション 2種 SPF45 PA++++ lilac fog vanilla lemon</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>ミルクタッチ</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>3982</v>
+      </c>
+      <c r="G123" t="n">
+        <v>0</v>
+      </c>
+      <c r="H123" t="b">
+        <v>0</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191655869</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>1188483946</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>seoulglowpick</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>キャロット カロテン デイリーマスク 30枚 #毎日使える栄養たっぷりのフェイスマスク</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>3777</v>
+      </c>
+      <c r="G124" t="n">
+        <v>0</v>
+      </c>
+      <c r="H124" t="b">
+        <v>0</v>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188483946</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>1203329038</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>beauty69</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>【新作】スムース＆ピュア アイス クーリング デオ スプレー 150ml 2種</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>アリウル</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>1581</v>
+      </c>
+      <c r="G125" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" t="b">
+        <v>0</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203329038</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>1210434904</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>beauty69</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>[新作] NAD フリーズセル グロウブーストクリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>5390</v>
+      </c>
+      <c r="G126" t="n">
+        <v>0</v>
+      </c>
+      <c r="H126" t="b">
+        <v>0</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210434904</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J117"/>
+  <autoFilter ref="A1:J126"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 3, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$135</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J126"/>
+  <dimension ref="A1:J135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5621,8 +5621,377 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>1210877861</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>K_Beauty_Station</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>【NEW・化粧ノリUPミスト】シェイキングシナジーミスト 50ml 3種</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>2438</v>
+      </c>
+      <c r="G127" t="n">
+        <v>0</v>
+      </c>
+      <c r="H127" t="b">
+        <v>0</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210877861</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>1197720706</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>K_Beauty_Station</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>【今だけ限定！企画】キャロットカロテンカーミングウォーターパッド, 60枚</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>1964</v>
+      </c>
+      <c r="G128" t="n">
+        <v>3</v>
+      </c>
+      <c r="H128" t="b">
+        <v>0</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197720706</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>1142629949</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>zozoro0213</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>セラ 水分バリア 日焼け止め SPF50+ PA++++ 50ml x 2個 (鎮静/弾力/保湿/栄養供給/活力/しわ防止)</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>リアルバリア</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0</v>
+      </c>
+      <c r="H129" t="b">
+        <v>0</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142629949</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>1212154617</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>gmarketplus</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>belif ビリーフ ザ・トゥルー クリーム モイスチャライジングバーム 50ml（保湿クリーム） (贈呈品なくなり次第贈呈終了)</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>ビリーフ</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>5170</v>
+      </c>
+      <c r="G130" t="n">
+        <v>0</v>
+      </c>
+      <c r="H130" t="b">
+        <v>0</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212154617</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>1207926681</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>gmarketplus</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>トリデン バランスフル シカ 鎮静クリーム 80ml(贈呈品なくなり次第贈呈終了)</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>3995</v>
+      </c>
+      <c r="G131" t="n">
+        <v>0</v>
+      </c>
+      <c r="H131" t="b">
+        <v>0</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207926681</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>1210186472</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>gmarketplus</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>ポリジェン シックニング ボリューム強化 スカルプトニック 120ml (贈呈品なくなり次第贈呈終了)</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>3775</v>
+      </c>
+      <c r="G132" t="n">
+        <v>0</v>
+      </c>
+      <c r="H132" t="b">
+        <v>0</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210186472</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>1207682253</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>resear</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>【4種から選べる】リッサー バイオミラパッド 10枚入り (ポアピーリング / シカカーミング / ビタシャイニング / トリプルショット) 鎮静・透明感・毛穴・ハリケア 韓国スキンケア トナーパッド</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>resear</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G133" t="n">
+        <v>0</v>
+      </c>
+      <c r="H133" t="b">
+        <v>0</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207682253</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>1209235398</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>エクソソーム保湿クリーム 50ml 韓国コスメ 韓国ブランド 公式ショップ 韓国スキンケア スキンケア 化粧品 敏感肌 乾燥肌 水分ケア うるおい 韓国アンプル ギフト PDRN CICA</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>2664</v>
+      </c>
+      <c r="G134" t="n">
+        <v>0</v>
+      </c>
+      <c r="H134" t="b">
+        <v>0</v>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209235398</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>1209222941</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>エクソソーム保湿トナー 150ml 韓国スキンケア 韓国コスメ スキンケア PDRN CICA ヒアルロン酸 水分ケア　乾燥肌 ローション 化粧水 整肌成分 毎日のケア 弱酸性 韓国商品 高保湿</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>2472</v>
+      </c>
+      <c r="G135" t="n">
+        <v>0</v>
+      </c>
+      <c r="H135" t="b">
+        <v>0</v>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209222941</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J126"/>
+  <autoFilter ref="A1:J135"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 27, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$376</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$390</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J376"/>
+  <dimension ref="A1:J390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15871,8 +15871,582 @@
         </is>
       </c>
     </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>1135668857</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>koco_store</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>[韓国人気保湿クリーム] グルカミュー(Glucamune)クリーム, 100ml (水分鎮静/スキンケア)</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F377" t="n">
+        <v>5833</v>
+      </c>
+      <c r="G377" t="n">
+        <v>0</v>
+      </c>
+      <c r="H377" t="b">
+        <v>0</v>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135668857</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>1188760323</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Lumora</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>ビタミン10PORESTRIXセラム, 20ml ビタミンC 美容液 ビタミンC セラム エッセンス 透明感 毛穴ケア 艶肌 低刺激 導入液 潤い 敏感肌 スキンケア 導入美容液 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F378" t="n">
+        <v>4250</v>
+      </c>
+      <c r="G378" t="n">
+        <v>0</v>
+      </c>
+      <c r="H378" t="b">
+        <v>0</v>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188760323</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>1188183806</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Lumora</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>ライス 70 グロウ ミルキー トナー 250ml 化粧水 米ぬか セラミド 艶肌 もちもち 潤いバリア 高浸透 インナードライ スキンケア 低刺激 乾燥肌 混合肌 韓国コスメ 導入液</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F379" t="n">
+        <v>3790</v>
+      </c>
+      <c r="G379" t="n">
+        <v>0</v>
+      </c>
+      <c r="H379" t="b">
+        <v>0</v>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188183806</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>1194595746</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Lumora</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>(50%容量プレゼント)ダーマUV365バリアハイドロミネラルサンスクリーン, (40ml+20ml)/ 低刺激 UVカット 敏感肌 保湿 バリア機能 ノンナノ 紫外線散乱剤 白浮きしない ドクターズ</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F380" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G380" t="n">
+        <v>0</v>
+      </c>
+      <c r="H380" t="b">
+        <v>0</v>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194595746</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>1192065873</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Lumora</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>[2個セット/大容量] PDRNリードルショットブラシヘアセラム 100ml×2 / 頭皮ケア スカルプケア 美容液 まとめ買い お得セット</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F381" t="n">
+        <v>6980</v>
+      </c>
+      <c r="G381" t="n">
+        <v>0</v>
+      </c>
+      <c r="H381" t="b">
+        <v>0</v>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192065873</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>1188758518</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Lumora</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>【2個セット】 ナイアシンアミド10%ダークスポットセラム, 30ml×2本 美容液 ダークスポットケア エッセンス 透明感 毛穴ケア 艶肌 低刺激 導入液 潤い ス킨ケア まとめ買い セット商品 韓</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F382" t="n">
+        <v>6989</v>
+      </c>
+      <c r="G382" t="n">
+        <v>0</v>
+      </c>
+      <c r="H382" t="b">
+        <v>0</v>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188758518</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>1161204302</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>kinakomall</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>[正規品]ドリクロ 20ml/脇汗デオドラント/デオドラント/脇汗/制汗剤/脇汗 韓国</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Driclor</t>
+        </is>
+      </c>
+      <c r="F383" t="n">
+        <v>1718</v>
+      </c>
+      <c r="G383" t="n">
+        <v>1</v>
+      </c>
+      <c r="H383" t="b">
+        <v>0</v>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1161204302</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>1194293129</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>hancony</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>ナイアシンアミド20 セラム 40ml</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>JUMISO</t>
+        </is>
+      </c>
+      <c r="F384" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G384" t="n">
+        <v>0</v>
+      </c>
+      <c r="H384" t="b">
+        <v>0</v>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194293129</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>1151302581</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>【正規品】頭皮強化クリニック 脱毛症状緩和 弱酸性低刺激 シャンプー 400ml</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>ラボエイチ</t>
+        </is>
+      </c>
+      <c r="F385" t="n">
+        <v>3390</v>
+      </c>
+      <c r="G385" t="n">
+        <v>0</v>
+      </c>
+      <c r="H385" t="b">
+        <v>0</v>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151302581</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>1147973479</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>【正規品】ダイブイン 低分子 ヒアルロン酸 セラム 50ml</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F386" t="n">
+        <v>3090</v>
+      </c>
+      <c r="G386" t="n">
+        <v>0</v>
+      </c>
+      <c r="H386" t="b">
+        <v>0</v>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1147973479</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>1145690161</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>【正規品】アストラ エイシカ365 クーリングパックパッド pH4.5 110ml 60枚</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F387" t="n">
+        <v>3450</v>
+      </c>
+      <c r="G387" t="n">
+        <v>0</v>
+      </c>
+      <c r="H387" t="b">
+        <v>0</v>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145690161</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>1149096041</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>【正規品】ソフトリセット グリーン クレンジング バーム 100ml</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>ヒュッゲ</t>
+        </is>
+      </c>
+      <c r="F388" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G388" t="n">
+        <v>2</v>
+      </c>
+      <c r="H388" t="b">
+        <v>0</v>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149096041</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>1209979406</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>【正規品】ハンーユル 幼いヨモギ 皮脂吸着 ヨモギ餅パックフォーム 120ml, 1個</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>ハンユル</t>
+        </is>
+      </c>
+      <c r="F389" t="n">
+        <v>3450</v>
+      </c>
+      <c r="G389" t="n">
+        <v>1</v>
+      </c>
+      <c r="H389" t="b">
+        <v>0</v>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209979406</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>1162429093</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>yoo_k1120</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>コダリビノパーフェクトラジアンズセラム30mlホワイト ニングホワイト ニングアンプル（フランスセラム）</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>コーダリー</t>
+        </is>
+      </c>
+      <c r="F390" t="n">
+        <v>7340</v>
+      </c>
+      <c r="G390" t="n">
+        <v>1</v>
+      </c>
+      <c r="H390" t="b">
+        <v>0</v>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162429093</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J376"/>
+  <autoFilter ref="A1:J390"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 30, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$390</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$397</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J390"/>
+  <dimension ref="A1:J397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16445,8 +16445,295 @@
         </is>
       </c>
     </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>1210078172</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>PartyTime</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>MAKE UP FOR EVER(メイクアップフォーエバー) ミスト&amp;amp;フィックス マット トラベルサイズ 30mL</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>メイクアップフォーエバー</t>
+        </is>
+      </c>
+      <c r="F391" t="n">
+        <v>2810</v>
+      </c>
+      <c r="G391" t="n">
+        <v>0</v>
+      </c>
+      <c r="H391" t="b">
+        <v>0</v>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210078172</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>1194303809</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>all-cosmetics</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>【選べる】大容量 詰め替え シャンプートリートメントセット スムース モイスト 1200ml</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>BOTANIST</t>
+        </is>
+      </c>
+      <c r="F392" t="n">
+        <v>6311</v>
+      </c>
+      <c r="G392" t="n">
+        <v>0</v>
+      </c>
+      <c r="H392" t="b">
+        <v>0</v>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194303809</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>1194303108</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>all-cosmetics</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>【選べる】KURO クリームシャンプー 白髪染めシャンプー</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>バランローズ</t>
+        </is>
+      </c>
+      <c r="F393" t="n">
+        <v>6221</v>
+      </c>
+      <c r="G393" t="n">
+        <v>0</v>
+      </c>
+      <c r="H393" t="b">
+        <v>0</v>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194303108</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>1193233635</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>all-cosmetics</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>【大容量 詰め替え セット　カームナイトリペア リラックスナイトリペア　ディープナイトリペア　シャンプー　トリートメント 詰め替え 大容量　1100ml】</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>YOLU</t>
+        </is>
+      </c>
+      <c r="F394" t="n">
+        <v>6499</v>
+      </c>
+      <c r="G394" t="n">
+        <v>3</v>
+      </c>
+      <c r="H394" t="b">
+        <v>0</v>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193233635</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>1138374893</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>besba</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>香栄化学 エルカラ20 400ml レフィル 詰替用</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>香栄化学</t>
+        </is>
+      </c>
+      <c r="F395" t="n">
+        <v>3657</v>
+      </c>
+      <c r="G395" t="n">
+        <v>0</v>
+      </c>
+      <c r="H395" t="b">
+        <v>0</v>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138374893</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>1117338699</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>besba</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>ブルガリ アクア プールオム EDT オードトワレ SP 30ml 香水 BVLGARI</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>ブルガリ</t>
+        </is>
+      </c>
+      <c r="F396" t="n">
+        <v>9631</v>
+      </c>
+      <c r="G396" t="n">
+        <v>1</v>
+      </c>
+      <c r="H396" t="b">
+        <v>0</v>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1117338699</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>1117341863</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>besba</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>メゾン マルジェラ レプリカ バブル バス EDT オードトワレ SP 10ml ミニ香水 MAISON MARGIELA</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>メゾンマルジェラ</t>
+        </is>
+      </c>
+      <c r="F397" t="n">
+        <v>3821</v>
+      </c>
+      <c r="G397" t="n">
+        <v>0</v>
+      </c>
+      <c r="H397" t="b">
+        <v>0</v>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1117341863</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J390"/>
+  <autoFilter ref="A1:J397"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 33, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$397</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$404</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J397"/>
+  <dimension ref="A1:J404"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16732,8 +16732,295 @@
         </is>
       </c>
     </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>1109964483</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Beauty-Life</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>ハイドラローションマックス 400ml</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>エステダム</t>
+        </is>
+      </c>
+      <c r="F398" t="n">
+        <v>8125</v>
+      </c>
+      <c r="G398" t="n">
+        <v>0</v>
+      </c>
+      <c r="H398" t="b">
+        <v>0</v>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1109964483</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>1109951025</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Beauty-Life</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>シアーシュガー スクラブ 510g 11種 ビタミンC</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>Tree Hut</t>
+        </is>
+      </c>
+      <c r="F399" t="n">
+        <v>4225</v>
+      </c>
+      <c r="G399" t="n">
+        <v>0</v>
+      </c>
+      <c r="H399" t="b">
+        <v>0</v>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1109951025</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>1175324790</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>transia</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>センシティブ スージング ジェルクリーム 100g ひんやりうるおい 低刺激 水分クリーム ベタつきにくい 敏感肌 朝夜兼用 オイルフリー ノンコメド印象 軽い使用感</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>Mary&amp;amp;May</t>
+        </is>
+      </c>
+      <c r="F400" t="n">
+        <v>2760</v>
+      </c>
+      <c r="G400" t="n">
+        <v>0</v>
+      </c>
+      <c r="H400" t="b">
+        <v>0</v>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175324790</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>1201200397</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>transia</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>アクネブレミッシュ鎮静ボディウォッシュ 460ml 背中ニキビ・肌トラブルを改善する 背中ニキビ・ボディのざらつきケア さっぱり洗浄 つっぱりにくい デイリー用</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>Nodor</t>
+        </is>
+      </c>
+      <c r="F401" t="n">
+        <v>3970</v>
+      </c>
+      <c r="G401" t="n">
+        <v>3</v>
+      </c>
+      <c r="H401" t="b">
+        <v>0</v>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201200397</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>1148702438</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>KBEAUTYCREW</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>RXザビタミンC23セラム, 20ml</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F402" t="n">
+        <v>2520</v>
+      </c>
+      <c r="G402" t="n">
+        <v>1</v>
+      </c>
+      <c r="H402" t="b">
+        <v>0</v>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1148702438</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>1163367685</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>leeleeshop</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>[NEW]レッド アクネ ボディピーリングショット 110g</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F403" t="n">
+        <v>2210</v>
+      </c>
+      <c r="G403" t="n">
+        <v>1</v>
+      </c>
+      <c r="H403" t="b">
+        <v>0</v>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163367685</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>1206889838</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>leeleeshop</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>スーディング プリップ リップマスク</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>Laka</t>
+        </is>
+      </c>
+      <c r="F404" t="n">
+        <v>2448</v>
+      </c>
+      <c r="G404" t="n">
+        <v>1</v>
+      </c>
+      <c r="H404" t="b">
+        <v>0</v>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206889838</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J397"/>
+  <autoFilter ref="A1:J404"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 36, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$404</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$416</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J404"/>
+  <dimension ref="A1:J416"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17019,8 +17019,500 @@
         </is>
       </c>
     </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>1189376677</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>velaskin</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>[NEW]シェイキング シナジー ミスト 50ml / 保湿ミスト / ツヤミスト / メイクキープ / うるおいケア / ミスト化粧水</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F405" t="n">
+        <v>3637</v>
+      </c>
+      <c r="G405" t="n">
+        <v>0</v>
+      </c>
+      <c r="H405" t="b">
+        <v>0</v>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189376677</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>1209641531</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>angelskinmall</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>[1+]NEWサイトカインブースタープロ 70ml＋70ml</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Refilled</t>
+        </is>
+      </c>
+      <c r="F406" t="n">
+        <v>5039</v>
+      </c>
+      <c r="G406" t="n">
+        <v>0</v>
+      </c>
+      <c r="H406" t="b">
+        <v>0</v>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209641531</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>1209148971</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>angelskinmall</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>【韓国正規品/NEW】Gureum o de perfume EDP 50ml</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>BiBiANG</t>
+        </is>
+      </c>
+      <c r="F407" t="n">
+        <v>11419</v>
+      </c>
+      <c r="G407" t="n">
+        <v>0</v>
+      </c>
+      <c r="H407" t="b">
+        <v>0</v>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209148971</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>1206526891</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>angelskinmall</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>[NEW]エアロクーリングシャンプー 400ml＋70ml / -5.2度急速冷却</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F408" t="n">
+        <v>3859</v>
+      </c>
+      <c r="G408" t="n">
+        <v>0</v>
+      </c>
+      <c r="H408" t="b">
+        <v>0</v>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206526891</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>1203766483</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>tbas</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>ウォータープルーフ サーフィン サンスティック 20g</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F409" t="n">
+        <v>3201</v>
+      </c>
+      <c r="G409" t="n">
+        <v>0</v>
+      </c>
+      <c r="H409" t="b">
+        <v>0</v>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203766483</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>1096782550</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>tbas</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>アクア ヒアルロニック エッセンス 大容量, 250ml</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>ロベクチン</t>
+        </is>
+      </c>
+      <c r="F410" t="n">
+        <v>3888</v>
+      </c>
+      <c r="G410" t="n">
+        <v>0</v>
+      </c>
+      <c r="H410" t="b">
+        <v>0</v>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1096782550</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>1205563457</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>markets7</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>ガラクトミー エンザイム ピーリングジェル, 75ml, 1個</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F411" t="n">
+        <v>1829</v>
+      </c>
+      <c r="G411" t="n">
+        <v>0</v>
+      </c>
+      <c r="H411" t="b">
+        <v>0</v>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205563457</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>1171042034</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>markets7</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>アクティブクリーンアップクレンジングパウダー酵素洗顔剤, 80g</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F412" t="n">
+        <v>4005</v>
+      </c>
+      <c r="G412" t="n">
+        <v>1</v>
+      </c>
+      <c r="H412" t="b">
+        <v>0</v>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171042034</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>1212713877</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Lulupi</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>【フィー】 シェイキングシナジーミスト 50ml 全3種</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F413" t="n">
+        <v>2654</v>
+      </c>
+      <c r="G413" t="n">
+        <v>0</v>
+      </c>
+      <c r="H413" t="b">
+        <v>0</v>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212713877</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>1211134600</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>seimyongkorea</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>【NEW】 シェイキングミスト</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F414" t="n">
+        <v>2222</v>
+      </c>
+      <c r="G414" t="n">
+        <v>2</v>
+      </c>
+      <c r="H414" t="b">
+        <v>0</v>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211134600</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>1206908379</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>onme</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>(+マスクパック贈呈)MGFリターンクリーム 70ml 再生クリーム</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>cellmedics</t>
+        </is>
+      </c>
+      <c r="F415" t="n">
+        <v>8600</v>
+      </c>
+      <c r="G415" t="n">
+        <v>0</v>
+      </c>
+      <c r="H415" t="b">
+        <v>0</v>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206908379</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>1136826440</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>onme</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>特許技術BBTMとともに安全に使用できる プレミアムビーガン女性用 プレミアム ビーガン 育毛シャンプー 韓国シャンプー 400ml</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>AGAIN ME</t>
+        </is>
+      </c>
+      <c r="F416" t="n">
+        <v>5050</v>
+      </c>
+      <c r="G416" t="n">
+        <v>1</v>
+      </c>
+      <c r="H416" t="b">
+        <v>0</v>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1136826440</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J404"/>
+  <autoFilter ref="A1:J416"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 39, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$416</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$425</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J416"/>
+  <dimension ref="A1:J425"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17511,8 +17511,377 @@
         </is>
       </c>
     </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>1213399617</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>SKINFOODHQ</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>【トナーパッド】キャロットカロテンカーミングウォーターパッド( 60枚入り, 2個)</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F417" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G417" t="n">
+        <v>0</v>
+      </c>
+      <c r="H417" t="b">
+        <v>0</v>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213399617</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>1207120904</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>ALife07</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>ダーマトロジー クリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F418" t="n">
+        <v>8823</v>
+      </c>
+      <c r="G418" t="n">
+        <v>0</v>
+      </c>
+      <c r="H418" t="b">
+        <v>0</v>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207120904</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>1196025757</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>ALife07</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>ポア ダークスポット ブライトニングクリーム 35ml</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F419" t="n">
+        <v>1938</v>
+      </c>
+      <c r="G419" t="n">
+        <v>0</v>
+      </c>
+      <c r="H419" t="b">
+        <v>0</v>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196025757</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>1196382835</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>HAPPYLADY</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>[100時間保湿/かゆみ緩和/会社員A] [正規品]シカサルブクリーム 230ml</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>MECHAI</t>
+        </is>
+      </c>
+      <c r="F420" t="n">
+        <v>5352</v>
+      </c>
+      <c r="G420" t="n">
+        <v>0</v>
+      </c>
+      <c r="H420" t="b">
+        <v>0</v>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196382835</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>1183055576</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Asteroid</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>シャンプー ダマスクローズの香り 1L</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>ミルクバオバブ</t>
+        </is>
+      </c>
+      <c r="F421" t="n">
+        <v>2745</v>
+      </c>
+      <c r="G421" t="n">
+        <v>0</v>
+      </c>
+      <c r="H421" t="b">
+        <v>0</v>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183055576</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>1133994465</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Asteroid</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>24K ラグジュアリー ゴールド アンプル 110ml</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>BERGAMO</t>
+        </is>
+      </c>
+      <c r="F422" t="n">
+        <v>3813</v>
+      </c>
+      <c r="G422" t="n">
+        <v>0</v>
+      </c>
+      <c r="H422" t="b">
+        <v>0</v>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1133994465</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>1206870778</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>mood_k</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>345 リリーフ クリームミスト 100ml+60ml 保湿ミスト 韓国コスメ 敏感肌 乾燥対策 フェイスミスト スキンケア</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>ドクターエルシア</t>
+        </is>
+      </c>
+      <c r="F423" t="n">
+        <v>4240</v>
+      </c>
+      <c r="G423" t="n">
+        <v>0</v>
+      </c>
+      <c r="H423" t="b">
+        <v>0</v>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206870778</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>1209089569</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>mokos_kshop</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>the SAEM アーバンエコ ハラケケ トナー 150ml1個 韓国化粧水 高保湿 乾燥肌 敏感肌 スキンケア 水分補給 保湿トナー</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>ザセム</t>
+        </is>
+      </c>
+      <c r="F424" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G424" t="n">
+        <v>0</v>
+      </c>
+      <c r="H424" t="b">
+        <v>0</v>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209089569</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>1209089497</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>mokos_kshop</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>the SAEM アーバンエコ ハラケケ トナー 150ml 2個 set/韓国化粧水 高保湿 乾燥肌 敏感肌 スキンケア 水分補給 保湿トナー</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>ザセム</t>
+        </is>
+      </c>
+      <c r="F425" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G425" t="n">
+        <v>0</v>
+      </c>
+      <c r="H425" t="b">
+        <v>0</v>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209089497</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J416"/>
+  <autoFilter ref="A1:J425"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 42, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$425</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$446</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J425"/>
+  <dimension ref="A1:J446"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17880,8 +17880,869 @@
         </is>
       </c>
     </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>1177385233</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>doitsistersseoul</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>フィックスディテールヘアマスカラ 15ml</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>チャホン</t>
+        </is>
+      </c>
+      <c r="F426" t="n">
+        <v>3230</v>
+      </c>
+      <c r="G426" t="n">
+        <v>0</v>
+      </c>
+      <c r="H426" t="b">
+        <v>0</v>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177385233</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>1170230232</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>doitsistersseoul</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>ドクダミシルキーモイスチャー日焼け止め 50ml</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F427" t="n">
+        <v>2250</v>
+      </c>
+      <c r="G427" t="n">
+        <v>0</v>
+      </c>
+      <c r="H427" t="b">
+        <v>0</v>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170230232</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>1177545076</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>doitsistersseoul</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>[!!超人気!!]ダーマヒーラーポアタイトニングトナーパッド 60枚</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F428" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G428" t="n">
+        <v>1</v>
+      </c>
+      <c r="H428" t="b">
+        <v>0</v>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177545076</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>1205368128</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>doitsistersseoul</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>ドクダミポアディープクレンジングフォーム 150ml</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F429" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G429" t="n">
+        <v>0</v>
+      </c>
+      <c r="H429" t="b">
+        <v>0</v>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205368128</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>1195011504</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>doitsistersseoul</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>ドクダミ トラベル クレンジングセット (オイル20ml + フォーム25ml)</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F430" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G430" t="n">
+        <v>0</v>
+      </c>
+      <c r="H430" t="b">
+        <v>0</v>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195011504</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>1209905260</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>hiseller</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>オドール オールインワン クリアボディウォッシュ 2個, 460ml</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Nodor</t>
+        </is>
+      </c>
+      <c r="F431" t="n">
+        <v>6898</v>
+      </c>
+      <c r="G431" t="n">
+        <v>0</v>
+      </c>
+      <c r="H431" t="b">
+        <v>0</v>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209905260</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>1209905066</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>hiseller</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>ポケモンエディションクリアボディミスト 200ml 企画 (ミニチュア 30ml + イーブイ防水パック)</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>NOT4U</t>
+        </is>
+      </c>
+      <c r="F432" t="n">
+        <v>3448</v>
+      </c>
+      <c r="G432" t="n">
+        <v>0</v>
+      </c>
+      <c r="H432" t="b">
+        <v>0</v>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209905066</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>1209905054</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>hiseller</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>ホワイトアプリコット ソリッドパフューム 塗る固体香水 フレグランス 携帯用 30ml</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>LUAFEE</t>
+        </is>
+      </c>
+      <c r="F433" t="n">
+        <v>2249</v>
+      </c>
+      <c r="G433" t="n">
+        <v>0</v>
+      </c>
+      <c r="H433" t="b">
+        <v>0</v>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209905054</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>1196415617</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Widgo2</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>【WiD2】 AHA・BHA配合 28デイズヒアルクリーム (30ml) ザラつきOFF！なめらか透明肌へ 1個</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F434" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G434" t="n">
+        <v>1</v>
+      </c>
+      <c r="H434" t="b">
+        <v>0</v>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196415617</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>1196366572</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Widgo2</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>【WiD2】 ガラクトナイアシンエッセンスマスク 10枚入り 肌をクリアに・高保湿・エイジングケア</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F435" t="n">
+        <v>2851</v>
+      </c>
+      <c r="G435" t="n">
+        <v>0</v>
+      </c>
+      <c r="H435" t="b">
+        <v>0</v>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196366572</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>1189270361</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>【Wid】 フォリゲン トニック 120ml 2個セット・頭皮ケア・ヘアトニック・抜け毛予防・頭皮栄養・スカルプケア</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F436" t="n">
+        <v>5287</v>
+      </c>
+      <c r="G436" t="n">
+        <v>0</v>
+      </c>
+      <c r="H436" t="b">
+        <v>0</v>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189270361</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>1188452071</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>【Wid】 アスコルビルテトラィソパルミテート ソリューション 20% イン ビタミンF / 30ml / 1個 / ビタミンC美容液 / オイル美容液 / 透明感 / ハリケア</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F437" t="n">
+        <v>5841</v>
+      </c>
+      <c r="G437" t="n">
+        <v>0</v>
+      </c>
+      <c r="H437" t="b">
+        <v>0</v>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188452071</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>1188452072</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>【Wid】 グリコール酸 7% エクスフォリエイティング トナー / 240ml / 2個セット / ふき取り化粧水 / 角質ケア / 肌キメ整え / ツヤ肌</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F438" t="n">
+        <v>6385</v>
+      </c>
+      <c r="G438" t="n">
+        <v>0</v>
+      </c>
+      <c r="H438" t="b">
+        <v>0</v>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188452072</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>1179809144</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>[角質ケア] マンデル酸 10％ + HA 30ml 毛穴ケア つるつる美肌 セラム</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F439" t="n">
+        <v>2485</v>
+      </c>
+      <c r="G439" t="n">
+        <v>0</v>
+      </c>
+      <c r="H439" t="b">
+        <v>0</v>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179809144</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>1211721947</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>SOULPRISM</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>ポアタイトニング クレンジングバーム 50ml × 2個セット</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F440" t="n">
+        <v>7482</v>
+      </c>
+      <c r="G440" t="n">
+        <v>0</v>
+      </c>
+      <c r="H440" t="b">
+        <v>0</v>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211721947</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>1137919225</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>SOULPRISM</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>パンテノール クリームウォッシュ 300ml × 2本</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F441" t="n">
+        <v>6253</v>
+      </c>
+      <c r="G441" t="n">
+        <v>0</v>
+      </c>
+      <c r="H441" t="b">
+        <v>0</v>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1137919225</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>1211388494</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>SOULPRISM</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>ウォーターカプセル サンセラム SPF50+ / PA+++ 40ml × 2個セット</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F442" t="n">
+        <v>7482</v>
+      </c>
+      <c r="G442" t="n">
+        <v>0</v>
+      </c>
+      <c r="H442" t="b">
+        <v>0</v>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211388494</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>1190175660</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>flymong-korea</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>マダガスカルセントラアンプル 55ml, 1個</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F443" t="n">
+        <v>2795</v>
+      </c>
+      <c r="G443" t="n">
+        <v>1</v>
+      </c>
+      <c r="H443" t="b">
+        <v>0</v>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190175660</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>1190175438</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>flymong-korea</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>ノーセバム サンクッション EX SPF50+ PA++++, 1個</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F444" t="n">
+        <v>2215</v>
+      </c>
+      <c r="G444" t="n">
+        <v>0</v>
+      </c>
+      <c r="H444" t="b">
+        <v>0</v>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190175438</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>1195083431</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>ITRADE</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>ダイブインセラム 20ml x 5個 (計100ml)</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F445" t="n">
+        <v>1780</v>
+      </c>
+      <c r="G445" t="n">
+        <v>3</v>
+      </c>
+      <c r="H445" t="b">
+        <v>0</v>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195083431</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>1212617523</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>ITRADE</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>アトバリア365クリーム30mL×3個 + ダーマUV365バリアハイドロミネラル日焼け止め20ml x3個</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F446" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G446" t="n">
+        <v>0</v>
+      </c>
+      <c r="H446" t="b">
+        <v>0</v>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212617523</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J425"/>
+  <autoFilter ref="A1:J446"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 45, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$446</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$458</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J446"/>
+  <dimension ref="A1:J458"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18741,8 +18741,500 @@
         </is>
       </c>
     </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>1057808818</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>djshopping</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>LAB+トリプルウォーターピールスージングパッド 60枚</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>SNP</t>
+        </is>
+      </c>
+      <c r="F447" t="n">
+        <v>2390</v>
+      </c>
+      <c r="G447" t="n">
+        <v>0</v>
+      </c>
+      <c r="H447" t="b">
+        <v>0</v>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1057808818</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>1183855839</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>ardistore</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>ジェイエムソリューション B5 ヒアモイスチャライジングクリーム 60ml 3本 JM 솔루션 B5 히어 모이스처라이징 크림 60ml 3병</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>JM solution</t>
+        </is>
+      </c>
+      <c r="F448" t="n">
+        <v>4700</v>
+      </c>
+      <c r="G448" t="n">
+        <v>0</v>
+      </c>
+      <c r="H448" t="b">
+        <v>0</v>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183855839</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>1208177592</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>ardistore</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>イェジフ ヨンビン 紅参化粧品 5種 1セット 예지후 영빈 홍삼 화장품 5종 1세트</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>禮知后</t>
+        </is>
+      </c>
+      <c r="F449" t="n">
+        <v>5950</v>
+      </c>
+      <c r="G449" t="n">
+        <v>0</v>
+      </c>
+      <c r="H449" t="b">
+        <v>0</v>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208177592</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>1169201226</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>JSKSHOPPING</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>[1+1]ジェントルブラック フレッシュ クレンジングオイル 150ml+150ml</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>dear,Klairs</t>
+        </is>
+      </c>
+      <c r="F450" t="n">
+        <v>4584</v>
+      </c>
+      <c r="G450" t="n">
+        <v>0</v>
+      </c>
+      <c r="H450" t="b">
+        <v>0</v>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169201226</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>1110101930</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>JSKSHOPPING</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>フォリゲンシャンプー 500ml</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F451" t="n">
+        <v>2847</v>
+      </c>
+      <c r="G451" t="n">
+        <v>0</v>
+      </c>
+      <c r="H451" t="b">
+        <v>0</v>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1110101930</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>1092755563</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>JSKSHOPPING</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>ベイキング パウダー サクサク 毛穴 スクラブ 200gx2個</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>エチュード</t>
+        </is>
+      </c>
+      <c r="F452" t="n">
+        <v>3148</v>
+      </c>
+      <c r="G452" t="n">
+        <v>5</v>
+      </c>
+      <c r="H452" t="b">
+        <v>0</v>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1092755563</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>1202396707</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>SUM</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>レッドブレミッシュ フォーメン オイルカットローションオールインワン, 150ml, 1本</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F453" t="n">
+        <v>2373</v>
+      </c>
+      <c r="G453" t="n">
+        <v>0</v>
+      </c>
+      <c r="H453" t="b">
+        <v>0</v>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202396707</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>1080682873</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>momonara</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>ザ ヒアルロニック アシード 3 セラム 20ml</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F454" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G454" t="n">
+        <v>0</v>
+      </c>
+      <c r="H454" t="b">
+        <v>0</v>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1080682873</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>1079892554</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>momonara</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>ピュアフィット シカ カーミング トゥルーシートマスク 10枚</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F455" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G455" t="n">
+        <v>0</v>
+      </c>
+      <c r="H455" t="b">
+        <v>0</v>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1079892554</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>1204813717</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Kbeauty_store</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>大容量トナー ツボクサ グリーンダーマ マイルド シカ ビッグトナー 500ml</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F456" t="n">
+        <v>3230</v>
+      </c>
+      <c r="G456" t="n">
+        <v>2</v>
+      </c>
+      <c r="H456" t="b">
+        <v>0</v>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204813717</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>1204188494</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Kbeauty_store</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>ドクダミ シカ クーリング 水分 クリーム 100ml</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>トニーモリー</t>
+        </is>
+      </c>
+      <c r="F457" t="n">
+        <v>2760</v>
+      </c>
+      <c r="G457" t="n">
+        <v>0</v>
+      </c>
+      <c r="H457" t="b">
+        <v>0</v>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204188494</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>1201899429</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Kbeauty_store</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>ドクダミ 70 スージング コラーゲン マスク 4枚</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F458" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G458" t="n">
+        <v>0</v>
+      </c>
+      <c r="H458" t="b">
+        <v>0</v>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201899429</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J446"/>
+  <autoFilter ref="A1:J458"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 48, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$458</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$468</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J458"/>
+  <dimension ref="A1:J468"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19233,8 +19233,418 @@
         </is>
       </c>
     </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>1188680603</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>relationmarketing</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>ルベル IAU イオ クレンジング リラックスメント シャンプー 1000ml＆イオ クリーム シルキーリペア トリートメント1000ml 詰め替え セット</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>イオ</t>
+        </is>
+      </c>
+      <c r="F459" t="n">
+        <v>7709</v>
+      </c>
+      <c r="G459" t="n">
+        <v>1</v>
+      </c>
+      <c r="H459" t="b">
+        <v>0</v>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188680603</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>1209051021</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>zeesea</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>全日オイルコントロールメイクキープミスト 化粧崩れ防止 [ミルキーウェイ],[スプレー],[セッティング]</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>ZEESEA</t>
+        </is>
+      </c>
+      <c r="F460" t="n">
+        <v>2680</v>
+      </c>
+      <c r="G460" t="n">
+        <v>2</v>
+      </c>
+      <c r="H460" t="b">
+        <v>0</v>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209051021</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>1210528997</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>【1+1セット】クリーンティーツリーリポソーム カーミングマスク 5枚入×2個 ヒアルロン酸 パンテノール 水分 鎮静 保湿 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F461" t="n">
+        <v>3069</v>
+      </c>
+      <c r="G461" t="n">
+        <v>0</v>
+      </c>
+      <c r="H461" t="b">
+        <v>0</v>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210528997</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>1210272622</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>【1+1セット】ウォータフルエッセンスサンクリーム SPF50+ PA++++ 50ml×2個 保湿 UVケア エッセンス 日焼け止め 化粧下地 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F462" t="n">
+        <v>6442</v>
+      </c>
+      <c r="G462" t="n">
+        <v>0</v>
+      </c>
+      <c r="H462" t="b">
+        <v>0</v>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210272622</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>1206508858</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>【1+1セット】ソフトリセット グリーンクレンジングバーム 100ml 2個 メイク落とし 保湿洗顔 角質ケア 毛穴汚れケア 韓国コスメ しっとりディープクレンジング</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>ヒュッゲ</t>
+        </is>
+      </c>
+      <c r="F463" t="n">
+        <v>6279</v>
+      </c>
+      <c r="G463" t="n">
+        <v>0</v>
+      </c>
+      <c r="H463" t="b">
+        <v>0</v>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206508858</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>1206240655</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>ウォーターtoアンプルトリートメント 200ml 1個 毛髪保湿 ツヤ髪ケア しっとりヘアケア ホームケア 韓国コスメ 上品な香り デイリーケア</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>サミュ</t>
+        </is>
+      </c>
+      <c r="F464" t="n">
+        <v>6459</v>
+      </c>
+      <c r="G464" t="n">
+        <v>0</v>
+      </c>
+      <c r="H464" t="b">
+        <v>0</v>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206240655</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>781856183</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>bellcosme</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>モイスチャライジング トナー UFT （ウルトラフェイシャルトナー） 250ml</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>キールズ</t>
+        </is>
+      </c>
+      <c r="F465" t="n">
+        <v>3631</v>
+      </c>
+      <c r="G465" t="n">
+        <v>3</v>
+      </c>
+      <c r="H465" t="b">
+        <v>0</v>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=781856183</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>1204378750</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>bellcosme</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>フェイシャル トリートメント エッセンス 330ml 1個</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>SK-Ⅱ</t>
+        </is>
+      </c>
+      <c r="F466" t="n">
+        <v>33266</v>
+      </c>
+      <c r="G466" t="n">
+        <v>0</v>
+      </c>
+      <c r="H466" t="b">
+        <v>0</v>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204378750</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>1173903686</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>bettysbeauty</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>レプリカ ハンドクリーム レイジーサンデー モーニング 50ml/1.6fl.oz.</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>メゾンマルジェラ</t>
+        </is>
+      </c>
+      <c r="F467" t="n">
+        <v>4191</v>
+      </c>
+      <c r="G467" t="n">
+        <v>1</v>
+      </c>
+      <c r="H467" t="b">
+        <v>0</v>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1173903686</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>638382548</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>bettysbeauty</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>ヴァーベナ ボディローション 250ml</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>ロクシタン</t>
+        </is>
+      </c>
+      <c r="F468" t="n">
+        <v>3135</v>
+      </c>
+      <c r="G468" t="n">
+        <v>2</v>
+      </c>
+      <c r="H468" t="b">
+        <v>0</v>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=638382548</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J458"/>
+  <autoFilter ref="A1:J468"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 51, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$468</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$477</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J468"/>
+  <dimension ref="A1:J477"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19643,8 +19643,377 @@
         </is>
       </c>
     </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>1059030924</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>strawberrynet-beauty</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Davines モアインサイド ディス イズ ア カールビルディング セラム (カールヘア用)</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>ダビネス</t>
+        </is>
+      </c>
+      <c r="F469" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G469" t="n">
+        <v>1</v>
+      </c>
+      <c r="H469" t="b">
+        <v>0</v>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1059030924</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>1135055592</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>strawberrynet-beauty</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Valentino バレンチノ ウォモ ボーン イン ローマ オー ド トワレ スプレー*</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>ヴァレンティノ</t>
+        </is>
+      </c>
+      <c r="F470" t="n">
+        <v>20200</v>
+      </c>
+      <c r="G470" t="n">
+        <v>0</v>
+      </c>
+      <c r="H470" t="b">
+        <v>0</v>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135055592</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>1181475483</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>strawberrynet-beauty</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Giorgio Armani ルミナス シルク ファンデーション - # 4 (Light Sand) 202611</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>ジョルジオアルマーニ</t>
+        </is>
+      </c>
+      <c r="F471" t="n">
+        <v>10300</v>
+      </c>
+      <c r="G471" t="n">
+        <v>0</v>
+      </c>
+      <c r="H471" t="b">
+        <v>0</v>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181475483</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>1206682479</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>cafebespoke</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>グリーンプロポリス 頭皮クレンジング シャンプー+トリートメント [1000ml+1000ml] セット</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F472" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G472" t="n">
+        <v>3</v>
+      </c>
+      <c r="H472" t="b">
+        <v>0</v>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206682479</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>1112935346</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>puerueme</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>【選べる2個セット】デビルズ パフュームファンタジーシャンプー &amp;amp; コンディショナー, 1L+1L</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F473" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G473" t="n">
+        <v>1</v>
+      </c>
+      <c r="H473" t="b">
+        <v>0</v>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1112935346</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>1084157476</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>puerueme</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>【NEW COLOR】イージーブロウトーンチェンジャー (5回分) /ブリーチ / 眉毛脱色 /眉カラーケア</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>サムバイミー</t>
+        </is>
+      </c>
+      <c r="F474" t="n">
+        <v>4110</v>
+      </c>
+      <c r="G474" t="n">
+        <v>0</v>
+      </c>
+      <c r="H474" t="b">
+        <v>0</v>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1084157476</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>1192529297</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>cald</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>ポア リフティング アンプル プラス 75ml</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>グリーントマト</t>
+        </is>
+      </c>
+      <c r="F475" t="n">
+        <v>3825</v>
+      </c>
+      <c r="G475" t="n">
+        <v>2</v>
+      </c>
+      <c r="H475" t="b">
+        <v>0</v>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192529297</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>1188176132</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>cald</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>デイリーケアマスクパック5枚企画4種（+1枚追加贈呈）</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F476" t="n">
+        <v>2250</v>
+      </c>
+      <c r="G476" t="n">
+        <v>0</v>
+      </c>
+      <c r="H476" t="b">
+        <v>0</v>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188176132</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>1208012735</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>cald</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>【トーンアップ・UVケア】ディオプラス ブルーフェザー トーンアップ サンスクリーン 40ml</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>ディオプラス</t>
+        </is>
+      </c>
+      <c r="F477" t="n">
+        <v>3610</v>
+      </c>
+      <c r="G477" t="n">
+        <v>0</v>
+      </c>
+      <c r="H477" t="b">
+        <v>0</v>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208012735</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J468"/>
+  <autoFilter ref="A1:J477"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 54, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$477</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$487</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J477"/>
+  <dimension ref="A1:J487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20012,8 +20012,418 @@
         </is>
       </c>
     </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>1185790423</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>junglix</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>LPT ケラチン リペア ノーウォッシュ トリートメント 70ml / 洗い流さない ヘアパック / 高濃縮 タンパク質</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>ダリーフ</t>
+        </is>
+      </c>
+      <c r="F478" t="n">
+        <v>2716</v>
+      </c>
+      <c r="G478" t="n">
+        <v>0</v>
+      </c>
+      <c r="H478" t="b">
+        <v>0</v>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185790423</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>1184898677</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>junglix</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>スンジョンディレクタートーンアップコレックティング日焼け止め SPF50+ PA++++ 40ml</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>エチュード</t>
+        </is>
+      </c>
+      <c r="F479" t="n">
+        <v>2572</v>
+      </c>
+      <c r="G479" t="n">
+        <v>0</v>
+      </c>
+      <c r="H479" t="b">
+        <v>0</v>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1184898677</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>1203960088</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>HEYDAYS</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>345リリーフクリーム, 50ml</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>ドクターエルシア</t>
+        </is>
+      </c>
+      <c r="F480" t="n">
+        <v>2453</v>
+      </c>
+      <c r="G480" t="n">
+        <v>1</v>
+      </c>
+      <c r="H480" t="b">
+        <v>0</v>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203960088</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>1192047927</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>HEYDAYS</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>グリコリックアシッド7%トーニングソリューション 240ml トーニング ソリューション</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F481" t="n">
+        <v>2216</v>
+      </c>
+      <c r="G481" t="n">
+        <v>2</v>
+      </c>
+      <c r="H481" t="b">
+        <v>0</v>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192047927</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>1194573796</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>1989</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>レッドブレミッシュクリアスージングクリーム, 70ml, 2個</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F482" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G482" t="n">
+        <v>0</v>
+      </c>
+      <c r="H482" t="b">
+        <v>0</v>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194573796</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>1203144925</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>ohnewcompany</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>【企画】オールアバウト グロウ カバークリーム (35g) + 大王パフ 1枚付き SPF50+ PA++++ 韓国コスメ ベースメイク 24時間持続 崩れない</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>CHASIN’ RABBITS</t>
+        </is>
+      </c>
+      <c r="F483" t="n">
+        <v>1946</v>
+      </c>
+      <c r="G483" t="n">
+        <v>1</v>
+      </c>
+      <c r="H483" t="b">
+        <v>0</v>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203144925</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>1186319083</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>wb</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>韓国正規品 AMPLE:N ペプチドショットアンプル2X 100ml 大容量美容液 ペプチド 高保湿 ハリケア 弾力ケア 韓国コスメ 韓国直送</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>アンプルエヌ</t>
+        </is>
+      </c>
+      <c r="F484" t="n">
+        <v>2999</v>
+      </c>
+      <c r="G484" t="n">
+        <v>0</v>
+      </c>
+      <c r="H484" t="b">
+        <v>0</v>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1186319083</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>1174996099</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>wb</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>韓国正規品 3Dハリクリームセット 50ml 美容液15ml+ミスト20ml付 豪華2点特典 保湿 ハリケア 韓国コスメ 韓国直送</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F485" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G485" t="n">
+        <v>1</v>
+      </c>
+      <c r="H485" t="b">
+        <v>0</v>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174996099</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>1213260537</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>wb</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>韓国正規品 リニューアル MLE保湿ローション 120ml／200ml 敏感肌 乾燥肌 ベビー 全身 肌バリア 韓国直送</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F486" t="n">
+        <v>2465</v>
+      </c>
+      <c r="G486" t="n">
+        <v>0</v>
+      </c>
+      <c r="H486" t="b">
+        <v>0</v>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213260537</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>1171696930</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>C2Y</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>ワセリン マスクパック シリーズ 3種 23ml*30枚(1箱10枚入)/保湿ケア/水分/シカ/弾力 3種 選択</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>C2Y</t>
+        </is>
+      </c>
+      <c r="F487" t="n">
+        <v>3726</v>
+      </c>
+      <c r="G487" t="n">
+        <v>0</v>
+      </c>
+      <c r="H487" t="b">
+        <v>0</v>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171696930</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J477"/>
+  <autoFilter ref="A1:J487"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 57, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$487</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$497</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J487"/>
+  <dimension ref="A1:J497"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20422,8 +20422,418 @@
         </is>
       </c>
     </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>1193418611</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>KVIVE</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>ヒーラー ポア タイトニング トナーパッド 本品60枚+詰め替え用 60枚入り/PDRN トナーパッド 美容液 /韓国 人気 トナーパッド/弾力/保湿/水分アンプル/c-PDRN/エイジングケアトナー</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F488" t="n">
+        <v>6870</v>
+      </c>
+      <c r="G488" t="n">
+        <v>0</v>
+      </c>
+      <c r="H488" t="b">
+        <v>0</v>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193418611</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>1191891158</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>KVIVE</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>赤小豆 毛穴クレイマスク 140ml + 水分ウォータージェル 100ml セット/毛穴ケア/皮脂ケア/角質ケア/毛穴汚れ/韓国コスメ/韓国スキンケア/boj 赤小豆/米蜜グロウマスク</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F489" t="n">
+        <v>7130</v>
+      </c>
+      <c r="G489" t="n">
+        <v>0</v>
+      </c>
+      <c r="H489" t="b">
+        <v>0</v>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191891158</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>1212343699</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>pickary</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>【5枚入り】 垢すりグローブ ソフトボディ レッドグローブ クリーン角質ケア・ボディクレンジング 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>ランドリーユー</t>
+        </is>
+      </c>
+      <c r="F490" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G490" t="n">
+        <v>0</v>
+      </c>
+      <c r="H490" t="b">
+        <v>0</v>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212343699</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>1192678454</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>olivegreen</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>【韓国皮膚科医推奨No.1】 肌荒れ・乾燥くすみ対策に！エイシカ365 トラブルリリーフセラムpH4.5 40ml 肌荒れ くすみ 乾燥 美容液</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F491" t="n">
+        <v>2910</v>
+      </c>
+      <c r="G491" t="n">
+        <v>0</v>
+      </c>
+      <c r="H491" t="b">
+        <v>0</v>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192678454</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>1192676012</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>olivegreen</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>【韓国皮膚科医推奨No.1】アトバリア365 クリーム 80mL 保湿クリーム 水分クリーム 保湿カプセル セラミド クリーム 肌荒れ 水分</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F492" t="n">
+        <v>2470</v>
+      </c>
+      <c r="G492" t="n">
+        <v>1</v>
+      </c>
+      <c r="H492" t="b">
+        <v>0</v>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192676012</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>1192160801</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>olivegreen</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>レチノール シカ リペア セラム 30mL</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F493" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G493" t="n">
+        <v>0</v>
+      </c>
+      <c r="H493" t="b">
+        <v>0</v>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192160801</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>1192597637</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>strawberryshop</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Axenda ルティナー クリーム 毛穴バーム スリープバーム マルチバーム 15ml 2個</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>aXENDA</t>
+        </is>
+      </c>
+      <c r="F494" t="n">
+        <v>9850</v>
+      </c>
+      <c r="G494" t="n">
+        <v>0</v>
+      </c>
+      <c r="H494" t="b">
+        <v>0</v>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192597637</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>1189809546</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>strawberryshop</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>レッドフィルティンググルセラム 35ml + レッドピルホワイトセラム 35ML</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F495" t="n">
+        <v>6999</v>
+      </c>
+      <c r="G495" t="n">
+        <v>0</v>
+      </c>
+      <c r="H495" t="b">
+        <v>0</v>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189809546</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>1123787663</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>BOMAMALL</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>UVイデア XL プロテクショントーンアップ ローズ 30ml</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>ラロッシュポゼ</t>
+        </is>
+      </c>
+      <c r="F496" t="n">
+        <v>6961</v>
+      </c>
+      <c r="G496" t="n">
+        <v>0</v>
+      </c>
+      <c r="H496" t="b">
+        <v>0</v>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123787663</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>1146152293</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>BOMAMALL</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>パフュームヘアトリートメント/ヒノキ/ふんわりヒノキの香り/Hinoki/香水のトリートメント/髪の栄養と香りを一度に解決/毛髪栄養改善/毛髪切れ改善/柔らかさ改善</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>La'dor</t>
+        </is>
+      </c>
+      <c r="F497" t="n">
+        <v>5811</v>
+      </c>
+      <c r="G497" t="n">
+        <v>0</v>
+      </c>
+      <c r="H497" t="b">
+        <v>0</v>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146152293</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J487"/>
+  <autoFilter ref="A1:J497"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 60, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$497</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$520</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J497"/>
+  <dimension ref="A1:J520"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20832,8 +20832,951 @@
         </is>
       </c>
     </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>1083089713</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>fresh-aka</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>ピュアフィットシカ 弱酸性クレンジングパッド 100枚入 * 1個</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F498" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G498" t="n">
+        <v>0</v>
+      </c>
+      <c r="H498" t="b">
+        <v>0</v>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1083089713</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>1082221247</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>fresh-aka</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>ムード ペブル ネイル 29種</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>ロムアンド</t>
+        </is>
+      </c>
+      <c r="F499" t="n">
+        <v>1810</v>
+      </c>
+      <c r="G499" t="n">
+        <v>0</v>
+      </c>
+      <c r="H499" t="b">
+        <v>0</v>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1082221247</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>1205514714</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Nandak</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>[ダーママスク10枚プレゼント] マデカクリームハイドラカーミング50ml3個韓国人気化粧品</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F500" t="n">
+        <v>5850</v>
+      </c>
+      <c r="G500" t="n">
+        <v>1</v>
+      </c>
+      <c r="H500" t="b">
+        <v>0</v>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205514714</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>1093898160</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>PeonyAgit</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>発酵豆 バウンス タンパク質 エッセンス 80ml/低刺激/保湿/水分/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>フラスキン</t>
+        </is>
+      </c>
+      <c r="F501" t="n">
+        <v>4372</v>
+      </c>
+      <c r="G501" t="n">
+        <v>0</v>
+      </c>
+      <c r="H501" t="b">
+        <v>0</v>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093898160</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>1096256291</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>PeonyAgit</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>【正規品】コラーゲンプロフェッショナルプログラムセット (マイクロコラーゲン200mg*4ea+アクティベーションブースター30ml+ドロッパー4ea)/コラーゲン/光沢/高栄養/活力/弾力</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>LAVIEN</t>
+        </is>
+      </c>
+      <c r="F502" t="n">
+        <v>15010</v>
+      </c>
+      <c r="G502" t="n">
+        <v>0</v>
+      </c>
+      <c r="H502" t="b">
+        <v>0</v>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1096256291</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>1094315646</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>PeonyAgit</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>【1+1】ブイ コラーゲン ハートフィット マルチバーム 10g/肌バリアケア/ スローエイジング/ 高濃縮/ 弾力/ 水分バリア/ 鎮静/ 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F503" t="n">
+        <v>6786</v>
+      </c>
+      <c r="G503" t="n">
+        <v>1</v>
+      </c>
+      <c r="H503" t="b">
+        <v>0</v>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1094315646</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>1093734916</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>PeonyAgit</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>【1+1】スピキュールセラム(ニードルアクション100) 30ml/ 塗る毛穴セラム針 / ニードルショット / ブースティングセラム / 肌のキメ改善 / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>BIOME ACTIVATE</t>
+        </is>
+      </c>
+      <c r="F504" t="n">
+        <v>3995</v>
+      </c>
+      <c r="G504" t="n">
+        <v>0</v>
+      </c>
+      <c r="H504" t="b">
+        <v>0</v>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J504" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093734916</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>1125939784</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>mellia</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>【正規品】グローアップインシャワートーンアップミルク300g</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>MEDIPICKME</t>
+        </is>
+      </c>
+      <c r="F505" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G505" t="n">
+        <v>2</v>
+      </c>
+      <c r="H505" t="b">
+        <v>0</v>
+      </c>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J505" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1125939784</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>1111189488</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>mellia</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>[単品] JunJun共同開発_クレンジングバーム2種 100ml (毛穴/トーンアップ)</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>ビープレーン</t>
+        </is>
+      </c>
+      <c r="F506" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G506" t="n">
+        <v>0</v>
+      </c>
+      <c r="H506" t="b">
+        <v>0</v>
+      </c>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1111189488</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>1205453339</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>mellia</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>ネックパッチプレステージ（5枚入り）首　シワ　弾力 ネックケア　アイロン　ハリケア 首のシワ 保湿 たるみ デコルテケア</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>VELLA</t>
+        </is>
+      </c>
+      <c r="F507" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G507" t="n">
+        <v>0</v>
+      </c>
+      <c r="H507" t="b">
+        <v>0</v>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J507" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205453339</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>1097540476</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>EPONA</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>【公式】 プレミアム紅参ゴールドクリーム / 50ml / 1個</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>エポナ</t>
+        </is>
+      </c>
+      <c r="F508" t="n">
+        <v>5090</v>
+      </c>
+      <c r="G508" t="n">
+        <v>1</v>
+      </c>
+      <c r="H508" t="b">
+        <v>0</v>
+      </c>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J508" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097540476</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>1175249089</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>KIRAKORE</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>ザ セラミド スキンバリア モイスチャライザークリーム 80ml 2個</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F509" t="n">
+        <v>6230</v>
+      </c>
+      <c r="G509" t="n">
+        <v>0</v>
+      </c>
+      <c r="H509" t="b">
+        <v>0</v>
+      </c>
+      <c r="I509" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175249089</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>1152704413</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>KIRAKORE</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>オーガニック ホホバオイル ゴールド 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>FRANCOISE&amp;amp;Fragrance</t>
+        </is>
+      </c>
+      <c r="F510" t="n">
+        <v>2506</v>
+      </c>
+      <c r="G510" t="n">
+        <v>0</v>
+      </c>
+      <c r="H510" t="b">
+        <v>0</v>
+      </c>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J510" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152704413</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>1154992110</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>KIRAKORE</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>レッド ブレミッシュ スージング アップ サンクリーム SPF50+ PA++++ 50ml 2個</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F511" t="n">
+        <v>4149</v>
+      </c>
+      <c r="G511" t="n">
+        <v>0</v>
+      </c>
+      <c r="H511" t="b">
+        <v>0</v>
+      </c>
+      <c r="I511" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J511" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154992110</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>1154991907</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>KIRAKORE</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>マダガスカル センテラ エアフィット サンクリーム プラス 50ml 2個</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F512" t="n">
+        <v>3984</v>
+      </c>
+      <c r="G512" t="n">
+        <v>0</v>
+      </c>
+      <c r="H512" t="b">
+        <v>0</v>
+      </c>
+      <c r="I512" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J512" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154991907</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>1162421706</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>クラシック ウォームコットン EDP 30ml SP （香水）</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>クリーン</t>
+        </is>
+      </c>
+      <c r="F513" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G513" t="n">
+        <v>0</v>
+      </c>
+      <c r="H513" t="b">
+        <v>0</v>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J513" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162421706</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>1159643310</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>ハッピー フォーメン EDC 50ml SP （香水）</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>クリニーク</t>
+        </is>
+      </c>
+      <c r="F514" t="n">
+        <v>3530</v>
+      </c>
+      <c r="G514" t="n">
+        <v>0</v>
+      </c>
+      <c r="H514" t="b">
+        <v>0</v>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J514" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159643310</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>1158430479</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>アベンヌウォーター 300ml 3本セット （化粧水）</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>アベンヌ</t>
+        </is>
+      </c>
+      <c r="F515" t="n">
+        <v>3620</v>
+      </c>
+      <c r="G515" t="n">
+        <v>3</v>
+      </c>
+      <c r="H515" t="b">
+        <v>0</v>
+      </c>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J515" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158430479</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>1110913352</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>hottempr</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Olive Young ideal FOR MEN パーフェクト オールインワン企画 (オールインワン150ml+150ml)</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>アイデアルforメンズ</t>
+        </is>
+      </c>
+      <c r="F516" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G516" t="n">
+        <v>0</v>
+      </c>
+      <c r="H516" t="b">
+        <v>0</v>
+      </c>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J516" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1110913352</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>1193980815</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>hottempr</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>【産毛スタイリング】ハイプフィットヘアケアマスカラ／ハードフィックスヘアマスカラ／エギョモリ／バーコード前髪／韓国アイドルヘア／アホ毛スティック／前髪アレンジ</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>narka</t>
+        </is>
+      </c>
+      <c r="F517" t="n">
+        <v>2960</v>
+      </c>
+      <c r="G517" t="n">
+        <v>0</v>
+      </c>
+      <c r="H517" t="b">
+        <v>0</v>
+      </c>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J517" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193980815</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>1203744619</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>treasurebeauty</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>ベルベット クレンジング ミルク 200ml x 2 お得な2個セット</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>クラランス</t>
+        </is>
+      </c>
+      <c r="F518" t="n">
+        <v>6230</v>
+      </c>
+      <c r="G518" t="n">
+        <v>0</v>
+      </c>
+      <c r="H518" t="b">
+        <v>0</v>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203744619</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>1173946856</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>treasurebeauty</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>デイリーPD 50ml/1.7fl.oz.</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>ZO SKIN</t>
+        </is>
+      </c>
+      <c r="F519" t="n">
+        <v>21465</v>
+      </c>
+      <c r="G519" t="n">
+        <v>0</v>
+      </c>
+      <c r="H519" t="b">
+        <v>0</v>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1173946856</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>1154827017</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>treasurebeauty</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>メン ハード バーム 60g</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>アリミノ</t>
+        </is>
+      </c>
+      <c r="F520" t="n">
+        <v>1979</v>
+      </c>
+      <c r="G520" t="n">
+        <v>0</v>
+      </c>
+      <c r="H520" t="b">
+        <v>0</v>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154827017</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J497"/>
+  <autoFilter ref="A1:J520"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 63, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$520</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$530</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J520"/>
+  <dimension ref="A1:J530"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21775,8 +21775,418 @@
         </is>
       </c>
     </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>1204744207</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>TOMOSONGSTORE</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>リードルショット 300 50ml 2個セット（1+1）</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F521" t="n">
+        <v>8720</v>
+      </c>
+      <c r="G521" t="n">
+        <v>0</v>
+      </c>
+      <c r="H521" t="b">
+        <v>0</v>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J521" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204744207</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>1206857284</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>k_town</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>【正規品】コンブチャミスト 100ml + 選べるプレゼント / スペシャルケアマスクパック</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>エリシャコイ</t>
+        </is>
+      </c>
+      <c r="F522" t="n">
+        <v>2123</v>
+      </c>
+      <c r="G522" t="n">
+        <v>0</v>
+      </c>
+      <c r="H522" t="b">
+        <v>0</v>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J522" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206857284</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>1193149194</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>realkbeauty</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>[NEW] A.G.E. インタラプター ウルトラ弾力リフティングセラムセット(+4ml+ 4ml+ 4ml)＋スーパーカラゲンマスク</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>スキンシューティカルズ</t>
+        </is>
+      </c>
+      <c r="F523" t="n">
+        <v>21695</v>
+      </c>
+      <c r="G523" t="n">
+        <v>0</v>
+      </c>
+      <c r="H523" t="b">
+        <v>0</v>
+      </c>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J523" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193149194</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>1190578211</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>realkbeauty</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>デイリーマスク7種+1マスク/毛穴の弾力 ドングリ/ニキビ跡 ジャガイモ/水分保湿 キャロット/ビタユズ/美白 栄養ライス/肌の鎮静/バジルティーツリー</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F524" t="n">
+        <v>2450</v>
+      </c>
+      <c r="G524" t="n">
+        <v>0</v>
+      </c>
+      <c r="H524" t="b">
+        <v>0</v>
+      </c>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J524" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190578211</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>1139807140</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>gpgp</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>パルファムボディウォッシュ/ 500ml/ 2個</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>ミルクバオバブ</t>
+        </is>
+      </c>
+      <c r="F525" t="n">
+        <v>3492</v>
+      </c>
+      <c r="G525" t="n">
+        <v>0</v>
+      </c>
+      <c r="H525" t="b">
+        <v>0</v>
+      </c>
+      <c r="I525" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J525" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139807140</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>1139805675</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>gpgp</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>オードパルファム(07シュガーフローラル)/ 25ml/ 1個</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>After blow</t>
+        </is>
+      </c>
+      <c r="F526" t="n">
+        <v>5505</v>
+      </c>
+      <c r="G526" t="n">
+        <v>1</v>
+      </c>
+      <c r="H526" t="b">
+        <v>0</v>
+      </c>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J526" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139805675</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>1203684966</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>KBeautyCenter</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>elom トラブルスケーリングパッチマスク 3枚 /トラブルケア</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>EIoM</t>
+        </is>
+      </c>
+      <c r="F527" t="n">
+        <v>2490</v>
+      </c>
+      <c r="G527" t="n">
+        <v>0</v>
+      </c>
+      <c r="H527" t="b">
+        <v>0</v>
+      </c>
+      <c r="I527" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J527" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203684966</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>1179656795</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>KBeautyCenter</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>こすアールエックス ワンステップパッド/おじさんパッド/ピンプルパッド 70枚</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F528" t="n">
+        <v>3490</v>
+      </c>
+      <c r="G528" t="n">
+        <v>0</v>
+      </c>
+      <c r="H528" t="b">
+        <v>0</v>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J528" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179656795</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>1190674241</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>KBeautyCenter</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>カロテンクラリファイングビタパッド, 60枚</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>エイプリルスキン</t>
+        </is>
+      </c>
+      <c r="F529" t="n">
+        <v>3590</v>
+      </c>
+      <c r="G529" t="n">
+        <v>0</v>
+      </c>
+      <c r="H529" t="b">
+        <v>0</v>
+      </c>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J529" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190674241</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>1202082347</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>lindalinda</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>【垢すり/角質ケア】ソフトボディ レッドグローブ クリーン 1BOX(5枚入) / 個包装 / ボディクレンジング / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>ランドリーユー</t>
+        </is>
+      </c>
+      <c r="F530" t="n">
+        <v>2520</v>
+      </c>
+      <c r="G530" t="n">
+        <v>5</v>
+      </c>
+      <c r="H530" t="b">
+        <v>0</v>
+      </c>
+      <c r="I530" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J530" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202082347</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J520"/>
+  <autoFilter ref="A1:J530"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 66, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$530</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$541</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J530"/>
+  <dimension ref="A1:J541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22185,8 +22185,459 @@
         </is>
       </c>
     </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>1138225289</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>dreamus</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>シグネチャーパルファム, 50ml, 1個</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>FORMENT</t>
+        </is>
+      </c>
+      <c r="F531" t="n">
+        <v>5517</v>
+      </c>
+      <c r="G531" t="n">
+        <v>0</v>
+      </c>
+      <c r="H531" t="b">
+        <v>0</v>
+      </c>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138225289</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>1109209881</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>korkorshop</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>[NEW]ヒストラップイージーエフコンプレックスアンプル63％80ml / EGF</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>HISTOLAB</t>
+        </is>
+      </c>
+      <c r="F532" t="n">
+        <v>9737</v>
+      </c>
+      <c r="G532" t="n">
+        <v>0</v>
+      </c>
+      <c r="H532" t="b">
+        <v>0</v>
+      </c>
+      <c r="I532" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J532" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1109209881</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>1211103356</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>iS2japan</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>ツバキディープコラーゲン弾力アンプル, 30ml</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F533" t="n">
+        <v>2160</v>
+      </c>
+      <c r="G533" t="n">
+        <v>0</v>
+      </c>
+      <c r="H533" t="b">
+        <v>0</v>
+      </c>
+      <c r="I533" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J533" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211103356</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>1192583562</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>iS2japan</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>ツバキディープコラーゲン弾力クリーム, 50ml</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F534" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G534" t="n">
+        <v>0</v>
+      </c>
+      <c r="H534" t="b">
+        <v>0</v>
+      </c>
+      <c r="I534" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J534" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192583562</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>1192583554</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>iS2japan</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>[正規品] Biodance ハイドロセラノールアンプル, 30ml</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F535" t="n">
+        <v>2450</v>
+      </c>
+      <c r="G535" t="n">
+        <v>0</v>
+      </c>
+      <c r="H535" t="b">
+        <v>0</v>
+      </c>
+      <c r="I535" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J535" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192583554</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>1213549964</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>CHERIBEAU</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>【SEVENTEEN ミンギュ ミニスタンディ2種付き】アノブ 選べるヘアケアセット / ヘアオイル / 洗い流さないトリートメント / シャンプー / ヘアマスク / 韓国ヘアケア</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F536" t="n">
+        <v>5170</v>
+      </c>
+      <c r="G536" t="n">
+        <v>0</v>
+      </c>
+      <c r="H536" t="b">
+        <v>0</v>
+      </c>
+      <c r="I536" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213549964</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>1206876078</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>CHERIBEAU</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>[1+1] 復活草ビフィダセラム ファーミングドロップ 50ml</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F537" t="n">
+        <v>3660</v>
+      </c>
+      <c r="G537" t="n">
+        <v>0</v>
+      </c>
+      <c r="H537" t="b">
+        <v>0</v>
+      </c>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J537" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206876078</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>1194719971</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>CHERIBEAU</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>アイラッシュ ティンティング セラム ショット 1個</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>ミュード</t>
+        </is>
+      </c>
+      <c r="F538" t="n">
+        <v>1790</v>
+      </c>
+      <c r="G538" t="n">
+        <v>1</v>
+      </c>
+      <c r="H538" t="b">
+        <v>0</v>
+      </c>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J538" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194719971</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>1211535086</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>DEARHOUR</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>【選べる2点SET】PDRNゼリーセラムミスト/キャビアPDRNリアルディープマスク(4枚)/PDRNリポソームバブルブースター</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F539" t="n">
+        <v>3650</v>
+      </c>
+      <c r="G539" t="n">
+        <v>0</v>
+      </c>
+      <c r="H539" t="b">
+        <v>0</v>
+      </c>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J539" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211535086</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>1073637416</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>DEARHOUR</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>バイタル ハイドラ ソリューション ハイドロプランプ ウォータークリーム 50ml 1EA</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F540" t="n">
+        <v>3170</v>
+      </c>
+      <c r="G540" t="n">
+        <v>0</v>
+      </c>
+      <c r="H540" t="b">
+        <v>0</v>
+      </c>
+      <c r="I540" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J540" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1073637416</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>1073637368</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>DEARHOUR</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>シカペア スリーペア インテンシブ S リペア マスク 75ml 1EA</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F541" t="n">
+        <v>3340</v>
+      </c>
+      <c r="G541" t="n">
+        <v>0</v>
+      </c>
+      <c r="H541" t="b">
+        <v>0</v>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J541" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1073637368</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J530"/>
+  <autoFilter ref="A1:J541"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 69, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$541</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$549</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J541"/>
+  <dimension ref="A1:J549"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22636,8 +22636,336 @@
         </is>
       </c>
     </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>1141815797</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>skincept</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>[正規品] ヒョヨン 自養(ジャヤン) アイクリーム30ml+クリーム15ml贈呈_蓮華ステムセル/ハリ_目元の弾力/保湿/集中栄養ケア</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>クダモノナラ</t>
+        </is>
+      </c>
+      <c r="F542" t="n">
+        <v>2950</v>
+      </c>
+      <c r="G542" t="n">
+        <v>1</v>
+      </c>
+      <c r="H542" t="b">
+        <v>0</v>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J542" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1141815797</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>1194263979</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>skincept</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>[1+1] フレグランスボディウォッシュ 600mlx2個セット_選べる2種 [White Musk/Citrus]_ブライトニング/パフューム ボディクレンザー</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>VEILMENT</t>
+        </is>
+      </c>
+      <c r="F543" t="n">
+        <v>3700</v>
+      </c>
+      <c r="G543" t="n">
+        <v>0</v>
+      </c>
+      <c r="H543" t="b">
+        <v>0</v>
+      </c>
+      <c r="I543" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J543" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194263979</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>1080048114</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>hy_international</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>ルミワイズブライトニングアンプルセラム30mL</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>雪花秀</t>
+        </is>
+      </c>
+      <c r="F544" t="n">
+        <v>12299</v>
+      </c>
+      <c r="G544" t="n">
+        <v>0</v>
+      </c>
+      <c r="H544" t="b">
+        <v>0</v>
+      </c>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J544" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1080048114</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>1067976758</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>hy_international</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>クレンジングミルク500ml/カレンデュラクリーム75ml</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>Bioturm</t>
+        </is>
+      </c>
+      <c r="F545" t="n">
+        <v>6299</v>
+      </c>
+      <c r="G545" t="n">
+        <v>0</v>
+      </c>
+      <c r="H545" t="b">
+        <v>0</v>
+      </c>
+      <c r="I545" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J545" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1067976758</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>1210139793</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>hy_international</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>UV プロテクター トーンアップ ピーチ / ラベンダー 50ml SPF50+ PA++++ トーンアップ 日焼け止め UVカット＆保湿ケア</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>ヘラ</t>
+        </is>
+      </c>
+      <c r="F546" t="n">
+        <v>3699</v>
+      </c>
+      <c r="G546" t="n">
+        <v>0</v>
+      </c>
+      <c r="H546" t="b">
+        <v>0</v>
+      </c>
+      <c r="I546" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210139793</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>1172777299</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>fmalwm</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>パフューム ヘアミスト サンセットフォグ 100ml 1個</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>ハクスリー</t>
+        </is>
+      </c>
+      <c r="F547" t="n">
+        <v>5833</v>
+      </c>
+      <c r="G547" t="n">
+        <v>0</v>
+      </c>
+      <c r="H547" t="b">
+        <v>0</v>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172777299</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>1160698785</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>DRsChoice</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>ジェントルマンオードパルファム50ml（3種類の香り）</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>I GENTLEMAN</t>
+        </is>
+      </c>
+      <c r="F548" t="n">
+        <v>5890</v>
+      </c>
+      <c r="G548" t="n">
+        <v>0</v>
+      </c>
+      <c r="H548" t="b">
+        <v>0</v>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160698785</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>1160698982</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>DRsChoice</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>ジェニーハウスプレミアムヘアカラー1+1企画セット5種類から選1</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>ジェニーハウス</t>
+        </is>
+      </c>
+      <c r="F549" t="n">
+        <v>3480</v>
+      </c>
+      <c r="G549" t="n">
+        <v>1</v>
+      </c>
+      <c r="H549" t="b">
+        <v>0</v>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160698982</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J541"/>
+  <autoFilter ref="A1:J549"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 72, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$549</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$561</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J549"/>
+  <dimension ref="A1:J561"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22964,8 +22964,500 @@
         </is>
       </c>
     </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>1202568510</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>HonestHouse</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>プロテインクリニック 10000 タンパク質 1L (シャンプー／トリートメント)</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>エラスティン</t>
+        </is>
+      </c>
+      <c r="F550" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G550" t="n">
+        <v>0</v>
+      </c>
+      <c r="H550" t="b">
+        <v>0</v>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202568510</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>1191542494</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>HonestHouse</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>モデリングパック スーパーレモン グルタチオン 10個</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F551" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G551" t="n">
+        <v>0</v>
+      </c>
+      <c r="H551" t="b">
+        <v>0</v>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191542494</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>1209154400</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>AnchorBlue</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>[密着ハリツヤ/5枚入] コラーゲン 100 メルティング シート マスク 2.5g x 5枚 / 濃密 潤い 水分 パッチ 弾力 肌キメ ス킨케어 高保湿 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F552" t="n">
+        <v>7376</v>
+      </c>
+      <c r="G552" t="n">
+        <v>0</v>
+      </c>
+      <c r="H552" t="b">
+        <v>0</v>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J552" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209154400</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>1208338165</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>AnchorBlue</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>[サロン級ホームケア] エクストリーム ダメージ クリニック ヘア アンプル 10ml 9個入り / 傷んだ髪 高濃縮 補修 保湿 ツヤ髪 トリートメント 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F553" t="n">
+        <v>3818</v>
+      </c>
+      <c r="G553" t="n">
+        <v>0</v>
+      </c>
+      <c r="H553" t="b">
+        <v>0</v>
+      </c>
+      <c r="I553" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J553" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208338165</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>1199411031</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Seoullys</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>[2+2] 白樺 水分 日焼け止めスプレー, 100ml 4ea(SPF 50 + PA ++++)</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F554" t="n">
+        <v>6007</v>
+      </c>
+      <c r="G554" t="n">
+        <v>0</v>
+      </c>
+      <c r="H554" t="b">
+        <v>0</v>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199411031</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>1136125175</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Seoullys</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>テラクネ 365 ハイドロ アクティブ トナー 化粧水, 200ml</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F555" t="n">
+        <v>2967</v>
+      </c>
+      <c r="G555" t="n">
+        <v>5</v>
+      </c>
+      <c r="H555" t="b">
+        <v>0</v>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J555" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1136125175</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>1143335244</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>jjunabeauty</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>[CLAIR-GYN]クレアジン 女性ウォッシュ 200ml+50ml, 1個</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>Hanmi PRO-CALM</t>
+        </is>
+      </c>
+      <c r="F556" t="n">
+        <v>2467</v>
+      </c>
+      <c r="G556" t="n">
+        <v>0</v>
+      </c>
+      <c r="H556" t="b">
+        <v>0</v>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J556" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1143335244</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>1129888999</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>jjunabeauty</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>スージング リペアクリーム R4, 50ml, 1個</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>DERMAFIRM</t>
+        </is>
+      </c>
+      <c r="F557" t="n">
+        <v>3828</v>
+      </c>
+      <c r="G557" t="n">
+        <v>0</v>
+      </c>
+      <c r="H557" t="b">
+        <v>0</v>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J557" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1129888999</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>1202055978</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>yeppun</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>UVクリーム SPF50+ PA ++++ 敏感肌向けトーンアップ韓国コスメの人気日焼け止め</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F558" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G558" t="n">
+        <v>0</v>
+      </c>
+      <c r="H558" t="b">
+        <v>0</v>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J558" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202055978</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>1174315936</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>yeppun</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>1. マデカラボ マスク 10枚×2箱（リンクル リバイタライズ）</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F559" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G559" t="n">
+        <v>0</v>
+      </c>
+      <c r="H559" t="b">
+        <v>0</v>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174315936</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>1087617512</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>QueenMall</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>パフューム スプレー ボディローション 250ml 5種</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>hedn</t>
+        </is>
+      </c>
+      <c r="F560" t="n">
+        <v>4320</v>
+      </c>
+      <c r="G560" t="n">
+        <v>1</v>
+      </c>
+      <c r="H560" t="b">
+        <v>0</v>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1087617512</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>1170080586</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>QueenMall</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>PDRN ピンク ジェル ツーフォーム クレンザー 200ml 企画(+クレンジングブラシ 贈呈)</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F561" t="n">
+        <v>2972</v>
+      </c>
+      <c r="G561" t="n">
+        <v>0</v>
+      </c>
+      <c r="H561" t="b">
+        <v>0</v>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170080586</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J549"/>
+  <autoFilter ref="A1:J561"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 75, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$561</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$570</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J561"/>
+  <dimension ref="A1:J570"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23456,8 +23456,377 @@
         </is>
       </c>
     </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>1199098148</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>kiri</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>[モンチッチコラボ] ベージュトーンアップ365ヴィーガンサンクリーム 40ml SPF50 トーンアップUV ノーファンデ 化粧下地 韓国日焼け止め</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>アミューズ</t>
+        </is>
+      </c>
+      <c r="F562" t="n">
+        <v>3470</v>
+      </c>
+      <c r="G562" t="n">
+        <v>1</v>
+      </c>
+      <c r="H562" t="b">
+        <v>0</v>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J562" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199098148</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>1109779971</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>K--beautyshop</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>[V T] リードルショット 2ステップ マスク 5枚セット (50/100/300) 針美容 毛穴 導入 フェイスパック 集中ケア スキンケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F563" t="n">
+        <v>2739</v>
+      </c>
+      <c r="G563" t="n">
+        <v>0</v>
+      </c>
+      <c r="H563" t="b">
+        <v>0</v>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1109779971</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>1192596376</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>K--beautyshop</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>[メガ割] manyo factory 魔女工場 ガラクナイアシン エッセンス クリーム 50ml ガラクトミセス 保湿 弾力 ハリ ツヤ 潤い 浸透 スキンケア 基礎化粧品 韓国コスメ 人気 公式</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F564" t="n">
+        <v>4726</v>
+      </c>
+      <c r="G564" t="n">
+        <v>0</v>
+      </c>
+      <c r="H564" t="b">
+        <v>0</v>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192596376</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>1193869990</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>K--beautyshop</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>[1+1特典] S*NATURE エ*スネイチャー アクア スクワラン 水分クリーム 2個セット 120ml 保湿 ツヤ肌 卵肌 韓国 スキンケア オリーブヤング プレゼント 敏感肌 乾燥肌</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>エスネイチャー</t>
+        </is>
+      </c>
+      <c r="F565" t="n">
+        <v>3930</v>
+      </c>
+      <c r="G565" t="n">
+        <v>0</v>
+      </c>
+      <c r="H565" t="b">
+        <v>0</v>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193869990</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>1190058759</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>slowhummingjp</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>【Slow Humming公式】フルーティナリーリリーフパフュームバーム 6.5g タッチピーチ/練り香水/香水/パヒューム/ヘアパヒューム</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>Slow Humming</t>
+        </is>
+      </c>
+      <c r="F566" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G566" t="n">
+        <v>0</v>
+      </c>
+      <c r="H566" t="b">
+        <v>0</v>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190058759</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>1135414332</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>calluna</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>[ギフト包装] ミスト セラム 100ml + ハンドクリーム 30ml + 鏡</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F567" t="n">
+        <v>3934</v>
+      </c>
+      <c r="G567" t="n">
+        <v>2</v>
+      </c>
+      <c r="H567" t="b">
+        <v>0</v>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135414332</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>1170532806</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>calluna</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>【ポムポムプリン限定企画】ビーガンパックレンザー3種択1 (グリーントマト120ml/ レッドトマト120ml/ ライスドウ130ml)</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>FULLY</t>
+        </is>
+      </c>
+      <c r="F568" t="n">
+        <v>2525</v>
+      </c>
+      <c r="G568" t="n">
+        <v>3</v>
+      </c>
+      <c r="H568" t="b">
+        <v>0</v>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170532806</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>1102457193</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>JJDD</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>ブランマジックティーツリーオイル 20ml 5倍高濃縮ティーツリー成分 /ニキビ超急速ケア/赤ニキビ,白ニキビ,大人ニキビ,思春期ニキビ,ニキビ跡</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>ブランネイチャー</t>
+        </is>
+      </c>
+      <c r="F569" t="n">
+        <v>2350</v>
+      </c>
+      <c r="G569" t="n">
+        <v>1</v>
+      </c>
+      <c r="H569" t="b">
+        <v>0</v>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1102457193</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>1081864235</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>kor-store</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>テリーファーマー 160g スタンダード ホテルタオル 10枚 タオル タオルセット タオル 洗面タオル 輪</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>Terry Special</t>
+        </is>
+      </c>
+      <c r="F570" t="n">
+        <v>4930</v>
+      </c>
+      <c r="G570" t="n">
+        <v>0</v>
+      </c>
+      <c r="H570" t="b">
+        <v>0</v>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J570" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1081864235</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J561"/>
+  <autoFilter ref="A1:J570"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 78, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$570</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$583</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J570"/>
+  <dimension ref="A1:J583"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23825,8 +23825,541 @@
         </is>
       </c>
     </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>1129908462</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>leelix</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>PHセンシティブ クリーム 60ml x 2個セット (チューブタイプ 高保湿 敏感肌)</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>サミュ</t>
+        </is>
+      </c>
+      <c r="F571" t="n">
+        <v>9322</v>
+      </c>
+      <c r="G571" t="n">
+        <v>0</v>
+      </c>
+      <c r="H571" t="b">
+        <v>0</v>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J571" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1129908462</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>1132004375</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>leelix</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>フルフィット プロポリス ライト アンプル 40ml +40ml</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F572" t="n">
+        <v>3996</v>
+      </c>
+      <c r="G572" t="n">
+        <v>1</v>
+      </c>
+      <c r="H572" t="b">
+        <v>0</v>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J572" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1132004375</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>1211243856</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Seoulika</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>【クレヨンしんちゃんコラボ】 スーパーメルティングセバムソフトナー 150ml 企画セット (+ステッカー2種+ブラックヘッドリムーバー+コットン40枚)</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>ilso</t>
+        </is>
+      </c>
+      <c r="F573" t="n">
+        <v>2669</v>
+      </c>
+      <c r="G573" t="n">
+        <v>1</v>
+      </c>
+      <c r="H573" t="b">
+        <v>0</v>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211243856</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>1207298088</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Seoulika</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>[ポケモン コラボ] グロウターン 3Dボリュームシャンプー 大容量 500ml 企画 セット(+100ml+キーホルダーポーチ)</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>lily eve</t>
+        </is>
+      </c>
+      <c r="F574" t="n">
+        <v>3092</v>
+      </c>
+      <c r="G574" t="n">
+        <v>0</v>
+      </c>
+      <c r="H574" t="b">
+        <v>0</v>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207298088</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>1101761023</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>sharonne</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>[NEW]オールデイ ノーセバム トーンアップ サンクッション / SPF50+ PA++++ / UVカット / トーンアップ / ノーセバム / 日焼け止め</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>ミルクタッチ</t>
+        </is>
+      </c>
+      <c r="F575" t="n">
+        <v>3321</v>
+      </c>
+      <c r="G575" t="n">
+        <v>1</v>
+      </c>
+      <c r="H575" t="b">
+        <v>0</v>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J575" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1101761023</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>1074817764</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>sharonne</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>紅茶栄養頭皮シャンプー450ml</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>ANILLO</t>
+        </is>
+      </c>
+      <c r="F576" t="n">
+        <v>6124</v>
+      </c>
+      <c r="G576" t="n">
+        <v>0</v>
+      </c>
+      <c r="H576" t="b">
+        <v>0</v>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1074817764</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>1188002169</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>steadyseller</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>リフティングクリーム 1618 グローラディアンス 保湿 50ml</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>AlpenMOOR1618</t>
+        </is>
+      </c>
+      <c r="F577" t="n">
+        <v>1690</v>
+      </c>
+      <c r="G577" t="n">
+        <v>0</v>
+      </c>
+      <c r="H577" t="b">
+        <v>0</v>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J577" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188002169</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>1179082021</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>steadyseller</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>エクソソーム PDRN ブースター アンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>IZEZE</t>
+        </is>
+      </c>
+      <c r="F578" t="n">
+        <v>3650</v>
+      </c>
+      <c r="G578" t="n">
+        <v>0</v>
+      </c>
+      <c r="H578" t="b">
+        <v>0</v>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J578" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179082021</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>1204443091</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>steadyseller</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>プレミアム水染め 3+3リフィル企画 3種 択1</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>SEEDBEE</t>
+        </is>
+      </c>
+      <c r="F579" t="n">
+        <v>4470</v>
+      </c>
+      <c r="G579" t="n">
+        <v>0</v>
+      </c>
+      <c r="H579" t="b">
+        <v>0</v>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204443091</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>1067475495</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>A-HASHOP</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>ビタミンヒアルロニックアンプルトナー 150mL&amp;amp;エマルジョン150mL企画(クリーム30mL贈呈)</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F580" t="n">
+        <v>4988</v>
+      </c>
+      <c r="G580" t="n">
+        <v>0</v>
+      </c>
+      <c r="H580" t="b">
+        <v>0</v>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J580" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1067475495</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>1072009140</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>KOR--STORE</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>バイオ スキン クレンジング パッド 6g 30枚入 x 2</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>EKE</t>
+        </is>
+      </c>
+      <c r="F581" t="n">
+        <v>5250</v>
+      </c>
+      <c r="G581" t="n">
+        <v>0</v>
+      </c>
+      <c r="H581" t="b">
+        <v>0</v>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1072009140</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>1079690675</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>KOR--STORE</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>CELL LINE PRO リペアクリーム [100口] 半永久化粧材料 アフターケア 1g100個入り</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>Clear_pro</t>
+        </is>
+      </c>
+      <c r="F582" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G582" t="n">
+        <v>0</v>
+      </c>
+      <c r="H582" t="b">
+        <v>0</v>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J582" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1079690675</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>1142729311</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>CreatorBUBU</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>[SNP] Glutathione Dark Zero Toning Patch 60ea, Gold Collagen Perfection Eye Patch 60ea</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>SNP</t>
+        </is>
+      </c>
+      <c r="F583" t="n">
+        <v>3236</v>
+      </c>
+      <c r="G583" t="n">
+        <v>0</v>
+      </c>
+      <c r="H583" t="b">
+        <v>0</v>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J583" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142729311</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J570"/>
+  <autoFilter ref="A1:J583"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 81, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$583</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$595</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J583"/>
+  <dimension ref="A1:J595"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24358,8 +24358,500 @@
         </is>
       </c>
     </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>1117324982</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>goldstarstore</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>西洋プラムピンクグルタチオンデイリースペシャルマスク 30枚入 1個</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>ミルクタッチ</t>
+        </is>
+      </c>
+      <c r="F584" t="n">
+        <v>5075</v>
+      </c>
+      <c r="G584" t="n">
+        <v>0</v>
+      </c>
+      <c r="H584" t="b">
+        <v>0</v>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1117324982</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>1207285368</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>goldstarstore</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>アルガンエッセンシャルディープケアヘアパック大容量470ml 1個</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F585" t="n">
+        <v>2660</v>
+      </c>
+      <c r="G585" t="n">
+        <v>0</v>
+      </c>
+      <c r="H585" t="b">
+        <v>0</v>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J585" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207285368</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>1201631207</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>goldstarstore</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>ルートジェン脱毛症状専門ケア頭皮エッセンス80ml 2個</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>呂</t>
+        </is>
+      </c>
+      <c r="F586" t="n">
+        <v>3755</v>
+      </c>
+      <c r="G586" t="n">
+        <v>0</v>
+      </c>
+      <c r="H586" t="b">
+        <v>0</v>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J586" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201631207</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>1164356074</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>goldstarstore</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>アドベンスドスネイル92オールインワンチューブ型クリーム100g 1個</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F587" t="n">
+        <v>3440</v>
+      </c>
+      <c r="G587" t="n">
+        <v>0</v>
+      </c>
+      <c r="H587" t="b">
+        <v>0</v>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164356074</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>1188963997</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Qoo10JapanDaae</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>タイムレボリューション ザ ファースト エッセンス パッド 250ml 75枚入 1個</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F588" t="n">
+        <v>3011</v>
+      </c>
+      <c r="G588" t="n">
+        <v>0</v>
+      </c>
+      <c r="H588" t="b">
+        <v>0</v>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188963997</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>1175139603</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Qoo10JapanDaae</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>モイスチャー バランシング 無シリコン シャンプー 530ml 1個</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>アドル</t>
+        </is>
+      </c>
+      <c r="F589" t="n">
+        <v>3743</v>
+      </c>
+      <c r="G589" t="n">
+        <v>0</v>
+      </c>
+      <c r="H589" t="b">
+        <v>0</v>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175139603</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>1139814745</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>vip_s</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>ティルティールオフザサンエアムース/ 40ml/ 1個</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>ティルティル</t>
+        </is>
+      </c>
+      <c r="F590" t="n">
+        <v>2247</v>
+      </c>
+      <c r="G590" t="n">
+        <v>0</v>
+      </c>
+      <c r="H590" t="b">
+        <v>0</v>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139814745</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>1151569871</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>vip_s</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>デイリー アンチヘアロス タンパク質 トリートメント 500ml</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>ダシュ</t>
+        </is>
+      </c>
+      <c r="F591" t="n">
+        <v>3048</v>
+      </c>
+      <c r="G591" t="n">
+        <v>1</v>
+      </c>
+      <c r="H591" t="b">
+        <v>0</v>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151569871</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>1097995675</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>kor_shop</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>ルビーセル最新本物の保護マイルドラインミルク50ml強力で純粋なデイリーラインミルク50+</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>Ruby-Cell</t>
+        </is>
+      </c>
+      <c r="F592" t="n">
+        <v>5826</v>
+      </c>
+      <c r="G592" t="n">
+        <v>0</v>
+      </c>
+      <c r="H592" t="b">
+        <v>0</v>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J592" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097995675</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>1141190063</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>korchannel</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>[1+1]トゥクールフォースクールアートクラスアーティストモチパフ</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>トゥークールフォースクール</t>
+        </is>
+      </c>
+      <c r="F593" t="n">
+        <v>2430</v>
+      </c>
+      <c r="G593" t="n">
+        <v>1</v>
+      </c>
+      <c r="H593" t="b">
+        <v>0</v>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J593" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1141190063</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>1141209058</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>korchannel</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>ユーソプルニチ香水ベリーノワール50ml 30代男性香水</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>YOUSSOFUL</t>
+        </is>
+      </c>
+      <c r="F594" t="n">
+        <v>11610</v>
+      </c>
+      <c r="G594" t="n">
+        <v>1</v>
+      </c>
+      <c r="H594" t="b">
+        <v>0</v>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1141209058</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>1210683594</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>82lounge</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>メディAHAクリーム 25ml :: AHAクリーム / クリーム 角質除去 / クリーム スポットケア / クリーム ニキビ</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F595" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G595" t="n">
+        <v>0</v>
+      </c>
+      <c r="H595" t="b">
+        <v>0</v>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210683594</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J583"/>
+  <autoFilter ref="A1:J595"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 84, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$595</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$614</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J595"/>
+  <dimension ref="A1:J614"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24850,8 +24850,787 @@
         </is>
       </c>
     </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>1158685803</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>hahahaya</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>グリコリック アシッド 7% エクスポリエイティングトナー 100ml</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F596" t="n">
+        <v>1860</v>
+      </c>
+      <c r="G596" t="n">
+        <v>1</v>
+      </c>
+      <c r="H596" t="b">
+        <v>0</v>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158685803</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>1211859799</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>ゼロキャスト デイリー 透明 保湿サンスクリーン 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F597" t="n">
+        <v>3211</v>
+      </c>
+      <c r="G597" t="n">
+        <v>0</v>
+      </c>
+      <c r="H597" t="b">
+        <v>0</v>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211859799</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>1211855765</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>ビタC フォーストリックス トーニング セラムマスク 22ml 10枚</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F598" t="n">
+        <v>3173</v>
+      </c>
+      <c r="G598" t="n">
+        <v>0</v>
+      </c>
+      <c r="H598" t="b">
+        <v>0</v>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211855765</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>1209466651</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>ラクトリメディ レディース カミングクリーム 15ml</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>メディオン</t>
+        </is>
+      </c>
+      <c r="F599" t="n">
+        <v>5161</v>
+      </c>
+      <c r="G599" t="n">
+        <v>1</v>
+      </c>
+      <c r="H599" t="b">
+        <v>0</v>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209466651</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>1209446667</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>【クーリング/Yーンケア】ポエリエ フェミニン インナーパフューム デイリー マルチ香水</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>フォエリー</t>
+        </is>
+      </c>
+      <c r="F600" t="n">
+        <v>2331</v>
+      </c>
+      <c r="G600" t="n">
+        <v>1</v>
+      </c>
+      <c r="H600" t="b">
+        <v>0</v>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J600" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209446667</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>1172106877</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>KOREAMALL1</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>ジークップ ケアセラ エコアスノウ 硫黄石鹸 (4個入)</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>ケアセラ</t>
+        </is>
+      </c>
+      <c r="F601" t="n">
+        <v>3710</v>
+      </c>
+      <c r="G601" t="n">
+        <v>0</v>
+      </c>
+      <c r="H601" t="b">
+        <v>0</v>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J601" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172106877</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>1169173710</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>KOREAMALL1</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>ニューヨーク インティリー オードパルファムEDP 10ml</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>BiBiANG</t>
+        </is>
+      </c>
+      <c r="F602" t="n">
+        <v>7780</v>
+      </c>
+      <c r="G602" t="n">
+        <v>0</v>
+      </c>
+      <c r="H602" t="b">
+        <v>0</v>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J602" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169173710</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>1169173462</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>KOREAMALL1</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>ローストウッド オードパルファムEDP 10ml</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>BiBiANG</t>
+        </is>
+      </c>
+      <c r="F603" t="n">
+        <v>7780</v>
+      </c>
+      <c r="G603" t="n">
+        <v>0</v>
+      </c>
+      <c r="H603" t="b">
+        <v>0</v>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J603" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169173462</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>1181384570</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>KOREAMALL1</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>[ギャラリア] MADET LEN レッドムスク オードパルファム RED MUSC</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>MAD et LEN</t>
+        </is>
+      </c>
+      <c r="F604" t="n">
+        <v>63970</v>
+      </c>
+      <c r="G604" t="n">
+        <v>0</v>
+      </c>
+      <c r="H604" t="b">
+        <v>0</v>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181384570</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>1082804410</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>SuperStarK</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>【国内発送】 ターンオーバーアンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F605" t="n">
+        <v>5478</v>
+      </c>
+      <c r="G605" t="n">
+        <v>1</v>
+      </c>
+      <c r="H605" t="b">
+        <v>0</v>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1082804410</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>1200649177</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>cosmenana</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>ululis ウルリス プレミアム ウォーターコンク ブラックセラム ヘアオイル 100ml 黒[3559] 宅配無料</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>ululis</t>
+        </is>
+      </c>
+      <c r="F606" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G606" t="n">
+        <v>0</v>
+      </c>
+      <c r="H606" t="b">
+        <v>0</v>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200649177</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>1198894604</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>bestone1</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>ティファニー TIFFANY ＆ラブ フォーヒム EDT + ＆ラブ フォーハー EDP ミニ香水 セット 1.2ml×2 サンプル[6495] メール便無料[B][BP3]</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>Tiffany</t>
+        </is>
+      </c>
+      <c r="F607" t="n">
+        <v>3980</v>
+      </c>
+      <c r="G607" t="n">
+        <v>1</v>
+      </c>
+      <c r="H607" t="b">
+        <v>0</v>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198894604</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>1091387881</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>JUJUHONG</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>バイビード インアンドアウト マスクパック,1個入り,5個,/In &amp;amp; Out Facial Mask/毛穴の老廃物を除去</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>バイビッド</t>
+        </is>
+      </c>
+      <c r="F608" t="n">
+        <v>3690</v>
+      </c>
+      <c r="G608" t="n">
+        <v>5</v>
+      </c>
+      <c r="H608" t="b">
+        <v>0</v>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J608" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1091387881</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>1095687901</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>JUJUHONG</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>[KERASYS] ADVANCED KERAMIDE トリートメント！ ヘアパック！ シャンプー！ 人気商品集電線 1+1 [正規品] 韓国ブランド(鎮静/弾力/保湿/栄養供給/活力)</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F609" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G609" t="n">
+        <v>0</v>
+      </c>
+      <c r="H609" t="b">
+        <v>0</v>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J609" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1095687901</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>1101562835</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>JUJUHONG</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>ビフィダ バイオーム アンプル パッド 70枚</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F610" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G610" t="n">
+        <v>1</v>
+      </c>
+      <c r="H610" t="b">
+        <v>0</v>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J610" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1101562835</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>1094393233</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>GYUWOO</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>THEビタAレチナールショットタイトニングブースター 15ml</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F611" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G611" t="n">
+        <v>4</v>
+      </c>
+      <c r="H611" t="b">
+        <v>0</v>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J611" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1094393233</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>1103977398</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>GYUWOO</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>ノスカナゲル /アクノンクリーム /アクリンゲル /メラトーニンクリーム /メラノサ ヒドロキノン /Dパンテノール軟膏</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>東亜製薬</t>
+        </is>
+      </c>
+      <c r="F612" t="n">
+        <v>6256</v>
+      </c>
+      <c r="G612" t="n">
+        <v>0</v>
+      </c>
+      <c r="H612" t="b">
+        <v>0</v>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1103977398</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>1093319609</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>GYUWOO</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>THE ビタA レチノールセラム 30ml + レチナールブースター 15ml セット</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F613" t="n">
+        <v>4250</v>
+      </c>
+      <c r="G613" t="n">
+        <v>3</v>
+      </c>
+      <c r="H613" t="b">
+        <v>0</v>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093319609</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>1119598747</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>GYUWOO</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>ノニアクネバブルクレンザー 155ml</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F614" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G614" t="n">
+        <v>1</v>
+      </c>
+      <c r="H614" t="b">
+        <v>0</v>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1119598747</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J595"/>
+  <autoFilter ref="A1:J614"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 87, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$614</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$623</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J614"/>
+  <dimension ref="A1:J623"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25629,8 +25629,377 @@
         </is>
       </c>
     </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>1167121017</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>TwoK</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>リンゼイ 鎮静薬草モデリングパック (カップパック) 28g [66冠/1位]</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>LINDSAY</t>
+        </is>
+      </c>
+      <c r="F615" t="n">
+        <v>2278</v>
+      </c>
+      <c r="G615" t="n">
+        <v>1</v>
+      </c>
+      <c r="H615" t="b">
+        <v>0</v>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J615" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167121017</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>1204303349</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>TwoK</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>ラエル オーガニックコットンカバー 履くオーバーナイト M 2個入 x3個</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>ラエル</t>
+        </is>
+      </c>
+      <c r="F616" t="n">
+        <v>3059</v>
+      </c>
+      <c r="G616" t="n">
+        <v>0</v>
+      </c>
+      <c r="H616" t="b">
+        <v>0</v>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204303349</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>1202040262</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>TwoK</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>ジョソンアビューティ ワンダーバス レモンシロップ パッククレンザー 200ml (+50ml)</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>WONDER BATH</t>
+        </is>
+      </c>
+      <c r="F617" t="n">
+        <v>4332</v>
+      </c>
+      <c r="G617" t="n">
+        <v>0</v>
+      </c>
+      <c r="H617" t="b">
+        <v>0</v>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J617" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202040262</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>1199549438</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>sunnyline</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>クライオ ソルベ アイシー フェイシャル マスク (4個入) / クーリング 冷却 パック むくみケア</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F618" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G618" t="n">
+        <v>1</v>
+      </c>
+      <c r="H618" t="b">
+        <v>0</v>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J618" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199549438</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>1205600340</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>sunnyline</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>デカッソシド サンスティック エアリフィット 10g + 10g (1+1 セット) 日焼け止め スティック UVケア CICA 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F619" t="n">
+        <v>4200</v>
+      </c>
+      <c r="G619" t="n">
+        <v>0</v>
+      </c>
+      <c r="H619" t="b">
+        <v>0</v>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J619" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205600340</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>1204317855</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>sunnyline</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>プロテインボンド ウォーターエッセンス＋ピカチュウ ミラーコーム セット</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>ヘアプラス</t>
+        </is>
+      </c>
+      <c r="F620" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G620" t="n">
+        <v>1</v>
+      </c>
+      <c r="H620" t="b">
+        <v>0</v>
+      </c>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J620" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204317855</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>1119858758</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>KORKORMALL</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>エピエルアボカドオイル+ヒマワリオイル抽出モイスチャーハンドパック/バルパック12パック</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>epille</t>
+        </is>
+      </c>
+      <c r="F621" t="n">
+        <v>2137</v>
+      </c>
+      <c r="G621" t="n">
+        <v>1</v>
+      </c>
+      <c r="H621" t="b">
+        <v>0</v>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1119858758</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>1151670543</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>KORKORMALL</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>[国内百貨店]ディープディックフレッドポッドボディバーム200ml</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>ディプティック</t>
+        </is>
+      </c>
+      <c r="F622" t="n">
+        <v>16500</v>
+      </c>
+      <c r="G622" t="n">
+        <v>0</v>
+      </c>
+      <c r="H622" t="b">
+        <v>0</v>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J622" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151670543</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>1148898608</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>KORKORMALL</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>エバーセルセルバイタルセルチャージャーエッセンス14p252ml1個</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>エバーセル</t>
+        </is>
+      </c>
+      <c r="F623" t="n">
+        <v>8150</v>
+      </c>
+      <c r="G623" t="n">
+        <v>0</v>
+      </c>
+      <c r="H623" t="b">
+        <v>0</v>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J623" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1148898608</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J614"/>
+  <autoFilter ref="A1:J623"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 90, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$623</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$632</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J623"/>
+  <dimension ref="A1:J632"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25998,8 +25998,377 @@
         </is>
       </c>
     </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>1162204761</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>lifetipsshop</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>[NEW] クライオアイスマスク 30枚</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F624" t="n">
+        <v>2070</v>
+      </c>
+      <c r="G624" t="n">
+        <v>4</v>
+      </c>
+      <c r="H624" t="b">
+        <v>0</v>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J624" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162204761</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>1190357115</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>lifetipsshop</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>アゼライン酸CICAスキンクリアトナー 250ml</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F625" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G625" t="n">
+        <v>0</v>
+      </c>
+      <c r="H625" t="b">
+        <v>0</v>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J625" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190357115</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>1157789377</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>lifetipsshop</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>ドクダミLHAモイスチャーピーリングジェル 120ml</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F626" t="n">
+        <v>1710</v>
+      </c>
+      <c r="G626" t="n">
+        <v>0</v>
+      </c>
+      <c r="H626" t="b">
+        <v>0</v>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J626" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157789377</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>1148824104</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>HappyBGLD</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>【20%OFF 全ブランド跨ぎ割引】 イロン 当帰スディンゲル 500ml 大容量 水分エッセンス 肌バリア 赤み 속건조+マスクパックをプレゼント</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F627" t="n">
+        <v>7970</v>
+      </c>
+      <c r="G627" t="n">
+        <v>4</v>
+      </c>
+      <c r="H627" t="b">
+        <v>0</v>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J627" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1148824104</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>1176812478</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>meisonmatcha</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>[2個]トータルリペア5 ミラクル ヘアパック 170ml</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>LOREAL PARIS</t>
+        </is>
+      </c>
+      <c r="F628" t="n">
+        <v>1626</v>
+      </c>
+      <c r="G628" t="n">
+        <v>0</v>
+      </c>
+      <c r="H628" t="b">
+        <v>0</v>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J628" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176812478</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>1197665370</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>K-Life-Style</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>オンリーフォーマンオールインワンエッセンス 200ml 2個 皮脂ケア テカリ防止</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>AHC</t>
+        </is>
+      </c>
+      <c r="F629" t="n">
+        <v>5683</v>
+      </c>
+      <c r="G629" t="n">
+        <v>0</v>
+      </c>
+      <c r="H629" t="b">
+        <v>0</v>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J629" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197665370</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>1197665508</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>K-Life-Style</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>レッドブレミッシュフォーマン鎮静オールインワン 200ml 3個 お得 ストック</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F630" t="n">
+        <v>12618</v>
+      </c>
+      <c r="G630" t="n">
+        <v>0</v>
+      </c>
+      <c r="H630" t="b">
+        <v>0</v>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J630" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197665508</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>1197665474</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>K-Life-Style</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>メンズグッドルックスアイブローペンシル ナチュラルブラック 1個 目力 男子メイク</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>ダシュ</t>
+        </is>
+      </c>
+      <c r="F631" t="n">
+        <v>1921</v>
+      </c>
+      <c r="G631" t="n">
+        <v>0</v>
+      </c>
+      <c r="H631" t="b">
+        <v>0</v>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J631" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197665474</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>1197665466</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>K-Life-Style</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>広報ジンクリーム 50ml 1個 栄養補給 ツヤ</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>多娜嫺</t>
+        </is>
+      </c>
+      <c r="F632" t="n">
+        <v>2396</v>
+      </c>
+      <c r="G632" t="n">
+        <v>1</v>
+      </c>
+      <c r="H632" t="b">
+        <v>0</v>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J632" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197665466</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J623"/>
+  <autoFilter ref="A1:J632"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 93, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$632</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$639</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J632"/>
+  <dimension ref="A1:J639"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26367,8 +26367,295 @@
         </is>
       </c>
     </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>1047570493</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>SJOCEAN</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>[1+1] リアル ヒアルロニック 100 クリーム 80ml+80ml / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>WELLAGE</t>
+        </is>
+      </c>
+      <c r="F633" t="n">
+        <v>5040</v>
+      </c>
+      <c r="G633" t="n">
+        <v>0</v>
+      </c>
+      <c r="H633" t="b">
+        <v>0</v>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J633" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1047570493</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>1115552034</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>[1+1] [SNS, AMAZON 大人気] 米サンクリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F634" t="n">
+        <v>3558</v>
+      </c>
+      <c r="G634" t="n">
+        <v>0</v>
+      </c>
+      <c r="H634" t="b">
+        <v>0</v>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J634" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1115552034</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>1193643194</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>【正規品】【Qoo10人気】レチノールリペアセラム30ml ヴィーガンリポソームレチノール3%セラム</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>スキンアンドラブ</t>
+        </is>
+      </c>
+      <c r="F635" t="n">
+        <v>4736</v>
+      </c>
+      <c r="G635" t="n">
+        <v>0</v>
+      </c>
+      <c r="H635" t="b">
+        <v>0</v>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J635" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193643194</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>1193643034</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>【正規品】コラーゲンナイトラッピングマスク 75ml + ブラシ</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>メディキューブバイオ</t>
+        </is>
+      </c>
+      <c r="F636" t="n">
+        <v>1590</v>
+      </c>
+      <c r="G636" t="n">
+        <v>0</v>
+      </c>
+      <c r="H636" t="b">
+        <v>0</v>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193643034</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>1193642954</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>【正規品】[ライスシリーズ] 7 ライス セラミド グローセラム /ライス 70 インテンス モイスチャー ミルク /ライス ブライトニング酵素洗顔パウダー /ライス70 グロウミルキートナー</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F637" t="n">
+        <v>4516</v>
+      </c>
+      <c r="G637" t="n">
+        <v>0</v>
+      </c>
+      <c r="H637" t="b">
+        <v>0</v>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J637" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193642954</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>1193642948</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>GIVENCY 【正規品】 プリズム リーブル ミニパウダー No0/No1/No2/No3/No4 ジバンシイ プリズム リーブル PRISME LIBRE ルース パウダー</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>タンバリンズ</t>
+        </is>
+      </c>
+      <c r="F638" t="n">
+        <v>7570</v>
+      </c>
+      <c r="G638" t="n">
+        <v>0</v>
+      </c>
+      <c r="H638" t="b">
+        <v>0</v>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J638" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193642948</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>1197470722</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>mangobeautylab</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>ネイチャー シャンプー 詰め替え 4個セット ベビーパウダー 香り 400ml リフィル 大容量 まとめ買い 自然由来 家族用</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F639" t="n">
+        <v>5594</v>
+      </c>
+      <c r="G639" t="n">
+        <v>1</v>
+      </c>
+      <c r="H639" t="b">
+        <v>0</v>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J639" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197470722</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J632"/>
+  <autoFilter ref="A1:J639"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 96, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$639</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$657</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J639"/>
+  <dimension ref="A1:J657"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26654,8 +26654,746 @@
         </is>
       </c>
     </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>1121575025</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>unicornmall</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>バイオコラーゲンリアルディープマスク, 8枚/バイオコラーゲンリアルディープマスク(8枚入り)/高保湿/弾力毛穴ツヤ肌ケア/アンプル１個分をそのまま固めたハイドロゲル/べたつきかない/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F640" t="n">
+        <v>6655</v>
+      </c>
+      <c r="G640" t="n">
+        <v>3</v>
+      </c>
+      <c r="H640" t="b">
+        <v>0</v>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J640" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1121575025</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>1149796005</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>KLand</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>センテラ トーニングトナー 鎮静 シカ 化粧水 210ml</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F641" t="n">
+        <v>1974</v>
+      </c>
+      <c r="G641" t="n">
+        <v>0</v>
+      </c>
+      <c r="H641" t="b">
+        <v>0</v>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J641" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149796005</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>1157524219</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>KLand</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>バイオEXセルペプチド3種セット1個 水分・保湿・栄養・肌のハリ・シワケア</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>トニーモリー</t>
+        </is>
+      </c>
+      <c r="F642" t="n">
+        <v>5979</v>
+      </c>
+      <c r="G642" t="n">
+        <v>0</v>
+      </c>
+      <c r="H642" t="b">
+        <v>0</v>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J642" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157524219</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>1151012307</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>KLand</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>ドクダミポアコントロールクレンジングオイル 200ml</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F643" t="n">
+        <v>2691</v>
+      </c>
+      <c r="G643" t="n">
+        <v>1</v>
+      </c>
+      <c r="H643" t="b">
+        <v>0</v>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J643" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151012307</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>1172781112</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>KLand</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>[3点セット/企画構成/復活草マスクパック1枚贈呈]復活草 パハトナー200ml+復活草 ビフィダ セラム ファーミング ドロップ 50ml+復活草 クリーム ニュートリション チューブ 75ml</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F644" t="n">
+        <v>5819</v>
+      </c>
+      <c r="G644" t="n">
+        <v>0</v>
+      </c>
+      <c r="H644" t="b">
+        <v>0</v>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J644" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172781112</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>1155298751</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>KLand</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>【リニューアル】ゼロ毛穴 ワンデーセラム 30ml 1本 毛穴ケア 肌のキメ</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F645" t="n">
+        <v>2348</v>
+      </c>
+      <c r="G645" t="n">
+        <v>0</v>
+      </c>
+      <c r="H645" t="b">
+        <v>0</v>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J645" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1155298751</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>1200851127</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>mrm</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>PDRNヒアルロン酸カプセル100セラム30ml +モイスチャライジングクリーム30ml+ PDRN 100 ヒアルロン酸 ブースター トナー 250ml + 40ml</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F646" t="n">
+        <v>6880</v>
+      </c>
+      <c r="G646" t="n">
+        <v>4</v>
+      </c>
+      <c r="H646" t="b">
+        <v>0</v>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J646" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200851127</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>1200850420</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>mrm</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>PDRN ヒアルロン酸 水分カプセルミスト 100ml + 100ml / 保湿ミスト 韓国ブランド ミスト</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F647" t="n">
+        <v>4980</v>
+      </c>
+      <c r="G647" t="n">
+        <v>5</v>
+      </c>
+      <c r="H647" t="b">
+        <v>0</v>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J647" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200850420</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>1205030887</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>mrm</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>シラカバ保湿サンスティック + シラカバ水分サンクリーム [韓国サンスティック]</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F648" t="n">
+        <v>7380</v>
+      </c>
+      <c r="G648" t="n">
+        <v>2</v>
+      </c>
+      <c r="H648" t="b">
+        <v>0</v>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205030887</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>1201003595</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>mrm</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>PDRN ヒアルロン酸カプセル100 セラム 30ml + PDRN ヒアルロン酸 水分カプセルミスト 100ml</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F649" t="n">
+        <v>6980</v>
+      </c>
+      <c r="G649" t="n">
+        <v>2</v>
+      </c>
+      <c r="H649" t="b">
+        <v>0</v>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J649" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201003595</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>1152724729</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>MAYSHOP</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>ドクダミ77%スージングトナー, 250ml</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F650" t="n">
+        <v>1760</v>
+      </c>
+      <c r="G650" t="n">
+        <v>0</v>
+      </c>
+      <c r="H650" t="b">
+        <v>0</v>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152724729</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>1191147953</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>MAYSHOP</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>ピュア ボディミスト ベビーパウダーの香り 128ml 2個</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F651" t="n">
+        <v>1867</v>
+      </c>
+      <c r="G651" t="n">
+        <v>1</v>
+      </c>
+      <c r="H651" t="b">
+        <v>0</v>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191147953</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>1185851789</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>MAYSHOP</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>[1+1] レッド ラクト コラーゲン ラッピング マスクパック 70ml *2 + ブラシ</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F652" t="n">
+        <v>3587</v>
+      </c>
+      <c r="G652" t="n">
+        <v>1</v>
+      </c>
+      <c r="H652" t="b">
+        <v>0</v>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J652" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185851789</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>1157601678</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>MAYSHOP</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>[SET] プロテインダメージケアシャンプー500ml+トリートメント250ml</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F653" t="n">
+        <v>3630</v>
+      </c>
+      <c r="G653" t="n">
+        <v>4</v>
+      </c>
+      <c r="H653" t="b">
+        <v>0</v>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J653" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157601678</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>1152724831</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>MAYSHOP</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>6番 爆睡マスクパックセラム50ml</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F654" t="n">
+        <v>2360</v>
+      </c>
+      <c r="G654" t="n">
+        <v>0</v>
+      </c>
+      <c r="H654" t="b">
+        <v>0</v>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J654" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152724831</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>1208195309</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>klumin</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>パフュームシルキーハンドクリーム50ml フレグランス12種, ご購入でMEDIHEAL ローズPDRNマスク1枚プレゼント</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>ヘトラス</t>
+        </is>
+      </c>
+      <c r="F655" t="n">
+        <v>1940</v>
+      </c>
+      <c r="G655" t="n">
+        <v>0</v>
+      </c>
+      <c r="H655" t="b">
+        <v>0</v>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J655" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208195309</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>1209668463</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>klumin</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>[MEDIHEAL マスク1枚付き]ドクダミ77スージングトナー，350ml</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F656" t="n">
+        <v>2926</v>
+      </c>
+      <c r="G656" t="n">
+        <v>0</v>
+      </c>
+      <c r="H656" t="b">
+        <v>0</v>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J656" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209668463</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>1205779441</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>albami</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>エストラ アトバリア365 ハイドロ スージングクリーム 80ml セット(トナー25ml+クレンジングフォーム30g)</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>ハイドロ</t>
+        </is>
+      </c>
+      <c r="F657" t="n">
+        <v>4450</v>
+      </c>
+      <c r="G657" t="n">
+        <v>0</v>
+      </c>
+      <c r="H657" t="b">
+        <v>0</v>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J657" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205779441</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J639"/>
+  <autoFilter ref="A1:J657"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 99, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$657</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$666</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J657"/>
+  <dimension ref="A1:J666"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27392,8 +27392,377 @@
         </is>
       </c>
     </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>1195242230</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>k10shop</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>イリユン セラミドアトローション 無香料 508ml 1個</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>イリユン</t>
+        </is>
+      </c>
+      <c r="F658" t="n">
+        <v>2655</v>
+      </c>
+      <c r="G658" t="n">
+        <v>0</v>
+      </c>
+      <c r="H658" t="b">
+        <v>0</v>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J658" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195242230</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>1208323570</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>k10shop</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>SKIN1004 マダガスカルセンテラ ヒアルーシカ ウォーターフィットサンセラム 日焼け止め SPF50+ PA++++ 100ml 1個</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>ティーゼン</t>
+        </is>
+      </c>
+      <c r="F659" t="n">
+        <v>3076</v>
+      </c>
+      <c r="G659" t="n">
+        <v>0</v>
+      </c>
+      <c r="H659" t="b">
+        <v>0</v>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J659" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208323570</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>1123888012</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>unopick</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>リードルショット1000 エッセンス 15ml</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F660" t="n">
+        <v>5700</v>
+      </c>
+      <c r="G660" t="n">
+        <v>1</v>
+      </c>
+      <c r="H660" t="b">
+        <v>0</v>
+      </c>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J660" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123888012</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>1123548274</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>unopick</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>ナイアシンアミド 10 TXA 4 ダークスポット コレクティング セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F661" t="n">
+        <v>4940</v>
+      </c>
+      <c r="G661" t="n">
+        <v>0</v>
+      </c>
+      <c r="H661" t="b">
+        <v>0</v>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J661" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123548274</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>1206710414</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>k-wonderland</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>超高含有ヒアルロニックインテンストナー 100時間保湿持続力300g</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F662" t="n">
+        <v>3148</v>
+      </c>
+      <c r="G662" t="n">
+        <v>0</v>
+      </c>
+      <c r="H662" t="b">
+        <v>0</v>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206710414</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>1209385392</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>k-wonderland</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>アドール パフューム ヘアオイル 80ml 5種類から選べる</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>アドル</t>
+        </is>
+      </c>
+      <c r="F663" t="n">
+        <v>3456</v>
+      </c>
+      <c r="G663" t="n">
+        <v>1</v>
+      </c>
+      <c r="H663" t="b">
+        <v>0</v>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J663" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209385392</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>1168069878</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>morningmood</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>白樺 水分トナー 300ml</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F664" t="n">
+        <v>2345</v>
+      </c>
+      <c r="G664" t="n">
+        <v>1</v>
+      </c>
+      <c r="H664" t="b">
+        <v>0</v>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J664" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168069878</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>1210851756</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>kglowshop</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>「当日発送」 リアルカロテンIPMPブレミッシュセラムパックパッド, 80枚</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>エイプリルスキン</t>
+        </is>
+      </c>
+      <c r="F665" t="n">
+        <v>2460</v>
+      </c>
+      <c r="G665" t="n">
+        <v>1</v>
+      </c>
+      <c r="H665" t="b">
+        <v>0</v>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J665" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210851756</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>1210850141</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>smuse</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>リアルカロテンIPMPブレミッシュセラムパックパッド, 80枚</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>エイプリルスキン</t>
+        </is>
+      </c>
+      <c r="F666" t="n">
+        <v>2260</v>
+      </c>
+      <c r="G666" t="n">
+        <v>0</v>
+      </c>
+      <c r="H666" t="b">
+        <v>0</v>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J666" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210850141</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J657"/>
+  <autoFilter ref="A1:J666"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 102, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$666</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$672</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J666"/>
+  <dimension ref="A1:J672"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27761,8 +27761,254 @@
         </is>
       </c>
     </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>1195129454</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>K_AUTHENTIC</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>[韓國正品店]NEW Love portion オードパルファム 香水 9種/韓国人氣</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>After blow</t>
+        </is>
+      </c>
+      <c r="F667" t="n">
+        <v>5950</v>
+      </c>
+      <c r="G667" t="n">
+        <v>0</v>
+      </c>
+      <c r="H667" t="b">
+        <v>0</v>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J667" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195129454</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>1194218772</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>glowkorea</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>ハイドロセラミック水分エッセンス日焼け止めクリーム50ml2個</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>Dr.Melaxin</t>
+        </is>
+      </c>
+      <c r="F668" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G668" t="n">
+        <v>0</v>
+      </c>
+      <c r="H668" t="b">
+        <v>0</v>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J668" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194218772</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>1193987745</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>kstar_pick</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>ミジャンセンサロン10 プロテイントリートメント ダメージヘア用250ml3個</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F669" t="n">
+        <v>4100</v>
+      </c>
+      <c r="G669" t="n">
+        <v>0</v>
+      </c>
+      <c r="H669" t="b">
+        <v>0</v>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J669" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193987745</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>1203335944</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>ボディローション ホワイトマスク520ml /韓国コスメ 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>ブーケガルニ</t>
+        </is>
+      </c>
+      <c r="F670" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G670" t="n">
+        <v>0</v>
+      </c>
+      <c r="H670" t="b">
+        <v>0</v>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J670" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203335944</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>1196699361</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>蓮花PDRNヒアルロン光彩セラム 30ml 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>ハンスキン</t>
+        </is>
+      </c>
+      <c r="F671" t="n">
+        <v>5039</v>
+      </c>
+      <c r="G671" t="n">
+        <v>0</v>
+      </c>
+      <c r="H671" t="b">
+        <v>0</v>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J671" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196699361</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>1193167209</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>パンテノール クリーム 100ml 韓国スキンケア 韓国 コスメ #水分#保湿 毛穴ケア</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F672" t="n">
+        <v>4504</v>
+      </c>
+      <c r="G672" t="n">
+        <v>1</v>
+      </c>
+      <c r="H672" t="b">
+        <v>0</v>
+      </c>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J672" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193167209</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J666"/>
+  <autoFilter ref="A1:J672"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 105, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$672</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$685</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J672"/>
+  <dimension ref="A1:J685"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28007,8 +28007,541 @@
         </is>
       </c>
     </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>1209812267</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>thebest_mall</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>SOSセラム, 50ml</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>ティルティル</t>
+        </is>
+      </c>
+      <c r="F673" t="n">
+        <v>3524</v>
+      </c>
+      <c r="G673" t="n">
+        <v>0</v>
+      </c>
+      <c r="H673" t="b">
+        <v>0</v>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J673" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209812267</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>1210345860</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>luxstargaram</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>ハートブラシ コンパクト ヘアブラシ</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>リファ</t>
+        </is>
+      </c>
+      <c r="F674" t="n">
+        <v>3579</v>
+      </c>
+      <c r="G674" t="n">
+        <v>0</v>
+      </c>
+      <c r="H674" t="b">
+        <v>0</v>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J674" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210345860</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>1196942000</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>luxstargaram</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>デーマトロジー ファーストパッケージ【ブースター130ml＋セラム45ml】</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F675" t="n">
+        <v>13449</v>
+      </c>
+      <c r="G675" t="n">
+        <v>3</v>
+      </c>
+      <c r="H675" t="b">
+        <v>0</v>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J675" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196942000</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>1183523136</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>luxstargaram</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>韓国スキンケア 洗顔パウダー 酵素洗顔 毛穴ケア フェイスウォッシュ クレンジングパウダー 80g</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F676" t="n">
+        <v>5177</v>
+      </c>
+      <c r="G676" t="n">
+        <v>1</v>
+      </c>
+      <c r="H676" t="b">
+        <v>0</v>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J676" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183523136</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>1191781202</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>A-RAUM</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>MEDIHEAL トナーパッド2.0 リフィル 70枚×2個セット 4タイプ選択可</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F677" t="n">
+        <v>1918</v>
+      </c>
+      <c r="G677" t="n">
+        <v>0</v>
+      </c>
+      <c r="H677" t="b">
+        <v>0</v>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J677" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191781202</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>1204359324</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>A-RAUM</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>【1+1 / SNS話題】ツヤ肌バブルエッセンストナー 95ml</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>curest</t>
+        </is>
+      </c>
+      <c r="F678" t="n">
+        <v>2131</v>
+      </c>
+      <c r="G678" t="n">
+        <v>0</v>
+      </c>
+      <c r="H678" t="b">
+        <v>0</v>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J678" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204359324</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>1180354766</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>risingmother</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>[1+1/限定企画] スキンフード キャロット カロチン カミング ウォーターパッド 60枚 ダブル企画</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F679" t="n">
+        <v>6791</v>
+      </c>
+      <c r="G679" t="n">
+        <v>0</v>
+      </c>
+      <c r="H679" t="b">
+        <v>0</v>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J679" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180354766</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>1207273381</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>risingmother</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>PDRN ピンク コラーゲン バーム セラム 95ml 炭酸 泡 美容液 水光肌 弾力 ほうれい線 乾燥肌 エイジングケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F680" t="n">
+        <v>5049</v>
+      </c>
+      <c r="G680" t="n">
+        <v>0</v>
+      </c>
+      <c r="H680" t="b">
+        <v>0</v>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J680" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207273381</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>1194254316</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>kanikemen</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>【正規品】 サロン10 シャンプー + トリートメント セット （シカプロテインシャンプー 480ml + シカプロテイントリートメント 215ml）</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F681" t="n">
+        <v>3690</v>
+      </c>
+      <c r="G681" t="n">
+        <v>0</v>
+      </c>
+      <c r="H681" t="b">
+        <v>0</v>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J681" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194254316</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>1207580983</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>kanikemen</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>【正規品】 1+1 計2個 グルタチオンセブンダークスポットセラム 30ml 2個</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F682" t="n">
+        <v>4290</v>
+      </c>
+      <c r="G682" t="n">
+        <v>0</v>
+      </c>
+      <c r="H682" t="b">
+        <v>0</v>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J682" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207580983</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>1093761271</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>primeland567</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>インテンシブロングラスティングサンスクリーンEX 60ml /SPF50+PA++++</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F683" t="n">
+        <v>1575</v>
+      </c>
+      <c r="G683" t="n">
+        <v>0</v>
+      </c>
+      <c r="H683" t="b">
+        <v>0</v>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J683" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093761271</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>1177950809</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>primeland567</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>ブドウ糖ハイドロエッセンストナー, 500ml</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>パティオン</t>
+        </is>
+      </c>
+      <c r="F684" t="n">
+        <v>3105</v>
+      </c>
+      <c r="G684" t="n">
+        <v>0</v>
+      </c>
+      <c r="H684" t="b">
+        <v>0</v>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J684" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177950809</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>1172804214</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>primeland567</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>海ぶどう レチノール 毛穴弾力クリーム 50g</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>Mommy Care</t>
+        </is>
+      </c>
+      <c r="F685" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G685" t="n">
+        <v>1</v>
+      </c>
+      <c r="H685" t="b">
+        <v>0</v>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J685" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172804214</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J672"/>
+  <autoFilter ref="A1:J685"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 108, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$685</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$697</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J685"/>
+  <dimension ref="A1:J697"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28540,8 +28540,500 @@
         </is>
       </c>
     </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>1162838579</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>tmashop</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>[単独企画]清楚ビタCジョブティケアパッド70枚（10枚贈呈）</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>グーダル</t>
+        </is>
+      </c>
+      <c r="F686" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G686" t="n">
+        <v>0</v>
+      </c>
+      <c r="H686" t="b">
+        <v>0</v>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J686" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162838579</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>1213378280</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>BB_KO</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>ザ・ビタA レチナールショット タイトニングブースター 15ml/더 비타 A 레티날 샷 타이트닝 부스터 15ml</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F687" t="n">
+        <v>2386</v>
+      </c>
+      <c r="G687" t="n">
+        <v>0</v>
+      </c>
+      <c r="H687" t="b">
+        <v>0</v>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J687" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213378280</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>1167189215</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>BB_KO</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>ドクダミヒアルロンスージング アンプル 50ml/ 어성초 히알루론 수딩 앰플 50ml</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>グーダル</t>
+        </is>
+      </c>
+      <c r="F688" t="n">
+        <v>2212</v>
+      </c>
+      <c r="G688" t="n">
+        <v>0</v>
+      </c>
+      <c r="H688" t="b">
+        <v>0</v>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J688" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167189215</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>1083286884</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>BB_KO</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>[ エンジェルスリキッド ] グルタチオンプラス ナイアシンアミド 700vクリーム 50ml/나이아신아마이드 700v 크림</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>Angel's Liquid</t>
+        </is>
+      </c>
+      <c r="F689" t="n">
+        <v>3085</v>
+      </c>
+      <c r="G689" t="n">
+        <v>3</v>
+      </c>
+      <c r="H689" t="b">
+        <v>0</v>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J689" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1083286884</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>1180574367</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>fromAnswer</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>[10Sマイクロバブルパック 4種] エア** バブルCDS マスク パック 80ml, 4種の中から選択 (ハリ/ブライトニング/鎮静/水分) 150 回分</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>Gear By Gash</t>
+        </is>
+      </c>
+      <c r="F690" t="n">
+        <v>4014</v>
+      </c>
+      <c r="G690" t="n">
+        <v>0</v>
+      </c>
+      <c r="H690" t="b">
+        <v>0</v>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J690" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180574367</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>1212561469</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>kselects</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>ディープクリーン クーリングシャンプー 500ml 2本</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F691" t="n">
+        <v>5240</v>
+      </c>
+      <c r="G691" t="n">
+        <v>0</v>
+      </c>
+      <c r="H691" t="b">
+        <v>0</v>
+      </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J691" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212561469</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>1209152772</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>kselects</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>ミステリーチョコマシュマロ 40g 6個セット 韓国お菓子 チョコマシュマロ 個包装</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>Pongsindang</t>
+        </is>
+      </c>
+      <c r="F692" t="n">
+        <v>6500</v>
+      </c>
+      <c r="G692" t="n">
+        <v>0</v>
+      </c>
+      <c r="H692" t="b">
+        <v>0</v>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J692" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209152772</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>1142237251</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>otonari</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>BTSジョングクPerfume 50ml / フォルメント コットンハグ BTS ジョングク</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>FORMENT</t>
+        </is>
+      </c>
+      <c r="F693" t="n">
+        <v>4700</v>
+      </c>
+      <c r="G693" t="n">
+        <v>1</v>
+      </c>
+      <c r="H693" t="b">
+        <v>0</v>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J693" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142237251</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>1159827458</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>otonari</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>クリーンイットゼロ ピンク 水分 トナー パッド</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>バニラコ</t>
+        </is>
+      </c>
+      <c r="F694" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G694" t="n">
+        <v>0</v>
+      </c>
+      <c r="H694" t="b">
+        <v>0</v>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J694" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159827458</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>1089140326</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>otonari</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>セラミド アト集中クリーム 無香, 500ml 1個</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>イリユン</t>
+        </is>
+      </c>
+      <c r="F695" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G695" t="n">
+        <v>4</v>
+      </c>
+      <c r="H695" t="b">
+        <v>0</v>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J695" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1089140326</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>1080079065</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>otonari</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>デイリー マスクパック 30枚</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F696" t="n">
+        <v>3550</v>
+      </c>
+      <c r="G696" t="n">
+        <v>1</v>
+      </c>
+      <c r="H696" t="b">
+        <v>0</v>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J696" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1080079065</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>1157090150</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>metime</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>[1位フケかゆみシャンプー] コルツプート アンチ - ダンドラフ シャンプー 200ml デュオ 企画</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>ラウシュ</t>
+        </is>
+      </c>
+      <c r="F697" t="n">
+        <v>5516</v>
+      </c>
+      <c r="G697" t="n">
+        <v>0</v>
+      </c>
+      <c r="H697" t="b">
+        <v>0</v>
+      </c>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J697" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157090150</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J685"/>
+  <autoFilter ref="A1:J697"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 111, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$697</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$706</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J697"/>
+  <dimension ref="A1:J706"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29032,8 +29032,377 @@
         </is>
       </c>
     </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>1200859567</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>ALLROUNDERBEAUTY</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>ティーツリーシカ ディープクレンジングオイル 200ml</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F698" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G698" t="n">
+        <v>0</v>
+      </c>
+      <c r="H698" t="b">
+        <v>0</v>
+      </c>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J698" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200859567</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>1213547055</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>jj_star</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>トリプルシールド ハイドロロック サンセラム SPF50+ PA++++ 50ml</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>Forencos</t>
+        </is>
+      </c>
+      <c r="F699" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G699" t="n">
+        <v>0</v>
+      </c>
+      <c r="H699" t="b">
+        <v>0</v>
+      </c>
+      <c r="I699" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J699" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213547055</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>1212836013</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>jj_star</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>スキン パーフェクティング BHA リキッド エクスフォリエント 118ml + 30ml / 角質ケア 毛穴ケア ピーリング 低刺激 スキンケア</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>ポーラチョイス</t>
+        </is>
+      </c>
+      <c r="F700" t="n">
+        <v>4490</v>
+      </c>
+      <c r="G700" t="n">
+        <v>0</v>
+      </c>
+      <c r="H700" t="b">
+        <v>0</v>
+      </c>
+      <c r="I700" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J700" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212836013</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>1211205774</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>jj_star</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>マルチペプチドトナー 50ml x 5個 / 肌保湿 / 保湿充填</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>ルネセル</t>
+        </is>
+      </c>
+      <c r="F701" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G701" t="n">
+        <v>0</v>
+      </c>
+      <c r="H701" t="b">
+        <v>0</v>
+      </c>
+      <c r="I701" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J701" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211205774</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>1171947071</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>CallaBoutique</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>【正規品】 デイリートナーパッド 80枚</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>NEEDLY</t>
+        </is>
+      </c>
+      <c r="F702" t="n">
+        <v>1990</v>
+      </c>
+      <c r="G702" t="n">
+        <v>0</v>
+      </c>
+      <c r="H702" t="b">
+        <v>0</v>
+      </c>
+      <c r="I702" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J702" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171947071</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>1171946936</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>CallaBoutique</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>【正規品】 センテラクイックカーミングパッド 70枚</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F703" t="n">
+        <v>1590</v>
+      </c>
+      <c r="G703" t="n">
+        <v>3</v>
+      </c>
+      <c r="H703" t="b">
+        <v>0</v>
+      </c>
+      <c r="I703" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J703" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171946936</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>1197892266</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>CallaBoutique</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>【正規品】 グロウクリーミーボディスクラブ ヌバニラ 300ml</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F704" t="n">
+        <v>3090</v>
+      </c>
+      <c r="G704" t="n">
+        <v>0</v>
+      </c>
+      <c r="H704" t="b">
+        <v>0</v>
+      </c>
+      <c r="I704" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J704" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197892266</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>1169812368</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>coneco</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>[NEW]ラウンドアラウンド センテッド ヘア&amp;amp;ボディ ミスト 100ml</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>ROUND A ROUND</t>
+        </is>
+      </c>
+      <c r="F705" t="n">
+        <v>1618</v>
+      </c>
+      <c r="G705" t="n">
+        <v>0</v>
+      </c>
+      <c r="H705" t="b">
+        <v>0</v>
+      </c>
+      <c r="I705" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J705" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169812368</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>1155304298</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>coneco</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>ZARA 香水 HIBISCUS 90ML オードパフューム [EDP]</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>ザラ</t>
+        </is>
+      </c>
+      <c r="F706" t="n">
+        <v>4669</v>
+      </c>
+      <c r="G706" t="n">
+        <v>0</v>
+      </c>
+      <c r="H706" t="b">
+        <v>0</v>
+      </c>
+      <c r="I706" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J706" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1155304298</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J697"/>
+  <autoFilter ref="A1:J706"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 114, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$706</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$714</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J706"/>
+  <dimension ref="A1:J714"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29401,8 +29401,336 @@
         </is>
       </c>
     </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>1178796694</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>[最新リニューアル] セルメディックス エムジーエフ リターンクリーム 70ml</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>cellmedics</t>
+        </is>
+      </c>
+      <c r="F707" t="n">
+        <v>8860</v>
+      </c>
+      <c r="G707" t="n">
+        <v>1</v>
+      </c>
+      <c r="H707" t="b">
+        <v>0</v>
+      </c>
+      <c r="I707" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J707" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178796694</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>1180095461</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>イーロン アンプル 50ml センシエンド</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F708" t="n">
+        <v>15970</v>
+      </c>
+      <c r="G708" t="n">
+        <v>0</v>
+      </c>
+      <c r="H708" t="b">
+        <v>0</v>
+      </c>
+      <c r="I708" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J708" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180095461</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>1180095290</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>イーロン ダンギ クレンジングジェル 200ml + 贈呈:マスクパック1枚</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F709" t="n">
+        <v>6550</v>
+      </c>
+      <c r="G709" t="n">
+        <v>0</v>
+      </c>
+      <c r="H709" t="b">
+        <v>0</v>
+      </c>
+      <c r="I709" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J709" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180095290</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>1180095287</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>ザ·イーロン イーロン メゾプロ プラスキット 1箱 2gx2個入 + スージング マスクパック 2枚</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F710" t="n">
+        <v>11880</v>
+      </c>
+      <c r="G710" t="n">
+        <v>0</v>
+      </c>
+      <c r="H710" t="b">
+        <v>0</v>
+      </c>
+      <c r="I710" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J710" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180095287</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>1180092834</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>サンテ 日焼け止め アズレン スーダー サンエッセンス 75ml 2個 デュオセット</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>SANTE</t>
+        </is>
+      </c>
+      <c r="F711" t="n">
+        <v>15970</v>
+      </c>
+      <c r="G711" t="n">
+        <v>1</v>
+      </c>
+      <c r="H711" t="b">
+        <v>0</v>
+      </c>
+      <c r="I711" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J711" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180092834</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>1191171558</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>sonny</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>[正規品] SKIN1004 プロバイオシカグロウサンアンプル, 50ml / SPF50+ PA++++ / 保湿 / スキンケア / 紫外線 / 乳液 / 白浮しない日焼け止め / オマケも /</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F712" t="n">
+        <v>2640</v>
+      </c>
+      <c r="G712" t="n">
+        <v>4</v>
+      </c>
+      <c r="H712" t="b">
+        <v>0</v>
+      </c>
+      <c r="I712" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J712" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191171558</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>1178760167</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>toseo</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>オードパルファムスノーサイ 30ML Snow Sai</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>LIBER</t>
+        </is>
+      </c>
+      <c r="F713" t="n">
+        <v>7430</v>
+      </c>
+      <c r="G713" t="n">
+        <v>0</v>
+      </c>
+      <c r="H713" t="b">
+        <v>0</v>
+      </c>
+      <c r="I713" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J713" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178760167</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>1168152797</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>beautyofkorea</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>米麹酵素サウナ コマジュフォーム 170ml 1個</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F714" t="n">
+        <v>1862</v>
+      </c>
+      <c r="G714" t="n">
+        <v>0</v>
+      </c>
+      <c r="H714" t="b">
+        <v>0</v>
+      </c>
+      <c r="I714" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J714" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168152797</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J706"/>
+  <autoFilter ref="A1:J714"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 117, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$714</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$721</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J714"/>
+  <dimension ref="A1:J721"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29729,8 +29729,295 @@
         </is>
       </c>
     </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>1168778005</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>BnD_official</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>コンプリートセット 5点セット ビーエヌディ アンダーアームクリーム100ｇ+ＡＨＡスクラブ200ｇ＋ネッククリーム50ｇ+ヒップクリーム100ｇ+ブルーミングヘアオイル</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>BnD</t>
+        </is>
+      </c>
+      <c r="F715" t="n">
+        <v>15437</v>
+      </c>
+      <c r="G715" t="n">
+        <v>3</v>
+      </c>
+      <c r="H715" t="b">
+        <v>0</v>
+      </c>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J715" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168778005</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>1211601601</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>JUNO_korea</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>【アヌ ア美容液】アゼライン酸10％マイルドスージングセラム 30ml(混合肌 敏感肌向け 韓国スキンケア)</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F716" t="n">
+        <v>3180</v>
+      </c>
+      <c r="G716" t="n">
+        <v>0</v>
+      </c>
+      <c r="H716" t="b">
+        <v>0</v>
+      </c>
+      <c r="I716" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J716" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211601601</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>1209266440</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>JUNO_korea</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>【PDRN配合/リピートアイテム】ペプタシカ セラムパッド ダブルセット（60枚＋60枚）</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>トーン28</t>
+        </is>
+      </c>
+      <c r="F717" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G717" t="n">
+        <v>0</v>
+      </c>
+      <c r="H717" t="b">
+        <v>0</v>
+      </c>
+      <c r="I717" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J717" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209266440</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>1212027043</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>SEOUL_ON</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>【重ね塗りしやすい首ケアスティック】プレミアムネックスティック, 20g　首のシワ改善クリーム／べたつかないネックケアライン／首元のハリケア／首のしわ ／首クリーム／首トーンアップ／首用クリーム／</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F718" t="n">
+        <v>3674</v>
+      </c>
+      <c r="G718" t="n">
+        <v>0</v>
+      </c>
+      <c r="H718" t="b">
+        <v>0</v>
+      </c>
+      <c r="I718" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J718" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212027043</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>1203787114</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>SEOUL_ON</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>【保湿クリーム】 クリームスカムトゥルー スクワランバリアリペアクリーム 50ml ツヤ肌 乾燥肌 水光肌 水分 乾燥 高保湿 うるおい もちもち ベタつかない 水分チャージ 肌荒れ</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>De:maf</t>
+        </is>
+      </c>
+      <c r="F719" t="n">
+        <v>4857</v>
+      </c>
+      <c r="G719" t="n">
+        <v>0</v>
+      </c>
+      <c r="H719" t="b">
+        <v>0</v>
+      </c>
+      <c r="I719" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J719" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203787114</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>1204259978</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>SEOUL_ON</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>【インナードライクリーム】ブラックライス5モイスチャライジングクリーム 50ml 保湿 乾燥肌 水光肌 水分 乾燥 高保湿 うるおい もちもち ベタつかない 水分チャージ</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>haruharu wonder</t>
+        </is>
+      </c>
+      <c r="F720" t="n">
+        <v>4396</v>
+      </c>
+      <c r="G720" t="n">
+        <v>0</v>
+      </c>
+      <c r="H720" t="b">
+        <v>0</v>
+      </c>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J720" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204259978</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>1208516387</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>SEOUL_ON</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>【夏向けサラサラ日焼け止め】3番 ノーファンデ陶器肌トーンアップUVクリームEX, 50ml／ベタつかない／さっぱり／日差し対策／紫外線対策／ベースメイク／化粧下地／</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F721" t="n">
+        <v>2609</v>
+      </c>
+      <c r="G721" t="n">
+        <v>0</v>
+      </c>
+      <c r="H721" t="b">
+        <v>0</v>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J721" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208516387</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J714"/>
+  <autoFilter ref="A1:J721"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 120, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$721</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$725</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J721"/>
+  <dimension ref="A1:J725"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30016,8 +30016,172 @@
         </is>
       </c>
     </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>1199604337</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>lilyhouse_jp</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>ヨモギクーリングカミングジェル100ml/アロエベラ/熱感鎮静/ナイトパック/鎮静パック/敏感肌/トラブル/熱感鎮静</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>グレイメリン</t>
+        </is>
+      </c>
+      <c r="F722" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G722" t="n">
+        <v>2</v>
+      </c>
+      <c r="H722" t="b">
+        <v>0</v>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J722" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199604337</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>1202850935</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>lilyhouse_jp</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>[単品]センテラクイックカーミングパッド70枚入り/パック/パッド/トナーパッド/化粧水/トナー/拭き取りシート/鎮静/水分/保湿</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F723" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G723" t="n">
+        <v>0</v>
+      </c>
+      <c r="H723" t="b">
+        <v>0</v>
+      </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J723" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202850935</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>1202849422</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>lilyhouse_jp</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>[1+1]センテラアンプルマダガスカル産CICA 美容液55ml/弱酸性pH/敏感肌/天然由来成分/ツボクサエキス/敏感肌鎮静効果</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F724" t="n">
+        <v>3980</v>
+      </c>
+      <c r="G724" t="n">
+        <v>0</v>
+      </c>
+      <c r="H724" t="b">
+        <v>0</v>
+      </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J724" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202849422</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>1202836073</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>lilyhouse_jp</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>[単品][集中ケア用]リードルショットヘアエッセンス300dL/スカルプエッセンス/スカルプリードルショット/ヘアアンプル</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F725" t="n">
+        <v>3580</v>
+      </c>
+      <c r="G725" t="n">
+        <v>0</v>
+      </c>
+      <c r="H725" t="b">
+        <v>0</v>
+      </c>
+      <c r="I725" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J725" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202836073</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J721"/>
+  <autoFilter ref="A1:J725"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 123, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$725</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$735</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J725"/>
+  <dimension ref="A1:J735"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30180,8 +30180,418 @@
         </is>
       </c>
     </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>1149453077</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>dal24</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>プロフェッショナル頭皮シャンプーブラシ1本 韓国 頭皮 ブラシ シャンプー 櫛 マッサージ 角質 フケ におい ヘアー</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>rolencos</t>
+        </is>
+      </c>
+      <c r="F726" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G726" t="n">
+        <v>0</v>
+      </c>
+      <c r="H726" t="b">
+        <v>0</v>
+      </c>
+      <c r="I726" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J726" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149453077</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>1157097518</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>JUBJUBSTORE</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>[NEW] アイスマスク 30枚 / アイス/PDRN/アゼラリン酸/トラネキサム酸/レチノール/CICA</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F727" t="n">
+        <v>2730</v>
+      </c>
+      <c r="G727" t="n">
+        <v>0</v>
+      </c>
+      <c r="H727" t="b">
+        <v>0</v>
+      </c>
+      <c r="I727" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J727" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157097518</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>1116944837</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>dal25</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>9種の中から 選択1 / ゴールドコアマックスキッズ肝臓ケア植物性糖ケアスリム50代 韓国製品 韓国乳酸菌 乳酸菌 キッズ プロバイオティクス ミルクシスル ガルシニア ビタミンD 生乳酸菌</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>ラクトフィット</t>
+        </is>
+      </c>
+      <c r="F728" t="n">
+        <v>2580</v>
+      </c>
+      <c r="G728" t="n">
+        <v>5</v>
+      </c>
+      <c r="H728" t="b">
+        <v>0</v>
+      </c>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J728" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1116944837</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>1115638534</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>dal25</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>旅行用ヘアボディ5種+コットンポーチ1セット 韓国シャンプー 純正品 旅行キット トラベルキット トリートメント ボディウォッシュ ボディローション クレンジングフォーム 旅行 携帯用シャンプー</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>NARD</t>
+        </is>
+      </c>
+      <c r="F729" t="n">
+        <v>2690</v>
+      </c>
+      <c r="G729" t="n">
+        <v>0</v>
+      </c>
+      <c r="H729" t="b">
+        <v>0</v>
+      </c>
+      <c r="I729" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J729" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1115638534</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>1191487583</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>marumarushop</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>大豆エッセンス 50ml</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>ミクスン</t>
+        </is>
+      </c>
+      <c r="F730" t="n">
+        <v>5076</v>
+      </c>
+      <c r="G730" t="n">
+        <v>1</v>
+      </c>
+      <c r="H730" t="b">
+        <v>0</v>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J730" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191487583</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>1176819992</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>marumarushop</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>フルイド フェルメント トーンアップパッド 250ml（50枚入り）</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>ネオゼン</t>
+        </is>
+      </c>
+      <c r="F731" t="n">
+        <v>5057</v>
+      </c>
+      <c r="G731" t="n">
+        <v>0</v>
+      </c>
+      <c r="H731" t="b">
+        <v>0</v>
+      </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J731" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176819992</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>1124910554</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>marumarushop</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>フレッシュマスク 10枚</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F732" t="n">
+        <v>2070</v>
+      </c>
+      <c r="G732" t="n">
+        <v>0</v>
+      </c>
+      <c r="H732" t="b">
+        <v>0</v>
+      </c>
+      <c r="I732" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J732" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1124910554</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>1168203274</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>happyclover</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>スピーディー マスカラリムーバー</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>ヒロインメイク</t>
+        </is>
+      </c>
+      <c r="F733" t="n">
+        <v>2417</v>
+      </c>
+      <c r="G733" t="n">
+        <v>4</v>
+      </c>
+      <c r="H733" t="b">
+        <v>0</v>
+      </c>
+      <c r="I733" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J733" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168203274</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>1202779298</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>ooznary</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>【New 毛穴レスケア】アイスレチノール37セラム 30ml　レチノール 美容液 ハリ キメケア 角質ケア 水光肌 毛穴引き締め たるみ毛穴 ナイアシンアミド AHA BHA</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>オーズナリー</t>
+        </is>
+      </c>
+      <c r="F734" t="n">
+        <v>3400</v>
+      </c>
+      <c r="G734" t="n">
+        <v>0</v>
+      </c>
+      <c r="H734" t="b">
+        <v>0</v>
+      </c>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J734" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202779298</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>1191236161</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>tiam_official</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>【毛穴ケア】 ポアミニマイジング21セラム 40ml</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>ティアム</t>
+        </is>
+      </c>
+      <c r="F735" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G735" t="n">
+        <v>2</v>
+      </c>
+      <c r="H735" t="b">
+        <v>0</v>
+      </c>
+      <c r="I735" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J735" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191236161</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J725"/>
+  <autoFilter ref="A1:J735"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 1, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$358</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$374</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J358"/>
+  <dimension ref="A1:J374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15133,8 +15133,664 @@
         </is>
       </c>
     </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>1206193902</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>loreallarocheposay</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>エファクラオイル＆ポア コレクト ローション / 150mL　【ダーマコスメ】</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>ラロッシュポゼ</t>
+        </is>
+      </c>
+      <c r="F359" t="n">
+        <v>4290</v>
+      </c>
+      <c r="G359" t="n">
+        <v>10</v>
+      </c>
+      <c r="H359" t="b">
+        <v>0</v>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206193902</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>1178044150</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>chronus</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>2袋セット ボディーソープ 詰め替え 400ml メンズ いい香り 体臭 加齢臭 マリンムスク 男性用 リフィル</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>リデン</t>
+        </is>
+      </c>
+      <c r="F360" t="n">
+        <v>1691</v>
+      </c>
+      <c r="G360" t="n">
+        <v>2</v>
+      </c>
+      <c r="H360" t="b">
+        <v>0</v>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J360" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178044150</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>1097778656</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>aihada</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>[大容量]パフュームシャンプー+リンスセット(Sweet&amp;amp;Flowery)(Fresh&amp;amp;Lush)香り高い毛髪ツヤケア</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F361" t="n">
+        <v>3050</v>
+      </c>
+      <c r="G361" t="n">
+        <v>9</v>
+      </c>
+      <c r="H361" t="b">
+        <v>0</v>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J361" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097778656</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>1212016574</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>laundryou</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>【公式】ランドリユー ソフトボディ レッドグローブクリーン 5枚入り</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>ランドリーユー</t>
+        </is>
+      </c>
+      <c r="F362" t="n">
+        <v>2060</v>
+      </c>
+      <c r="G362" t="n">
+        <v>18</v>
+      </c>
+      <c r="H362" t="b">
+        <v>0</v>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J362" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212016574</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>1168785073</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>laundryou</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>【公式】 個体ゼリーグロウPDRNミスト100g / グロウゼリーフェイスミストPDRN 100g　美容液/韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>ランドリーユー</t>
+        </is>
+      </c>
+      <c r="F363" t="n">
+        <v>3626</v>
+      </c>
+      <c r="G363" t="n">
+        <v>15</v>
+      </c>
+      <c r="H363" t="b">
+        <v>0</v>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168785073</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>1067860444</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>laundryou</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>【公式】クリーンフェイスモイストトナーパッドクイック60枚　トナーパッド/拭き取りパッド/保湿/韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>ランドリーユー</t>
+        </is>
+      </c>
+      <c r="F364" t="n">
+        <v>3222</v>
+      </c>
+      <c r="G364" t="n">
+        <v>14</v>
+      </c>
+      <c r="H364" t="b">
+        <v>0</v>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1067860444</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>1211272013</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>vicrea</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>【公式】 アンドハニー &amp;amp;honey×VT 限定ヘアオイル</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>アンドハニー</t>
+        </is>
+      </c>
+      <c r="F365" t="n">
+        <v>1078</v>
+      </c>
+      <c r="G365" t="n">
+        <v>9</v>
+      </c>
+      <c r="H365" t="b">
+        <v>0</v>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211272013</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>1200737932</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>vicrea</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>【公式】Re:KERATIN リ ケラチン リバーシ リペア シャンプー＆ヘアトリートメント</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Re:KERATIN</t>
+        </is>
+      </c>
+      <c r="F366" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G366" t="n">
+        <v>0</v>
+      </c>
+      <c r="H366" t="b">
+        <v>0</v>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200737932</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>1182232360</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>vicrea</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>2026福袋【公式】アンドハニー メルティ 4点セット シャンプー トリートメント ヘアオイル マトメイクスティック</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>アンドハニー</t>
+        </is>
+      </c>
+      <c r="F367" t="n">
+        <v>5698</v>
+      </c>
+      <c r="G367" t="n">
+        <v>0</v>
+      </c>
+      <c r="H367" t="b">
+        <v>0</v>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182232360</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>1180176379</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>cosmegt</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>フェルナンダ サスティナブル フレグランス ボディスプラッシュ ヨーグルトスムージー 95ml</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>フェルナンダ</t>
+        </is>
+      </c>
+      <c r="F368" t="n">
+        <v>1880</v>
+      </c>
+      <c r="G368" t="n">
+        <v>0</v>
+      </c>
+      <c r="H368" t="b">
+        <v>0</v>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180176379</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>1179921125</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>cosmegt</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>2個セット アトピアD 美白保湿フォーム オールインワン美白保湿ケア 詰替 100g</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>アトピアD</t>
+        </is>
+      </c>
+      <c r="F369" t="n">
+        <v>3880</v>
+      </c>
+      <c r="G369" t="n">
+        <v>0</v>
+      </c>
+      <c r="H369" t="b">
+        <v>0</v>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179921125</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>1211967820</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>cosmegt</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>数量限定！ お試し価格 JOOMO ジョーモ 除毛クリーム 100g</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>RITA COSME</t>
+        </is>
+      </c>
+      <c r="F370" t="n">
+        <v>1720</v>
+      </c>
+      <c r="G370" t="n">
+        <v>0</v>
+      </c>
+      <c r="H370" t="b">
+        <v>0</v>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>120000019</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211967820</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>1209499067</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>cosmegt</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>アンドハニー ピクシー モイストシルキー シャンプー&amp;amp;トリートメント つめかえセット</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>アンドハニー</t>
+        </is>
+      </c>
+      <c r="F371" t="n">
+        <v>2220</v>
+      </c>
+      <c r="G371" t="n">
+        <v>1</v>
+      </c>
+      <c r="H371" t="b">
+        <v>0</v>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209499067</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>1203997154</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>SPMARKET</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>【1+1セット】 韓国ダイソーデイリーコンマ モスト オードパルファム 30ml 全6種 2本セット 香水</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>daily comma</t>
+        </is>
+      </c>
+      <c r="F372" t="n">
+        <v>1643</v>
+      </c>
+      <c r="G372" t="n">
+        <v>0</v>
+      </c>
+      <c r="H372" t="b">
+        <v>0</v>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J372" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203997154</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>1132023348</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>TigerStore</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>1+1 オム ウォーター Whitening スキンローション オールインワンエッセンス 211ml 2個</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>PAUL MEDISON</t>
+        </is>
+      </c>
+      <c r="F373" t="n">
+        <v>4590</v>
+      </c>
+      <c r="G373" t="n">
+        <v>0</v>
+      </c>
+      <c r="H373" t="b">
+        <v>0</v>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1132023348</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>1179455683</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>menthology</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>【2SET】 スーパークールカーミングパッド(60枚入)x2/ フェイスパック/ 鎮静効果/ トナーパッド/ 鎮静パッド/ クールリング/ 毛穴ケア/ 保湿/ 速効性 / 敏感肌 / 水分補給</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>MENTHOLOGY</t>
+        </is>
+      </c>
+      <c r="F374" t="n">
+        <v>4200</v>
+      </c>
+      <c r="G374" t="n">
+        <v>3</v>
+      </c>
+      <c r="H374" t="b">
+        <v>0</v>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179455683</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J358"/>
+  <autoFilter ref="A1:J374"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 2, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$392</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$400</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J392"/>
+  <dimension ref="A1:J400"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16527,8 +16527,336 @@
         </is>
       </c>
     </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>1190165940</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>re-nk</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>【re:nk公式】ハイパー ヒアルプランピングトナー200ml</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>リエンケイ</t>
+        </is>
+      </c>
+      <c r="F393" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G393" t="n">
+        <v>1</v>
+      </c>
+      <c r="H393" t="b">
+        <v>0</v>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190165940</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>1171777671</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>anotherface_official</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>【究極の輝き】ナイアシン＋グルタチオン 1,100ppm アナザーフェイス 透明感爆発 ナイアチオン 光 クレンジングウォーター 500ml</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>ANOTHER FACE</t>
+        </is>
+      </c>
+      <c r="F394" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G394" t="n">
+        <v>10</v>
+      </c>
+      <c r="H394" t="b">
+        <v>0</v>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171777671</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>1149398781</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>houseofhur</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>【公式】 トロピカル デュー サンクリーム 日焼け止め 50ml / トーンアップ日焼け止め / 乾燥肌 / 高保湿 / うるおい感 / UVケーア /</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>HOUSE OF Hur</t>
+        </is>
+      </c>
+      <c r="F395" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G395" t="n">
+        <v>10</v>
+      </c>
+      <c r="H395" t="b">
+        <v>0</v>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149398781</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>1142906709</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>houseofhur</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>【公式】 ミッドナイト スージング クレンジングバーム 50ml / クレンジング / メイク落とし / オイルバーム / ダブル洗顔不要 / しっとり / 乾燥肌 / 敏感肌 /</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>HOUSE OF Hur</t>
+        </is>
+      </c>
+      <c r="F396" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G396" t="n">
+        <v>16</v>
+      </c>
+      <c r="H396" t="b">
+        <v>0</v>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142906709</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>922017363</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>mellifeshop</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>ブライトヴェールセラム ナイアシンアミド配合 1本40g 30日分 炭酸美容液</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>MELLIFE</t>
+        </is>
+      </c>
+      <c r="F397" t="n">
+        <v>5740</v>
+      </c>
+      <c r="G397" t="n">
+        <v>12</v>
+      </c>
+      <c r="H397" t="b">
+        <v>0</v>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=922017363</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>1147204343</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>mellifeshop</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>カームグリップツイン 洗顔　美容液セット アゼライン酸 グルタチオン ナイアシンアミド グリチルリチン酸</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>e'ltofia</t>
+        </is>
+      </c>
+      <c r="F398" t="n">
+        <v>8680</v>
+      </c>
+      <c r="G398" t="n">
+        <v>9</v>
+      </c>
+      <c r="H398" t="b">
+        <v>0</v>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1147204343</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>1147199196</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>mellifeshop</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>NA グリップセラム 医薬部外品美容液　ナイアシンアミド　グリチルリチン酸ジカリウム</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>e'ltofia</t>
+        </is>
+      </c>
+      <c r="F399" t="n">
+        <v>5740</v>
+      </c>
+      <c r="G399" t="n">
+        <v>16</v>
+      </c>
+      <c r="H399" t="b">
+        <v>0</v>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1147199196</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>1171722559</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>mellifeshop</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>RTインクレンジング クレンジングジェル 角栓 毛穴 サリチル酸 レチノール誘導体</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>e'ltofia</t>
+        </is>
+      </c>
+      <c r="F400" t="n">
+        <v>4100</v>
+      </c>
+      <c r="G400" t="n">
+        <v>0</v>
+      </c>
+      <c r="H400" t="b">
+        <v>0</v>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171722559</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J392"/>
+  <autoFilter ref="A1:J400"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 5, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$415</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$417</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J415"/>
+  <dimension ref="A1:J417"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17470,8 +17470,90 @@
         </is>
       </c>
     </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>1079637346</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>moicos</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>新型! 洗い流さない!高濃縮バクジュンLＰPノーウォッシュトリートメントパック200ml ヘアエッセンス,ヘアオイル 髪ダーメジ完璧ケア!カサカサヘア修復 アウトバス</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>PARKJUN BEAUTY LAB</t>
+        </is>
+      </c>
+      <c r="F416" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G416" t="n">
+        <v>12</v>
+      </c>
+      <c r="H416" t="b">
+        <v>0</v>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1079637346</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>1017343006</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>moicos</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>損傷毛専用! サロンクリニックUSB電気ヘアヒーティングキャップ 時短 ヘアケア加温器 トリートメント浸透 スチーマー サロン専売品 枝毛 切れ毛 染毛 脱色毛 損傷毛 ダメージヘア 集中ケア</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>PARKJUN BEAUTY LAB</t>
+        </is>
+      </c>
+      <c r="F417" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G417" t="n">
+        <v>3</v>
+      </c>
+      <c r="H417" t="b">
+        <v>0</v>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1017343006</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J415"/>
+  <autoFilter ref="A1:J417"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 8, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$429</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$432</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J429"/>
+  <dimension ref="A1:J432"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18044,8 +18044,131 @@
         </is>
       </c>
     </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>1025130982</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>tafomi_official</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>カミングタムシートマスク, 10枚</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>TAFOMI</t>
+        </is>
+      </c>
+      <c r="F430" t="n">
+        <v>2050</v>
+      </c>
+      <c r="G430" t="n">
+        <v>4</v>
+      </c>
+      <c r="H430" t="b">
+        <v>0</v>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1025130982</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>1025125639</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>tafomi_official</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>ビタタムシートマスク, 10枚</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>TAFOMI</t>
+        </is>
+      </c>
+      <c r="F431" t="n">
+        <v>2050</v>
+      </c>
+      <c r="G431" t="n">
+        <v>7</v>
+      </c>
+      <c r="H431" t="b">
+        <v>0</v>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1025125639</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>1078074138</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>tafomi_official</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>シカタムシートマスク, 20枚</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>TAFOMI</t>
+        </is>
+      </c>
+      <c r="F432" t="n">
+        <v>3550</v>
+      </c>
+      <c r="G432" t="n">
+        <v>1</v>
+      </c>
+      <c r="H432" t="b">
+        <v>0</v>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1078074138</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J429"/>
+  <autoFilter ref="A1:J432"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 10, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$432</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$433</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J432"/>
+  <dimension ref="A1:J433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18167,8 +18167,49 @@
         </is>
       </c>
     </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>1185613175</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Rani_House</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>レモン ハニー ブライトニング ウォッシュオフ 毛穴パック_ 100g_レモン蜂蜜パック_韓国人気パック</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>LABIORA</t>
+        </is>
+      </c>
+      <c r="F433" t="n">
+        <v>2920</v>
+      </c>
+      <c r="G433" t="n">
+        <v>0</v>
+      </c>
+      <c r="H433" t="b">
+        <v>0</v>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185613175</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J432"/>
+  <autoFilter ref="A1:J433"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 11, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$433</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$435</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J433"/>
+  <dimension ref="A1:J435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18208,8 +18208,90 @@
         </is>
       </c>
     </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>1195134429</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>justasiam</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>【公式 / Qoo10限定】IAM ヘアミルク企画セット/ヘアミルク/ ヘアケア/韓国ヘアケア/ ダメージケア/ 洗い流さないトリートメント/ ヘアエッセンス/特典付き</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>JUST AS I AM</t>
+        </is>
+      </c>
+      <c r="F434" t="n">
+        <v>2553</v>
+      </c>
+      <c r="G434" t="n">
+        <v>11</v>
+      </c>
+      <c r="H434" t="b">
+        <v>0</v>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195134429</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>1195134963</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>justasiam</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>【公式 / Qoo10限定】 IAM ヘアマスク N1 企画セット/ ヘアマスク/ヘアパック/大容量/ダメージケア/コンディショナー/トリートメント/ヘアトリートメント /ヘアケア/特典付き</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>JUST AS I AM</t>
+        </is>
+      </c>
+      <c r="F435" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G435" t="n">
+        <v>2</v>
+      </c>
+      <c r="H435" t="b">
+        <v>0</v>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195134963</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J433"/>
+  <autoFilter ref="A1:J435"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 4, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$437</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$441</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J437"/>
+  <dimension ref="A1:J441"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18372,8 +18372,172 @@
         </is>
       </c>
     </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>1154378888</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>kostyou</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>清光 マリン 真珠 ディープ モイスチャー マスク パール10個入り</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>JM solution</t>
+        </is>
+      </c>
+      <c r="F438" t="n">
+        <v>890</v>
+      </c>
+      <c r="G438" t="n">
+        <v>3</v>
+      </c>
+      <c r="H438" t="b">
+        <v>0</v>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154378888</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>1021098567</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>bimora</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>【ヘアケアセット】 トータルヘアケア メンズ シャンプー 200ml トリートメント 185ml トニック 100ml スカルプケア 日本製 ヒト幹細胞培養液配合 頭皮保湿ケア フケ かゆみ</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>BimoRa</t>
+        </is>
+      </c>
+      <c r="F439" t="n">
+        <v>12180</v>
+      </c>
+      <c r="G439" t="n">
+        <v>0</v>
+      </c>
+      <c r="H439" t="b">
+        <v>0</v>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1021098567</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>1010015951</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>bimora</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>【VC 美容液】【ビタミンC誘導体高濃度30%配合】日本製　ビタミンC美容液 スキンケア 毛穴 エイジングケア ニキビケア 肌荒れ 角質ケア 高保湿 乾燥肌 敏感肌 セラム 女性用 シミ 30ml</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>BimoRa</t>
+        </is>
+      </c>
+      <c r="F440" t="n">
+        <v>5040</v>
+      </c>
+      <c r="G440" t="n">
+        <v>9</v>
+      </c>
+      <c r="H440" t="b">
+        <v>0</v>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1010015951</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>1020889597</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>bimora</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>［公式］ベーシックヘアケアセット シャンプー:200ml トリートメント:185ml シャンプートリートメントセット シャンプー トリートメント メンズ 男性用 女性 ヘアケア 頭皮ケア 保湿 日本製</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>BimoRa</t>
+        </is>
+      </c>
+      <c r="F441" t="n">
+        <v>6090</v>
+      </c>
+      <c r="G441" t="n">
+        <v>5</v>
+      </c>
+      <c r="H441" t="b">
+        <v>0</v>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1020889597</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J437"/>
+  <autoFilter ref="A1:J441"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 3)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$450</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$451</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J450"/>
+  <dimension ref="A1:J451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18905,8 +18905,49 @@
         </is>
       </c>
     </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>1161261989</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>llongy</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>【 目元のクマ 】アイクリーム ハロキシル2% レチノール 目の下のクマ 目元 たるみ 色素沈着 くま 目元ケア アイクリーム 18g 目元美容液 青クマ 茶クマ 黒クマ レディース メンズ</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>llongy</t>
+        </is>
+      </c>
+      <c r="F451" t="n">
+        <v>4400</v>
+      </c>
+      <c r="G451" t="n">
+        <v>10</v>
+      </c>
+      <c r="H451" t="b">
+        <v>0</v>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1161261989</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J450"/>
+  <autoFilter ref="A1:J451"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 7, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$483</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$484</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J483"/>
+  <dimension ref="A1:J484"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20063,8 +20063,49 @@
         </is>
       </c>
     </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>1207275701</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>alleumjp</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>EGFx ダウンタイム オイント マスク 4枚 フェイスパック シートマスク 肌荒れケア 保湿 敏感肌 スキンケア</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>イージーデュー</t>
+        </is>
+      </c>
+      <c r="F484" t="n">
+        <v>2699</v>
+      </c>
+      <c r="G484" t="n">
+        <v>1</v>
+      </c>
+      <c r="H484" t="b">
+        <v>0</v>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207275701</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J483"/>
+  <autoFilter ref="A1:J484"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 16, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$488</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$489</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J488"/>
+  <dimension ref="A1:J489"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20268,8 +20268,49 @@
         </is>
       </c>
     </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>1161832347</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>JUHACOSMETIC</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>ナチュラルカバーファンデーション/ 極細毛ブラシ付/ スティック型/ 韓国化粧品</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>オブジェ</t>
+        </is>
+      </c>
+      <c r="F489" t="n">
+        <v>4950</v>
+      </c>
+      <c r="G489" t="n">
+        <v>0</v>
+      </c>
+      <c r="H489" t="b">
+        <v>0</v>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1161832347</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J488"/>
+  <autoFilter ref="A1:J489"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 19, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$489</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$490</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J489"/>
+  <dimension ref="A1:J490"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20309,8 +20309,49 @@
         </is>
       </c>
     </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>1186959741</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>medicareplus</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>IHADA イハダ 薬用クリアローション 美白化粧水 180mL</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>イハダ</t>
+        </is>
+      </c>
+      <c r="F490" t="n">
+        <v>1918</v>
+      </c>
+      <c r="G490" t="n">
+        <v>0</v>
+      </c>
+      <c r="H490" t="b">
+        <v>0</v>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1186959741</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J489"/>
+  <autoFilter ref="A1:J490"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 25, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$490</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$495</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J490"/>
+  <dimension ref="A1:J495"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20350,8 +20350,213 @@
         </is>
       </c>
     </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>1026840717</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>kyobi</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>セルローション　150ml　3本セット</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>アルソア</t>
+        </is>
+      </c>
+      <c r="F491" t="n">
+        <v>12690</v>
+      </c>
+      <c r="G491" t="n">
+        <v>8</v>
+      </c>
+      <c r="H491" t="b">
+        <v>0</v>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1026840717</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>1213893592</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>kyobi</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>【お試しセット】クイーンシルバー レフィル[枠練石けん] ＆ローション II</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>アルソア</t>
+        </is>
+      </c>
+      <c r="F492" t="n">
+        <v>7500</v>
+      </c>
+      <c r="G492" t="n">
+        <v>0</v>
+      </c>
+      <c r="H492" t="b">
+        <v>0</v>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213893592</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>1213893007</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>kyobi</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>【お試しセット】クイーンシルバー レフィル[枠練石けん] ＆セルローション</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>アルソア</t>
+        </is>
+      </c>
+      <c r="F493" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G493" t="n">
+        <v>0</v>
+      </c>
+      <c r="H493" t="b">
+        <v>0</v>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213893007</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>1026840719</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>kyobi</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>クレイパック 100g</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>アルソア</t>
+        </is>
+      </c>
+      <c r="F494" t="n">
+        <v>3120</v>
+      </c>
+      <c r="G494" t="n">
+        <v>3</v>
+      </c>
+      <c r="H494" t="b">
+        <v>0</v>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1026840719</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>1026840716</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>kyobi</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>セルローション　150ml</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>アルソア</t>
+        </is>
+      </c>
+      <c r="F495" t="n">
+        <v>4265</v>
+      </c>
+      <c r="G495" t="n">
+        <v>3</v>
+      </c>
+      <c r="H495" t="b">
+        <v>0</v>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1026840716</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J490"/>
+  <autoFilter ref="A1:J495"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 29, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$495</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$496</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J495"/>
+  <dimension ref="A1:J496"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20555,8 +20555,49 @@
         </is>
       </c>
     </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>1134404499</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>rbq</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>ハード ジェル LTD メンズ 200ｇ</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>ドアーズ</t>
+        </is>
+      </c>
+      <c r="F496" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G496" t="n">
+        <v>0</v>
+      </c>
+      <c r="H496" t="b">
+        <v>0</v>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1134404499</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J495"/>
+  <autoFilter ref="A1:J496"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 31, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$496</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$497</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J496"/>
+  <dimension ref="A1:J497"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20596,8 +20596,49 @@
         </is>
       </c>
     </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>1190275225</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>andginc</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>クーポンOK 　エニシーグローパック CLX フェ イシャルジェルパック　7回分</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>エニシー</t>
+        </is>
+      </c>
+      <c r="F497" t="n">
+        <v>19250</v>
+      </c>
+      <c r="G497" t="n">
+        <v>1</v>
+      </c>
+      <c r="H497" t="b">
+        <v>0</v>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190275225</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J496"/>
+  <autoFilter ref="A1:J497"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 34, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$497</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$498</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J497"/>
+  <dimension ref="A1:J498"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20637,8 +20637,49 @@
         </is>
       </c>
     </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>1166972261</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>cosmesse</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>新 ヘーラールーノ ゴールドミルクローション(乳液) 120ml</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>大高酵素</t>
+        </is>
+      </c>
+      <c r="F498" t="n">
+        <v>3564</v>
+      </c>
+      <c r="G498" t="n">
+        <v>1</v>
+      </c>
+      <c r="H498" t="b">
+        <v>0</v>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1166972261</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J497"/>
+  <autoFilter ref="A1:J498"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 35, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$498</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$500</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J498"/>
+  <dimension ref="A1:J500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20678,8 +20678,90 @@
         </is>
       </c>
     </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>1214979012</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>fromrier</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>[fromrier 公式] EGFシカウォーターサンアンプル 56ml SPF50+PA++++ [ウォーター/マット] フロムリエ</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>fromrier</t>
+        </is>
+      </c>
+      <c r="F499" t="n">
+        <v>3400</v>
+      </c>
+      <c r="G499" t="n">
+        <v>0</v>
+      </c>
+      <c r="H499" t="b">
+        <v>0</v>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214979012</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>1214463806</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>pinkri</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>[正規品] セメンザル ライトクリーム 100ml ㅣ 高保湿 · 肌バリアケア · 敏感肌向け · 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>CONAPIDIL</t>
+        </is>
+      </c>
+      <c r="F500" t="n">
+        <v>19590</v>
+      </c>
+      <c r="G500" t="n">
+        <v>0</v>
+      </c>
+      <c r="H500" t="b">
+        <v>0</v>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214463806</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J498"/>
+  <autoFilter ref="A1:J500"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 17, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$527</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$531</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J527"/>
+  <dimension ref="A1:J531"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21867,8 +21867,172 @@
         </is>
       </c>
     </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>973486483</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>kstargoods_JP</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>[Pyunkang Yul] DEEP CLEANSING OIL</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>ブランドなし</t>
+        </is>
+      </c>
+      <c r="F528" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G528" t="n">
+        <v>0</v>
+      </c>
+      <c r="H528" t="b">
+        <v>0</v>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J528" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=973486483</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>1083676754</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>kstargoods_JP</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>loccitane shea verbena liquid soap 300ml</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>ロクシタン</t>
+        </is>
+      </c>
+      <c r="F529" t="n">
+        <v>4999</v>
+      </c>
+      <c r="G529" t="n">
+        <v>0</v>
+      </c>
+      <c r="H529" t="b">
+        <v>0</v>
+      </c>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J529" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1083676754</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>969163642</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>kstargoods_JP</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>[Labelyoung] Shocking Vitamin Milk Whitening Cream</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>ラベルヤング</t>
+        </is>
+      </c>
+      <c r="F530" t="n">
+        <v>1899</v>
+      </c>
+      <c r="G530" t="n">
+        <v>4</v>
+      </c>
+      <c r="H530" t="b">
+        <v>0</v>
+      </c>
+      <c r="I530" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J530" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=969163642</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>821075839</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>kstargoods_JP</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>[THE SAEM] Urban Eco Harakeke Deep Moisture Toner</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>ブランドなし</t>
+        </is>
+      </c>
+      <c r="F531" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G531" t="n">
+        <v>0</v>
+      </c>
+      <c r="H531" t="b">
+        <v>0</v>
+      </c>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=821075839</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J527"/>
+  <autoFilter ref="A1:J531"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 22, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$535</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$538</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J535"/>
+  <dimension ref="A1:J538"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22195,8 +22195,131 @@
         </is>
       </c>
     </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>1175312429</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>kenkou1bankan</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>キュレル　リップケアクリーム　4.2g</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>キュレル</t>
+        </is>
+      </c>
+      <c r="F536" t="n">
+        <v>800</v>
+      </c>
+      <c r="G536" t="n">
+        <v>0</v>
+      </c>
+      <c r="H536" t="b">
+        <v>0</v>
+      </c>
+      <c r="I536" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175312429</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>1069156212</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>kenkou1bankan</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>いち髪　なめらかスムースケアシャンプー　詰替用　660mL</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>いち髪</t>
+        </is>
+      </c>
+      <c r="F537" t="n">
+        <v>1580</v>
+      </c>
+      <c r="G537" t="n">
+        <v>0</v>
+      </c>
+      <c r="H537" t="b">
+        <v>0</v>
+      </c>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J537" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1069156212</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>1096924691</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>kenkou1bankan</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>キュレル　皮脂トラブルケア　保湿ジェル　120ml</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>キュレル</t>
+        </is>
+      </c>
+      <c r="F538" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G538" t="n">
+        <v>1</v>
+      </c>
+      <c r="H538" t="b">
+        <v>0</v>
+      </c>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J538" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1096924691</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J535"/>
+  <autoFilter ref="A1:J538"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 26, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$543</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$550</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J543"/>
+  <dimension ref="A1:J550"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22523,8 +22523,295 @@
         </is>
       </c>
     </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>1203146466</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Janicekbeauty</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>[「顔からボディまで」全身ケア] アズレン スーディングローション 500ml (大容量) #デイリーケア #韓国美容 #保湿ケア #肌荒れ防止</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>Dr.SANTE</t>
+        </is>
+      </c>
+      <c r="F544" t="n">
+        <v>9950</v>
+      </c>
+      <c r="G544" t="n">
+        <v>0</v>
+      </c>
+      <c r="H544" t="b">
+        <v>0</v>
+      </c>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J544" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203146466</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>1211595698</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Janicekbeauty</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>[高級化粧水・初期ハリ弾力] ダンギ トナー 500ML (引き締め肌シェイパー) #エイジングケア #高保湿ケア #エステコスメ</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F545" t="n">
+        <v>7690</v>
+      </c>
+      <c r="G545" t="n">
+        <v>0</v>
+      </c>
+      <c r="H545" t="b">
+        <v>0</v>
+      </c>
+      <c r="I545" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J545" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211595698</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>1210784489</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Janicekbeauty</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>【韓国エステコスメ】アズレン スーダー トナー 500ml #大容量 #保湿 #肌を整える化粧水 #敏感肌ケア #エステ級ホームスキンケア</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>SANTE</t>
+        </is>
+      </c>
+      <c r="F546" t="n">
+        <v>9875</v>
+      </c>
+      <c r="G546" t="n">
+        <v>0</v>
+      </c>
+      <c r="H546" t="b">
+        <v>0</v>
+      </c>
+      <c r="I546" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210784489</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>1159296798</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Janicekbeauty</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】1025 独島アンプル 45ml#みずみずしい保湿ケア #うるおいチャージ#敏感肌にも#ヒアルロン酸×セラミド</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F547" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G547" t="n">
+        <v>0</v>
+      </c>
+      <c r="H547" t="b">
+        <v>0</v>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159296798</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>1205251780</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>ohnewcompany</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>【韓国1位】 サリシニック ポアクリア ブラックパッド 70枚＋10枚付 毛穴ケア</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>ダーマトリー</t>
+        </is>
+      </c>
+      <c r="F548" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G548" t="n">
+        <v>0</v>
+      </c>
+      <c r="H548" t="b">
+        <v>0</v>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205251780</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>1203144925</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>ohnewcompany</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>【企画】オールアバウト グロウ カバークリーム (35g) + 大王パフ 1枚付き SPF50+ PA++++ 韓国コスメ ベースメイク 24時間持続 崩れない</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>CHASIN’ RABBITS</t>
+        </is>
+      </c>
+      <c r="F549" t="n">
+        <v>1946</v>
+      </c>
+      <c r="G549" t="n">
+        <v>3</v>
+      </c>
+      <c r="H549" t="b">
+        <v>0</v>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203144925</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>1189310191</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>ohnewcompany</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>ローゼPDRN エッセンシャルマスク 10+1枚 (毛穴・キメ・ツヤ肌)</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F550" t="n">
+        <v>1706</v>
+      </c>
+      <c r="G550" t="n">
+        <v>1</v>
+      </c>
+      <c r="H550" t="b">
+        <v>0</v>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189310191</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J543"/>
+  <autoFilter ref="A1:J550"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 28, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$550</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$551</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J550"/>
+  <dimension ref="A1:J551"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22810,8 +22810,49 @@
         </is>
       </c>
     </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>1172255476</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>KVIVE</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>[セット商品]ボリューム シャンプー 500ml+スカルプ シャンプー 500ml /シャンプー 500ml+トリートメント 200ml/大容量/シャンプー 韓国 人気/香りいいシャンプー/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>MONCLOS</t>
+        </is>
+      </c>
+      <c r="F551" t="n">
+        <v>7990</v>
+      </c>
+      <c r="G551" t="n">
+        <v>0</v>
+      </c>
+      <c r="H551" t="b">
+        <v>0</v>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172255476</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J550"/>
+  <autoFilter ref="A1:J551"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 32, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$562</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$563</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J562"/>
+  <dimension ref="A1:J563"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23302,8 +23302,49 @@
         </is>
       </c>
     </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>1207681141</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>miraclim</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>【国内発送】AZケア クレンジングオイル 200ml【正規品】 REEDLE S AZ CARE CLEANSING OIL 韓国スキンケア 毛穴汚れ 皮脂 黒ずみ メイクオフ ディープクレ</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F563" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G563" t="n">
+        <v>0</v>
+      </c>
+      <c r="H563" t="b">
+        <v>0</v>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207681141</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J562"/>
+  <autoFilter ref="A1:J563"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 37, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$573</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$575</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J573"/>
+  <dimension ref="A1:J575"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23753,8 +23753,90 @@
         </is>
       </c>
     </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>1213388857</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>on_j4052</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>タンバリンズ シャワリーボディウォッシュ 240mL 全5種から選択（パピーキーリング＆パフューム2mL 限定プレゼント）</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>タンバリンズ</t>
+        </is>
+      </c>
+      <c r="F574" t="n">
+        <v>6490</v>
+      </c>
+      <c r="G574" t="n">
+        <v>0</v>
+      </c>
+      <c r="H574" t="b">
+        <v>0</v>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213388857</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>1212716725</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>on_j4052</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>【限定特典_ヘアシュシュ付き】NONFICTIONヘアセラムミスト 30mL うるおい ツヤ髪 ヘアケア ヘアミスト 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>ノンフィクション</t>
+        </is>
+      </c>
+      <c r="F575" t="n">
+        <v>6165</v>
+      </c>
+      <c r="G575" t="n">
+        <v>0</v>
+      </c>
+      <c r="H575" t="b">
+        <v>0</v>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J575" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212716725</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J573"/>
+  <autoFilter ref="A1:J575"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 40, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$575</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$576</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J575"/>
+  <dimension ref="A1:J576"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23835,8 +23835,49 @@
         </is>
       </c>
     </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>1148522073</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Marcella</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>朝鮮美人 アクアフレッシュ日焼け止め 50ml×2個 韓国コスメ敏感肌OK保湿タイプ</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F576" t="n">
+        <v>4842</v>
+      </c>
+      <c r="G576" t="n">
+        <v>0</v>
+      </c>
+      <c r="H576" t="b">
+        <v>0</v>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1148522073</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J575"/>
+  <autoFilter ref="A1:J576"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 41, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$576</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$578</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J576"/>
+  <dimension ref="A1:J578"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23876,8 +23876,90 @@
         </is>
       </c>
     </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>1208578817</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>wellcomkorea</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>基礎3点セット シワ・ハリ改善（ブースター130ml＋セラム45ml＋アクティブクリーム50ml）</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F577" t="n">
+        <v>23850</v>
+      </c>
+      <c r="G577" t="n">
+        <v>0</v>
+      </c>
+      <c r="H577" t="b">
+        <v>0</v>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J577" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208578817</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>1139832560</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>wellcomkorea</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>低刺激 皮むきクリーム200ml 1個</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>イリユン</t>
+        </is>
+      </c>
+      <c r="F578" t="n">
+        <v>3442</v>
+      </c>
+      <c r="G578" t="n">
+        <v>0</v>
+      </c>
+      <c r="H578" t="b">
+        <v>0</v>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J578" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139832560</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J576"/>
+  <autoFilter ref="A1:J578"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 43, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$579</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$582</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J579"/>
+  <dimension ref="A1:J582"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23999,8 +23999,131 @@
         </is>
       </c>
     </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>1202534389</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>LILIEN</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>[うす付プレミアムUV下地] トーンアップ サンスキン 40ml 1個 SPF50+ PA++++ 選べる3カラー</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>KAHI</t>
+        </is>
+      </c>
+      <c r="F580" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G580" t="n">
+        <v>0</v>
+      </c>
+      <c r="H580" t="b">
+        <v>0</v>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J580" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202534389</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>1196514379</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>LILIEN</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>[毛穴・キメケア] ゼロ毛穴パッド本品1+リフィル1＋10枚+ミニケース 計150枚 企画セット</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F581" t="n">
+        <v>6200</v>
+      </c>
+      <c r="G581" t="n">
+        <v>2</v>
+      </c>
+      <c r="H581" t="b">
+        <v>0</v>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196514379</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>1136771755</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>LILIEN</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>ホワイトトリュフ&amp;nbsp;ファースト&amp;nbsp;スプレーセラム100ml + ウォーターフル トーンアップ SUN CREAM(ピンク）50ml 企画セット</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F582" t="n">
+        <v>6700</v>
+      </c>
+      <c r="G582" t="n">
+        <v>0</v>
+      </c>
+      <c r="H582" t="b">
+        <v>0</v>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J582" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1136771755</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J579"/>
+  <autoFilter ref="A1:J582"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 44, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$582</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$587</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J582"/>
+  <dimension ref="A1:J587"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24122,8 +24122,213 @@
         </is>
       </c>
     </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>1193834160</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>KBEAUTYOFFICIALSTORE</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>BRINGGREEN 公式 ブリングリーン ティーツリーシカセンシティブクレンジングウォーター 500ml BRINGGREEN 洗顔 クレンジング</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F583" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G583" t="n">
+        <v>1</v>
+      </c>
+      <c r="H583" t="b">
+        <v>0</v>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J583" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193834160</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>1193834173</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>KBEAUTYOFFICIALSTORE</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>dAlba 公式 ダルバ 下地 グリーン ウォータフル トーンアップサンクリーム 50ml 5種 ピンク パープル カバーベージュ 21号 23号 日焼け止め</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F584" t="n">
+        <v>4290</v>
+      </c>
+      <c r="G584" t="n">
+        <v>0</v>
+      </c>
+      <c r="H584" t="b">
+        <v>0</v>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193834173</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>1191474289</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>KBEAUTYOFFICIALSTORE</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>REJURAN 公式 リジュラン PDRN (c-PDRN) ポアタイトニングトナーパッド 60枚+60枚 トナーパッド パック</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F585" t="n">
+        <v>7690</v>
+      </c>
+      <c r="G585" t="n">
+        <v>0</v>
+      </c>
+      <c r="H585" t="b">
+        <v>0</v>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J585" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191474289</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>1191474301</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>KBEAUTYOFFICIALSTORE</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>REJURAN 公式 リジュラン PDRN (c-PDRN) ポアタイトニングトナーパッド 60枚 トナーパッド パック</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F586" t="n">
+        <v>4490</v>
+      </c>
+      <c r="G586" t="n">
+        <v>0</v>
+      </c>
+      <c r="H586" t="b">
+        <v>0</v>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J586" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191474301</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>1212713877</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Lulupi</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>【フィー】 シェイキングシナジーミスト 50ml 全4種</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F587" t="n">
+        <v>2654</v>
+      </c>
+      <c r="G587" t="n">
+        <v>9</v>
+      </c>
+      <c r="H587" t="b">
+        <v>0</v>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212713877</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J582"/>
+  <autoFilter ref="A1:J587"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 46, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$588</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$592</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J588"/>
+  <dimension ref="A1:J592"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24368,8 +24368,172 @@
         </is>
       </c>
     </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>1215169640</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>serafinet</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>【日本正規品】トラベルサイズ エクスフォリエーティングポリッシュ 16.2g スクラブ洗顔料</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>ZO SKIN</t>
+        </is>
+      </c>
+      <c r="F589" t="n">
+        <v>3690</v>
+      </c>
+      <c r="G589" t="n">
+        <v>0</v>
+      </c>
+      <c r="H589" t="b">
+        <v>0</v>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1215169640</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>1198838562</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>serafinet</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>【日本正規品】ネックコンプレックス 50ml 美容液</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>ZO SKIN</t>
+        </is>
+      </c>
+      <c r="F590" t="n">
+        <v>21980</v>
+      </c>
+      <c r="G590" t="n">
+        <v>1</v>
+      </c>
+      <c r="H590" t="b">
+        <v>0</v>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198838562</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>1192787209</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>serafinet</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>ワイコ WiQo フェイスフルイド 30ml 美容液</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>WiQo</t>
+        </is>
+      </c>
+      <c r="F591" t="n">
+        <v>12300</v>
+      </c>
+      <c r="G591" t="n">
+        <v>2</v>
+      </c>
+      <c r="H591" t="b">
+        <v>0</v>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192787209</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>1211989928</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>good-mark</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>保湿化粧水さっぱりタイプ 詰替用</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>ちふれ</t>
+        </is>
+      </c>
+      <c r="F592" t="n">
+        <v>1393</v>
+      </c>
+      <c r="G592" t="n">
+        <v>0</v>
+      </c>
+      <c r="H592" t="b">
+        <v>0</v>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J592" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211989928</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J588"/>
+  <autoFilter ref="A1:J592"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 49, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$592</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$594</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J592"/>
+  <dimension ref="A1:J594"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24532,8 +24532,90 @@
         </is>
       </c>
     </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>1192705019</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>andnine-shop</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>【超保湿×サボテン抱水美容】サボン ド サボタ シャンプー &amp;amp; トリートメント セット [ モイストプランプ / マスターリペア ]</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>Savon du Savota</t>
+        </is>
+      </c>
+      <c r="F593" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G593" t="n">
+        <v>7</v>
+      </c>
+      <c r="H593" t="b">
+        <v>0</v>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J593" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192705019</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>1194273610</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>andnine-shop</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>【超保湿×サボテン抱水美容】サボン ド サボタ モイストプランプ 雪華ラベンダーティー お試し2連付き シャンプー &amp;amp; トリートメント ペアセット 420mL＋420g</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>Savon du Savota</t>
+        </is>
+      </c>
+      <c r="F594" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G594" t="n">
+        <v>5</v>
+      </c>
+      <c r="H594" t="b">
+        <v>0</v>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194273610</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J592"/>
+  <autoFilter ref="A1:J594"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 50, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$594</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$600</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J594"/>
+  <dimension ref="A1:J600"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24614,8 +24614,254 @@
         </is>
       </c>
     </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>1188691246</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>offselection</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>EVERYSKIN Pro+ スキンジェルplus 150g 化粧水 ジェル状化粧水 セラミド</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>Clear_pro</t>
+        </is>
+      </c>
+      <c r="F595" t="n">
+        <v>6650</v>
+      </c>
+      <c r="G595" t="n">
+        <v>1</v>
+      </c>
+      <c r="H595" t="b">
+        <v>0</v>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188691246</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>1146209578</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>offselection</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>ドクターリセラ アクアヴィーナス プラチナピール 40g</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>ドクターリセラ</t>
+        </is>
+      </c>
+      <c r="F596" t="n">
+        <v>9980</v>
+      </c>
+      <c r="G596" t="n">
+        <v>0</v>
+      </c>
+      <c r="H596" t="b">
+        <v>0</v>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146209578</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>1137830849</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>christinajapan</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>公式 【本品３本＋サンプルパウチ５袋】 THERASKIN　テラスキン ヒアルロン酸美容液 30ml サンプル付き</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>CHRISTINA</t>
+        </is>
+      </c>
+      <c r="F597" t="n">
+        <v>23100</v>
+      </c>
+      <c r="G597" t="n">
+        <v>1</v>
+      </c>
+      <c r="H597" t="b">
+        <v>0</v>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1137830849</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>1137830545</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>christinajapan</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>公式 【本品２本＋サンプルパウチ３袋】 THERASKIN　テラスキン ヒアルロン酸美容液 30ml サンプル付き</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>CHRISTINA</t>
+        </is>
+      </c>
+      <c r="F598" t="n">
+        <v>15400</v>
+      </c>
+      <c r="G598" t="n">
+        <v>7</v>
+      </c>
+      <c r="H598" t="b">
+        <v>0</v>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1137830545</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>1121854938</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>christinajapan</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>公式 BIO SATAIN SERUM ビオサテンセラム</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>CHRISTINA</t>
+        </is>
+      </c>
+      <c r="F599" t="n">
+        <v>13200</v>
+      </c>
+      <c r="G599" t="n">
+        <v>0</v>
+      </c>
+      <c r="H599" t="b">
+        <v>0</v>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1121854938</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>1121854937</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>christinajapan</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>公式 HYDRA FUSION CONCENTRATE ハイドラフュージョン コンセントレート</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>CHRISTINA</t>
+        </is>
+      </c>
+      <c r="F600" t="n">
+        <v>8690</v>
+      </c>
+      <c r="G600" t="n">
+        <v>0</v>
+      </c>
+      <c r="H600" t="b">
+        <v>0</v>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J600" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1121854937</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J594"/>
+  <autoFilter ref="A1:J600"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 52, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$600</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$601</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J600"/>
+  <dimension ref="A1:J601"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24860,8 +24860,49 @@
         </is>
       </c>
     </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>1159661232</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>engrace</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>熊野筆 フラワー 洗顔ブラシ フェイスブラシ 洗顔筆 ホワイト 化粧筆 熊の筆 熊野化粧筆 洗顔 洗顔用 クレンジング 泡立て ブラシ 贈り物 高級 ギフト お祝い おしゃれ 可愛い 熊野 おすすめ</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>KOYUDO</t>
+        </is>
+      </c>
+      <c r="F601" t="n">
+        <v>5500</v>
+      </c>
+      <c r="G601" t="n">
+        <v>0</v>
+      </c>
+      <c r="H601" t="b">
+        <v>0</v>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J601" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159661232</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J600"/>
+  <autoFilter ref="A1:J601"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 55, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$602</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$605</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J602"/>
+  <dimension ref="A1:J605"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24942,8 +24942,131 @@
         </is>
       </c>
     </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>1184605113</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>neobase</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>ディアダリア デイリーディフェンス PDRN BBクリーム SPF40 5ml デイリーベース ナチュラルトーン 携帯用ベース</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>Dermablock</t>
+        </is>
+      </c>
+      <c r="F603" t="n">
+        <v>1520</v>
+      </c>
+      <c r="G603" t="n">
+        <v>0</v>
+      </c>
+      <c r="H603" t="b">
+        <v>0</v>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J603" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1184605113</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>1181238873</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>neobase</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>【2本セット】スーパーアクア200ml×2 ウルトラ ヒアルロン クレンジングフォーム 洗顔フォーム 保湿 しっとり デイリー</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F604" t="n">
+        <v>2022</v>
+      </c>
+      <c r="G604" t="n">
+        <v>0</v>
+      </c>
+      <c r="H604" t="b">
+        <v>0</v>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181238873</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>1181238841</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>neobase</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>水トクス 光彩保湿パッド 2.0 50枚入</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F605" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G605" t="n">
+        <v>0</v>
+      </c>
+      <c r="H605" t="b">
+        <v>0</v>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181238841</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J602"/>
+  <autoFilter ref="A1:J605"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 56, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$605</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$608</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J605"/>
+  <dimension ref="A1:J608"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25065,8 +25065,131 @@
         </is>
       </c>
     </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>1165169271</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>truvio</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>[ミニパフューム/シナモロール キーリング 贈呈] パフューム ミスト 94ml 10種</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>ボディファンタジー</t>
+        </is>
+      </c>
+      <c r="F606" t="n">
+        <v>2996</v>
+      </c>
+      <c r="G606" t="n">
+        <v>0</v>
+      </c>
+      <c r="H606" t="b">
+        <v>0</v>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165169271</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>1210685384</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>milky</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>ダヴィネス オーセンティック バター 230ml【 ダヴィネス ( Davines )】 濃厚保湿バター ヘアケア スキンケア ボディケア ヘアクリーム</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>ダビネス</t>
+        </is>
+      </c>
+      <c r="F607" t="n">
+        <v>4380</v>
+      </c>
+      <c r="G607" t="n">
+        <v>0</v>
+      </c>
+      <c r="H607" t="b">
+        <v>0</v>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210685384</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>1199672854</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>milky</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>【送料込み】【自由に選べる3個】ピュレア クリアエッセンスマスク 7枚入り×3個【クリア・レチビタ・ライスなど】フェイスマスク シートマスク パック【メール便】</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>ピュレア</t>
+        </is>
+      </c>
+      <c r="F608" t="n">
+        <v>1670</v>
+      </c>
+      <c r="G608" t="n">
+        <v>5</v>
+      </c>
+      <c r="H608" t="b">
+        <v>0</v>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J608" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199672854</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J605"/>
+  <autoFilter ref="A1:J608"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 58, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$608</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$609</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J608"/>
+  <dimension ref="A1:J609"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25188,8 +25188,49 @@
         </is>
       </c>
     </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>835715938</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>cosmedenet</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>最安値挑戦中！クリニーク テイク ザ デイ オフ 125ml 2個セット</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>クリニーク</t>
+        </is>
+      </c>
+      <c r="F609" t="n">
+        <v>6310</v>
+      </c>
+      <c r="G609" t="n">
+        <v>1</v>
+      </c>
+      <c r="H609" t="b">
+        <v>0</v>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J609" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=835715938</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J608"/>
+  <autoFilter ref="A1:J609"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 61, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$611</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$612</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J611"/>
+  <dimension ref="A1:J612"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25311,8 +25311,49 @@
         </is>
       </c>
     </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>1213920984</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>demaf</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>【公式】ライスジェルクレンザー 150ml</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>De:maf</t>
+        </is>
+      </c>
+      <c r="F612" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G612" t="n">
+        <v>0</v>
+      </c>
+      <c r="H612" t="b">
+        <v>0</v>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213920984</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J611"/>
+  <autoFilter ref="A1:J612"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 62, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$612</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$616</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J612"/>
+  <dimension ref="A1:J616"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25352,8 +25352,172 @@
         </is>
       </c>
     </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>1134208958</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>bibian</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>AQ リペア ボリューム トリートメント コンディショナー　本体　 600g　【店頭同様の国内正規品】</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>コスメデコルテ</t>
+        </is>
+      </c>
+      <c r="F613" t="n">
+        <v>6480</v>
+      </c>
+      <c r="G613" t="n">
+        <v>0</v>
+      </c>
+      <c r="H613" t="b">
+        <v>0</v>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1134208958</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>1170473064</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>bibian</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>コアバランス オイル / 50mL　フェイスオイル・バーム　美容オイル　オイルなのにさらり</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>アスレティア</t>
+        </is>
+      </c>
+      <c r="F614" t="n">
+        <v>5700</v>
+      </c>
+      <c r="G614" t="n">
+        <v>0</v>
+      </c>
+      <c r="H614" t="b">
+        <v>0</v>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170473064</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>1114435128</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>bibian</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>AQ リペア スムース シャンプー Lサイズ 600mL　シャンプー・コンディショナー 頭皮ケア【店頭同様の国内正規品】</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>コスメデコルテ</t>
+        </is>
+      </c>
+      <c r="F615" t="n">
+        <v>5910</v>
+      </c>
+      <c r="G615" t="n">
+        <v>1</v>
+      </c>
+      <c r="H615" t="b">
+        <v>0</v>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J615" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1114435128</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>1209062941</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>domingojapan</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>【国内正規品 】　 スキン コンダクター 60g ベタつき 乾燥 クリーム モイスチャライザー うるおい べたつかない フェイスクリーム</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>カネボウ</t>
+        </is>
+      </c>
+      <c r="F616" t="n">
+        <v>5599</v>
+      </c>
+      <c r="G616" t="n">
+        <v>2</v>
+      </c>
+      <c r="H616" t="b">
+        <v>0</v>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209062941</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J612"/>
+  <autoFilter ref="A1:J616"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 65, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$616</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$618</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J616"/>
+  <dimension ref="A1:J618"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25516,8 +25516,90 @@
         </is>
       </c>
     </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>1209647884</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>oooooooOFFICIAL</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>オーラルスプレー 5種類のフレーバーがあります 口腔スプレー プロバイオティクス 長持ちする新鮮さと口腔ケア シュガーフリー</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>CEELIKE</t>
+        </is>
+      </c>
+      <c r="F617" t="n">
+        <v>1420</v>
+      </c>
+      <c r="G617" t="n">
+        <v>2</v>
+      </c>
+      <c r="H617" t="b">
+        <v>0</v>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J617" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209647884</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>1212300102</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>oooooooOFFICIAL</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>PRAMY メイクアップセッティングミスト (100ml) フィキシングスプレー だいようりょう 化粧崩れ防止 メイク長持ち 汗・皮脂に ナチュラル仕上げ高い保湿感</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>PRAMY</t>
+        </is>
+      </c>
+      <c r="F618" t="n">
+        <v>1179</v>
+      </c>
+      <c r="G618" t="n">
+        <v>0</v>
+      </c>
+      <c r="H618" t="b">
+        <v>0</v>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J618" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212300102</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J616"/>
+  <autoFilter ref="A1:J618"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 68, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$618</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$624</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J618"/>
+  <dimension ref="A1:J624"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25598,8 +25598,254 @@
         </is>
       </c>
     </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>1206596838</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>rdrd</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>【8/14~23限定セール+金額別GIFT付】 りんごトナー/セラム</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>rdrd</t>
+        </is>
+      </c>
+      <c r="F619" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G619" t="n">
+        <v>5</v>
+      </c>
+      <c r="H619" t="b">
+        <v>0</v>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J619" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206596838</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>1206596451</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>rdrd</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>【8/14~23限定セール+金額別GIFT付】 ミニセラム 7ml 選べる2＋1セット（各種類1個まで選択可能）</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>rdrd</t>
+        </is>
+      </c>
+      <c r="F620" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G620" t="n">
+        <v>5</v>
+      </c>
+      <c r="H620" t="b">
+        <v>0</v>
+      </c>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J620" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206596451</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>1206216824</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>rdrd</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>【8/14~23限定セール+金額別GIFT付】 ミニセラム 7ml 単品</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>rdrd</t>
+        </is>
+      </c>
+      <c r="F621" t="n">
+        <v>750</v>
+      </c>
+      <c r="G621" t="n">
+        <v>6</v>
+      </c>
+      <c r="H621" t="b">
+        <v>0</v>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206216824</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>1206216803</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>rdrd</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>【8/14~23限定セール+金額別GIFT付】 選べるセラム2個セット 30mlx2</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>rdrd</t>
+        </is>
+      </c>
+      <c r="F622" t="n">
+        <v>4400</v>
+      </c>
+      <c r="G622" t="n">
+        <v>2</v>
+      </c>
+      <c r="H622" t="b">
+        <v>0</v>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J622" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206216803</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>1195132806</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>purepusion</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>【毛穴1位】グリーントマト NMN ポア リフティング アンプル40ml</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>Sung Boon Editor</t>
+        </is>
+      </c>
+      <c r="F623" t="n">
+        <v>2480</v>
+      </c>
+      <c r="G623" t="n">
+        <v>0</v>
+      </c>
+      <c r="H623" t="b">
+        <v>0</v>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J623" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195132806</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>1183683721</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>purepusion</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>リペア モイスト エッセンス シートマスク 2.0 30ml/30本(大容量 パック/パック おすすめ/コラーゲン/睡眠パック/ハリツヤ)</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>GIK</t>
+        </is>
+      </c>
+      <c r="F624" t="n">
+        <v>3280</v>
+      </c>
+      <c r="G624" t="n">
+        <v>1</v>
+      </c>
+      <c r="H624" t="b">
+        <v>0</v>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J624" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183683721</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J618"/>
+  <autoFilter ref="A1:J624"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 70, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$625</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$628</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J625"/>
+  <dimension ref="A1:J628"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25885,8 +25885,131 @@
         </is>
       </c>
     </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>1151760666</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>w-arata</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>【濃密美容液】 CVITASプラス ビタミンC アゼライン酸 レチノール バクチオール C SERUM+ セラム 美容液 (約2ヶ月分) 50ml 毛穴ケア 柑橘 香り シービタス CVITAS +</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>CVITAS</t>
+        </is>
+      </c>
+      <c r="F626" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G626" t="n">
+        <v>7</v>
+      </c>
+      <c r="H626" t="b">
+        <v>0</v>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J626" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151760666</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>1170223360</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>generic-cosmetics</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>【単品】GC プレミアムオイル　クレンジングオイル</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>ジェネリック化粧品</t>
+        </is>
+      </c>
+      <c r="F627" t="n">
+        <v>2860</v>
+      </c>
+      <c r="G627" t="n">
+        <v>1</v>
+      </c>
+      <c r="H627" t="b">
+        <v>0</v>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J627" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170223360</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>1156716637</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>generic-cosmetics</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>【単品】GC スキンクリーム 50g 美容クリーム　ガラクトミセス培養液</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>ジェネリック化粧品</t>
+        </is>
+      </c>
+      <c r="F628" t="n">
+        <v>2530</v>
+      </c>
+      <c r="G628" t="n">
+        <v>5</v>
+      </c>
+      <c r="H628" t="b">
+        <v>0</v>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J628" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156716637</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J625"/>
+  <autoFilter ref="A1:J628"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 71, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$628</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$631</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J628"/>
+  <dimension ref="A1:J631"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26008,8 +26008,131 @@
         </is>
       </c>
     </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>1158161386</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>beenkong2</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>ピュリファイングソーダフォーム, 150ml</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F629" t="n">
+        <v>1199</v>
+      </c>
+      <c r="G629" t="n">
+        <v>8</v>
+      </c>
+      <c r="H629" t="b">
+        <v>0</v>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J629" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158161386</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>1158164812</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>beenkong2</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>リンクルバウンス水分パーフェクティングマスク 35g 3枚</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>KAHI</t>
+        </is>
+      </c>
+      <c r="F630" t="n">
+        <v>7500</v>
+      </c>
+      <c r="G630" t="n">
+        <v>2</v>
+      </c>
+      <c r="H630" t="b">
+        <v>0</v>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J630" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158164812</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>1158164452</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>beenkong2</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>インテンスケアゴールド24Kスネイルフォームクレンザー 150ml :: 弾力 栄養 保湿 クレンザ</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>トニーモリー</t>
+        </is>
+      </c>
+      <c r="F631" t="n">
+        <v>2330</v>
+      </c>
+      <c r="G631" t="n">
+        <v>0</v>
+      </c>
+      <c r="H631" t="b">
+        <v>0</v>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J631" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158164452</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J628"/>
+  <autoFilter ref="A1:J631"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 73, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$632</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$633</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J632"/>
+  <dimension ref="A1:J633"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26172,8 +26172,49 @@
         </is>
       </c>
     </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>1210367966</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>coscoskorea</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>ツーフェイスオイルミスト 50ml</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F633" t="n">
+        <v>5250</v>
+      </c>
+      <c r="G633" t="n">
+        <v>0</v>
+      </c>
+      <c r="H633" t="b">
+        <v>0</v>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J633" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210367966</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J632"/>
+  <autoFilter ref="A1:J633"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 79, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$634</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$635</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J634"/>
+  <dimension ref="A1:J635"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26254,8 +26254,49 @@
         </is>
       </c>
     </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>1179393260</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>neafneaf</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>ピーチフィットコラーゲン ゲルマスク (5枚入り) + ピーチフィットコラーゲン クリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>neaf neaf</t>
+        </is>
+      </c>
+      <c r="F635" t="n">
+        <v>5150</v>
+      </c>
+      <c r="G635" t="n">
+        <v>5</v>
+      </c>
+      <c r="H635" t="b">
+        <v>0</v>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J635" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179393260</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J634"/>
+  <autoFilter ref="A1:J635"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 80, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$635</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$638</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J635"/>
+  <dimension ref="A1:J638"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26295,8 +26295,131 @@
         </is>
       </c>
     </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>1105411201</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>venusmall</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>化粧異物トラブルのないチョンギュルのクレンザー150ml/韓国公式オリジナル</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>S2ND</t>
+        </is>
+      </c>
+      <c r="F636" t="n">
+        <v>3340</v>
+      </c>
+      <c r="G636" t="n">
+        <v>0</v>
+      </c>
+      <c r="H636" t="b">
+        <v>0</v>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1105411201</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>1183301096</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>venusmall</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>【正規品・並行輸入品】[NEW] 10秒ケア マイクロバブルパック 大容量150回分 エアバブルマスク 4種セット（ハリ/トーンアップ/整肌/保湿）</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>GASH</t>
+        </is>
+      </c>
+      <c r="F637" t="n">
+        <v>3830</v>
+      </c>
+      <c r="G637" t="n">
+        <v>0</v>
+      </c>
+      <c r="H637" t="b">
+        <v>0</v>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J637" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183301096</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>1133005945</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>venusmall</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>韓国 公式 正規品 [病院専用] ラポラピルナトックス50ml/rapporapy lunatox/かゆみ/ 肌トーン/ 肌のかゆみ/ 皮脂調節炎症減少/ 機能性化粧品</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>Dermagen</t>
+        </is>
+      </c>
+      <c r="F638" t="n">
+        <v>4060</v>
+      </c>
+      <c r="G638" t="n">
+        <v>0</v>
+      </c>
+      <c r="H638" t="b">
+        <v>0</v>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J638" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1133005945</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J635"/>
+  <autoFilter ref="A1:J638"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 82, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$640</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$642</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J640"/>
+  <dimension ref="A1:J642"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26500,8 +26500,90 @@
         </is>
       </c>
     </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>1197537497</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>kanalia</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>iroha koharu // スリムで コンパクト はじめての一歩にやさしさを / フェムケア 【国内配送】【最短翌日】</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>iroha</t>
+        </is>
+      </c>
+      <c r="F641" t="n">
+        <v>1968</v>
+      </c>
+      <c r="G641" t="n">
+        <v>1</v>
+      </c>
+      <c r="H641" t="b">
+        <v>0</v>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J641" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197537497</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>1111887703</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>schonuJ</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>クーリングボディソープ メントール クーリング感 天然レモンの香り ハンドメイド100%</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>SCHONU</t>
+        </is>
+      </c>
+      <c r="F642" t="n">
+        <v>990</v>
+      </c>
+      <c r="G642" t="n">
+        <v>4</v>
+      </c>
+      <c r="H642" t="b">
+        <v>0</v>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J642" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1111887703</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J640"/>
+  <autoFilter ref="A1:J642"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 83, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$642</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$645</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J642"/>
+  <dimension ref="A1:J645"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26582,8 +26582,131 @@
         </is>
       </c>
     </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>1204720270</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>atbq10</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>[3点セット] ディープレイヤー シャンプー ExV エクストラベルベッティ 500mL + トリートメント ExV 470g + H 40g セット モルトベーネ ビューティーエクスペリエンス</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>ディープレイヤー</t>
+        </is>
+      </c>
+      <c r="F643" t="n">
+        <v>6400</v>
+      </c>
+      <c r="G643" t="n">
+        <v>0</v>
+      </c>
+      <c r="H643" t="b">
+        <v>0</v>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J643" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204720270</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>1201828740</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>atbq10</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>コスティン クールシャンプー ブラック 3000mL 詰め替え 業務用 レフィル 日本製 爽快 クール メンズ 夏 シャンプー 暑さ対策 COSTIN 日本ケミコス リビック RIBIC エレガン</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>コスティン</t>
+        </is>
+      </c>
+      <c r="F644" t="n">
+        <v>4830</v>
+      </c>
+      <c r="G644" t="n">
+        <v>0</v>
+      </c>
+      <c r="H644" t="b">
+        <v>0</v>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J644" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201828740</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>1135253160</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>atbq10</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>プライミング シャンプー &amp;amp; フォーティファイング トリートメント ゴールドクレイ 800mL+800g 詰め替え レフィル セット CLAYESTHE GOLD CLAY 毛穴ケア</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>CLAY ESTHE</t>
+        </is>
+      </c>
+      <c r="F645" t="n">
+        <v>7200</v>
+      </c>
+      <c r="G645" t="n">
+        <v>6</v>
+      </c>
+      <c r="H645" t="b">
+        <v>0</v>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J645" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135253160</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J642"/>
+  <autoFilter ref="A1:J645"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 86, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$647</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$649</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J647"/>
+  <dimension ref="A1:J649"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26787,8 +26787,90 @@
         </is>
       </c>
     </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>1125135877</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>z-onemall</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>クレ・ド・ポー ボーテ / Cle de Peau Beaute　ローションエサンシエルＡ / 本体 / 170mL レフィル170mL</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>クレドポーボーテ</t>
+        </is>
+      </c>
+      <c r="F648" t="n">
+        <v>14300</v>
+      </c>
+      <c r="G648" t="n">
+        <v>0</v>
+      </c>
+      <c r="H648" t="b">
+        <v>0</v>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1125135877</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>1163060620</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>tairiku</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>7月21日リニューアル発売　国内正規品　クレ・ド・ポー ボーテ　スキンケア本体　全６種</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>資生堂</t>
+        </is>
+      </c>
+      <c r="F649" t="n">
+        <v>13748</v>
+      </c>
+      <c r="G649" t="n">
+        <v>5</v>
+      </c>
+      <c r="H649" t="b">
+        <v>0</v>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J649" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163060620</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J647"/>
+  <autoFilter ref="A1:J649"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 92, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$649</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$652</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J649"/>
+  <dimension ref="A1:J652"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26869,8 +26869,131 @@
         </is>
       </c>
     </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>1065488606</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>vipurasu</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>ブラックシリーズ ミハツシャンプー 350ml ヘアケア サロン専売品</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>MONNALI</t>
+        </is>
+      </c>
+      <c r="F650" t="n">
+        <v>4830</v>
+      </c>
+      <c r="G650" t="n">
+        <v>9</v>
+      </c>
+      <c r="H650" t="b">
+        <v>0</v>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1065488606</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>1065488626</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>vipurasu</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>ゴールドシリーズ TR50 クレンジング 500ml メイク落とし サロン専売</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>MONNALI</t>
+        </is>
+      </c>
+      <c r="F651" t="n">
+        <v>10070</v>
+      </c>
+      <c r="G651" t="n">
+        <v>8</v>
+      </c>
+      <c r="H651" t="b">
+        <v>0</v>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1065488626</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>1209089358</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>anetos</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>【毛穴ケア】00:00 クラリファイング クレイパック 泥パック100g天然クレイCICA配合 角栓ケア 黒ずみ吸着 毛穴引き締め 毛穴ケア AHA PHA ナイアシンアミド ざらつき</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>ANETOS</t>
+        </is>
+      </c>
+      <c r="F652" t="n">
+        <v>1560</v>
+      </c>
+      <c r="G652" t="n">
+        <v>1</v>
+      </c>
+      <c r="H652" t="b">
+        <v>0</v>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J652" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209089358</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J649"/>
+  <autoFilter ref="A1:J652"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 94, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$652</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$653</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J652"/>
+  <dimension ref="A1:J653"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26992,8 +26992,49 @@
         </is>
       </c>
     </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>1131446998</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>igalab</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>【公式】IGA LAB バリアサポート クレンジングオイル 100ml 毛穴ケア 黒ずみ 角質ケア ドクターズコスメ ニキビケア ニキビ跡 敏感肌 日本製 国産</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>IGA LAB</t>
+        </is>
+      </c>
+      <c r="F653" t="n">
+        <v>4940</v>
+      </c>
+      <c r="G653" t="n">
+        <v>3</v>
+      </c>
+      <c r="H653" t="b">
+        <v>0</v>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J653" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1131446998</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J652"/>
+  <autoFilter ref="A1:J653"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 98, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$654</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$658</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J654"/>
+  <dimension ref="A1:J658"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27074,8 +27074,172 @@
         </is>
       </c>
     </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>1193252073</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>lionel</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>mine コンセントレートセラム04 150g　集中補修 ヘアセラム 洗い流さない トリートメント ダメージケア 熱ダメージ対策</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>マイン</t>
+        </is>
+      </c>
+      <c r="F655" t="n">
+        <v>3080</v>
+      </c>
+      <c r="G655" t="n">
+        <v>0</v>
+      </c>
+      <c r="H655" t="b">
+        <v>0</v>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J655" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193252073</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>1195197102</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>lionel</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Skin Care Ism スキンケアイズム ベッドタイム レストマスク 100g　就寝用 美白 抗しわ 抗炎症 パック スキンケア 日本製</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>スキンケアイズム</t>
+        </is>
+      </c>
+      <c r="F656" t="n">
+        <v>11000</v>
+      </c>
+      <c r="G656" t="n">
+        <v>1</v>
+      </c>
+      <c r="H656" t="b">
+        <v>0</v>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J656" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195197102</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>1193315498</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>lionel</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Skin Care Ism スキンケアイズム ミルキー ホエイ ピーリングソープ 85g　洗顔 石けん 毛穴 くすみ ざらつき ケア 保湿</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>スキンケアイズム</t>
+        </is>
+      </c>
+      <c r="F657" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G657" t="n">
+        <v>0</v>
+      </c>
+      <c r="H657" t="b">
+        <v>0</v>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J657" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193315498</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>1175142824</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>lionel</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>ソフ umiumi サンライトUVスプレー ブーケ(フラワーフレグランス) SPF50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>soeff</t>
+        </is>
+      </c>
+      <c r="F658" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G658" t="n">
+        <v>2</v>
+      </c>
+      <c r="H658" t="b">
+        <v>0</v>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J658" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175142824</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J654"/>
+  <autoFilter ref="A1:J658"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 107, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$658</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$659</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J658"/>
+  <dimension ref="A1:J659"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27238,8 +27238,49 @@
         </is>
       </c>
     </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>727975892</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>skylakejapan</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>湖水宝鑑リラックスマスクパック</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>ハヌルホス</t>
+        </is>
+      </c>
+      <c r="F659" t="n">
+        <v>385</v>
+      </c>
+      <c r="G659" t="n">
+        <v>7</v>
+      </c>
+      <c r="H659" t="b">
+        <v>0</v>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J659" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=727975892</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J658"/>
+  <autoFilter ref="A1:J659"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 112, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$660</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$661</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J660"/>
+  <dimension ref="A1:J661"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27320,8 +27320,49 @@
         </is>
       </c>
     </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>999870496</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>megucorp</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>【レビュー特典200P】ハリーヴィーナス プラチナウォッシュ [100ｇ]　濃密泡 毛穴黒ずみ 角栓 ざらざら すっきり プラチナナノコロイド フラーレン 配合 大人女子 洗顔料 洗顔フォーム</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>MEGU</t>
+        </is>
+      </c>
+      <c r="F661" t="n">
+        <v>3993</v>
+      </c>
+      <c r="G661" t="n">
+        <v>0</v>
+      </c>
+      <c r="H661" t="b">
+        <v>0</v>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J661" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=999870496</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J660"/>
+  <autoFilter ref="A1:J661"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 115, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$661</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$665</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J661"/>
+  <dimension ref="A1:J665"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27361,8 +27361,172 @@
         </is>
       </c>
     </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>1214567988</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>monscompany</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>公式 illen【選べる2種】マスクウォッシュ 130g パック洗顔 クレイ洗顔 クラリティ／ハイドロ 毛穴汚れ 古い角質 皮脂 インナードライ 乾燥肌 弱酸性 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>illen</t>
+        </is>
+      </c>
+      <c r="F662" t="n">
+        <v>2380</v>
+      </c>
+      <c r="G662" t="n">
+        <v>0</v>
+      </c>
+      <c r="H662" t="b">
+        <v>0</v>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214567988</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>1209053534</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Lowlize</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>【公式/新発売】カーミング トラベルキット+(*カート番号ごとに一つ)シャシェ2種+バランスリカバリーマスク1枚</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>Lowlize</t>
+        </is>
+      </c>
+      <c r="F663" t="n">
+        <v>2916</v>
+      </c>
+      <c r="G663" t="n">
+        <v>6</v>
+      </c>
+      <c r="H663" t="b">
+        <v>0</v>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J663" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209053534</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>1205876934</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Lowlize</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>【公式】バランスリカバリーマスク1枚+(*カート番号ごとに一つ)シャシェ2種</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>Lowlize</t>
+        </is>
+      </c>
+      <c r="F664" t="n">
+        <v>378</v>
+      </c>
+      <c r="G664" t="n">
+        <v>7</v>
+      </c>
+      <c r="H664" t="b">
+        <v>0</v>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J664" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205876934</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>1200670476</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Lowlize</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>【公式】エアリーデュサンセラム+(*カート番号ごとに一つ)シャシェ2種</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>Lowlize</t>
+        </is>
+      </c>
+      <c r="F665" t="n">
+        <v>2736</v>
+      </c>
+      <c r="G665" t="n">
+        <v>6</v>
+      </c>
+      <c r="H665" t="b">
+        <v>0</v>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J665" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200670476</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J661"/>
+  <autoFilter ref="A1:J665"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 116, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$665</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$666</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J665"/>
+  <dimension ref="A1:J666"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27525,8 +27525,49 @@
         </is>
       </c>
     </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>1213121913</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>bismore</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>トロメルトクレンジング(150ml)</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>Bismore</t>
+        </is>
+      </c>
+      <c r="F666" t="n">
+        <v>4620</v>
+      </c>
+      <c r="G666" t="n">
+        <v>0</v>
+      </c>
+      <c r="H666" t="b">
+        <v>0</v>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J666" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213121913</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J665"/>
+  <autoFilter ref="A1:J666"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 118, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$673</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$675</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J673"/>
+  <dimension ref="A1:J675"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27853,8 +27853,90 @@
         </is>
       </c>
     </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>1171264782</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>benevolencejp</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>【百貨店ブランド】2本入り/スキンケアミスト/ 保湿 / 乾燥肌 / LUMINARIVA</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>Laguna Beauté</t>
+        </is>
+      </c>
+      <c r="F674" t="n">
+        <v>6930</v>
+      </c>
+      <c r="G674" t="n">
+        <v>1</v>
+      </c>
+      <c r="H674" t="b">
+        <v>0</v>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J674" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171264782</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>1171214421</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>benevolencejp</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>ボタニカルピールLevel7 ~2ヶ月セット(2回分)~</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>BOTANICAL PEEL</t>
+        </is>
+      </c>
+      <c r="F675" t="n">
+        <v>7976</v>
+      </c>
+      <c r="G675" t="n">
+        <v>7</v>
+      </c>
+      <c r="H675" t="b">
+        <v>0</v>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J675" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171214421</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J673"/>
+  <autoFilter ref="A1:J675"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 128, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$675</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$676</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J675"/>
+  <dimension ref="A1:J676"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27935,8 +27935,49 @@
         </is>
       </c>
     </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>872744432</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>nagomisabo</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>アルガンオイル 精製 オーガニック アルミパウチ 200ml リファインド / スタイリングオイル スタイリング キャリアオイル 100% マッサージオイル 美容オイル スキンケア ヘアオイル</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>naturalshop NAGOMI</t>
+        </is>
+      </c>
+      <c r="F676" t="n">
+        <v>3850</v>
+      </c>
+      <c r="G676" t="n">
+        <v>0</v>
+      </c>
+      <c r="H676" t="b">
+        <v>0</v>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J676" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=872744432</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J675"/>
+  <autoFilter ref="A1:J676"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 130, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$676</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$677</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J676"/>
+  <dimension ref="A1:J677"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27976,8 +27976,49 @@
         </is>
       </c>
     </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>1191178488</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>sangsanglabs</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>シャンプー1058ml＆トリートメント1058ml プレミアムヘアケアスペシャルセット(Baby Powder)</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F677" t="n">
+        <v>6400</v>
+      </c>
+      <c r="G677" t="n">
+        <v>0</v>
+      </c>
+      <c r="H677" t="b">
+        <v>0</v>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J677" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191178488</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J676"/>
+  <autoFilter ref="A1:J677"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 10)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$683</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$684</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J683"/>
+  <dimension ref="A1:J684"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28263,8 +28263,49 @@
         </is>
       </c>
     </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>1215131605</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Liveonkorea</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>[ニキビ跡ケア]トリプルレチノールポアアンプル 30ml/ニキビ / ニキビ跡 色素沈着/赤み / シミ / そばかす /ニキビ跡美容液/</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F684" t="n">
+        <v>4135</v>
+      </c>
+      <c r="G684" t="n">
+        <v>0</v>
+      </c>
+      <c r="H684" t="b">
+        <v>0</v>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J684" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1215131605</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J683"/>
+  <autoFilter ref="A1:J684"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 47, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$706</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$708</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J706"/>
+  <dimension ref="A1:J708"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29206,8 +29206,90 @@
         </is>
       </c>
     </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>1208116077</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>OHIROFFICIAL</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>【透けツヤ】ホワイトカメリアコア グロウリチュアル3点セット(化粧水/美容液/クリーム)</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>OHIR</t>
+        </is>
+      </c>
+      <c r="F707" t="n">
+        <v>10740</v>
+      </c>
+      <c r="G707" t="n">
+        <v>6</v>
+      </c>
+      <c r="H707" t="b">
+        <v>0</v>
+      </c>
+      <c r="I707" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J707" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208116077</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>1208116278</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>OHIROFFICIAL</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>【透けツヤフル】ホワイトカメリアコア コンプリートケア5点セット(洗顔フォーム/化粧水/美容液/クリーム/日焼け止め)</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>OHIR</t>
+        </is>
+      </c>
+      <c r="F708" t="n">
+        <v>14900</v>
+      </c>
+      <c r="G708" t="n">
+        <v>5</v>
+      </c>
+      <c r="H708" t="b">
+        <v>0</v>
+      </c>
+      <c r="I708" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J708" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208116278</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J706"/>
+  <autoFilter ref="A1:J708"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 59, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$718</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$722</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J718"/>
+  <dimension ref="A1:J722"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29698,8 +29698,172 @@
         </is>
       </c>
     </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>1162880522</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>lctradinghouse</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>速達便 税込SunsilkPower Shot Treatment Smooth Revival 治療スムーズリバイバル250Ml</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>sunsilk</t>
+        </is>
+      </c>
+      <c r="F719" t="n">
+        <v>4300</v>
+      </c>
+      <c r="G719" t="n">
+        <v>0</v>
+      </c>
+      <c r="H719" t="b">
+        <v>0</v>
+      </c>
+      <c r="I719" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J719" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162880522</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>1162882617</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>lctradinghouse</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>速達便 税込SunsilkPowerShotTreatment DamageRepairトリートメントダメージリペア250ml</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>sunsilk</t>
+        </is>
+      </c>
+      <c r="F720" t="n">
+        <v>4300</v>
+      </c>
+      <c r="G720" t="n">
+        <v>0</v>
+      </c>
+      <c r="H720" t="b">
+        <v>0</v>
+      </c>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J720" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162882617</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>1162491336</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>lctradinghouse</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>速達便 税込 Rexona (レクソーナ) Men Invisible + Antibacterial Roll On 男性インビジブル + 抗菌ロール オン 45ml x 5</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>レクソーナ</t>
+        </is>
+      </c>
+      <c r="F721" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G721" t="n">
+        <v>0</v>
+      </c>
+      <c r="H721" t="b">
+        <v>0</v>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J721" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162491336</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>809459822</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>lctradinghouse</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>速達便 税込 Rexona (レクソーナ) Men Quantum Dry Roll On メン量子ドライロールオン 45ml x 3</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>レクソーナ</t>
+        </is>
+      </c>
+      <c r="F722" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G722" t="n">
+        <v>1</v>
+      </c>
+      <c r="H722" t="b">
+        <v>0</v>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J722" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=809459822</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J718"/>
+  <autoFilter ref="A1:J722"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 77, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$732</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$733</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J732"/>
+  <dimension ref="A1:J733"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30272,8 +30272,49 @@
         </is>
       </c>
     </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>1165995217</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>songbyKbeauty486</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>ディープソルブ プランピングショットアンプル PDRN 植物性高麗人参 ハリ・ツヤケアエッセンス 30ml</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>deep solve</t>
+        </is>
+      </c>
+      <c r="F733" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G733" t="n">
+        <v>0</v>
+      </c>
+      <c r="H733" t="b">
+        <v>0</v>
+      </c>
+      <c r="I733" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J733" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165995217</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J732"/>
+  <autoFilter ref="A1:J733"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 46)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$771</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$773</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J771"/>
+  <dimension ref="A1:J773"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31871,8 +31871,90 @@
         </is>
       </c>
     </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>1114819772</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>skybottle</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>【公式】【韓国で大人気!】パフュームハンドクリーム 5種</t>
+        </is>
+      </c>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>スカイボトル</t>
+        </is>
+      </c>
+      <c r="F772" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G772" t="n">
+        <v>2</v>
+      </c>
+      <c r="H772" t="b">
+        <v>0</v>
+      </c>
+      <c r="I772" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J772" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1114819772</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>1087607248</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>skybottle</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>【セット商品】パフュームボディローション ボディウォッシュ セット3種から選択</t>
+        </is>
+      </c>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>スカイボトル</t>
+        </is>
+      </c>
+      <c r="F773" t="n">
+        <v>5600</v>
+      </c>
+      <c r="G773" t="n">
+        <v>4</v>
+      </c>
+      <c r="H773" t="b">
+        <v>0</v>
+      </c>
+      <c r="I773" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J773" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1087607248</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J771"/>
+  <autoFilter ref="A1:J773"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 13, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$781</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$782</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J781"/>
+  <dimension ref="A1:J782"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32281,8 +32281,49 @@
         </is>
       </c>
     </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>1212263577</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>niko66</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>NAKICO 薬用フェイスジェルクリーム 30g サラ肌 制汗 顔汗 メイク 仕上げ 崩れ防止 テカリ防止 フェイス クリーム</t>
+        </is>
+      </c>
+      <c r="E782" t="inlineStr">
+        <is>
+          <t>NAKICO</t>
+        </is>
+      </c>
+      <c r="F782" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G782" t="n">
+        <v>0</v>
+      </c>
+      <c r="H782" t="b">
+        <v>0</v>
+      </c>
+      <c r="I782" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J782" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212263577</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J781"/>
+  <autoFilter ref="A1:J782"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 14, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$784</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$789</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J784"/>
+  <dimension ref="A1:J789"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32404,8 +32404,213 @@
         </is>
       </c>
     </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>1193331149</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>kantanseries</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>カンタンシリーズ うるつや 90g メンズワックス ツヤ感 濡れ感</t>
+        </is>
+      </c>
+      <c r="E785" t="inlineStr">
+        <is>
+          <t>KANTAN SERIES</t>
+        </is>
+      </c>
+      <c r="F785" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G785" t="n">
+        <v>0</v>
+      </c>
+      <c r="H785" t="b">
+        <v>0</v>
+      </c>
+      <c r="I785" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J785" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193331149</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>1193332249</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>kantanseries</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>カンタンシリーズ うるたば 90g メンズワックス ツヤ感 セット力</t>
+        </is>
+      </c>
+      <c r="E786" t="inlineStr">
+        <is>
+          <t>KANTAN SERIES</t>
+        </is>
+      </c>
+      <c r="F786" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G786" t="n">
+        <v>3</v>
+      </c>
+      <c r="H786" t="b">
+        <v>0</v>
+      </c>
+      <c r="I786" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J786" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193332249</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>1208305015</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>kantanseries</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>KANTANSERIES カンタンシリーズ さらけあ 95g 洗い流さないトリートメント ホワイトリリー ヘアミルク</t>
+        </is>
+      </c>
+      <c r="E787" t="inlineStr">
+        <is>
+          <t>KANTAN SERIES</t>
+        </is>
+      </c>
+      <c r="F787" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G787" t="n">
+        <v>2</v>
+      </c>
+      <c r="H787" t="b">
+        <v>0</v>
+      </c>
+      <c r="I787" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J787" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208305015</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>1193331815</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>kantanseries</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>カンタンシリーズ ゆるたば 90g メンズワックス セミマット 操作性</t>
+        </is>
+      </c>
+      <c r="E788" t="inlineStr">
+        <is>
+          <t>KANTAN SERIES</t>
+        </is>
+      </c>
+      <c r="F788" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G788" t="n">
+        <v>2</v>
+      </c>
+      <c r="H788" t="b">
+        <v>0</v>
+      </c>
+      <c r="I788" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J788" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193331815</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>1193333122</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>kantanseries</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>カンタンシリーズ ニュアンス 90g ヘアバーム メンズ バーム ホワイトティー センターパート</t>
+        </is>
+      </c>
+      <c r="E789" t="inlineStr">
+        <is>
+          <t>KANTAN SERIES</t>
+        </is>
+      </c>
+      <c r="F789" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G789" t="n">
+        <v>3</v>
+      </c>
+      <c r="H789" t="b">
+        <v>0</v>
+      </c>
+      <c r="I789" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J789" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193333122</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J784"/>
+  <autoFilter ref="A1:J789"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 23, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$809</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$810</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J809"/>
+  <dimension ref="A1:J810"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33429,8 +33429,49 @@
         </is>
       </c>
     </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>1167854617</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>roomania</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>髪を洗うシャンプー　1000ml　チアパック</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>あんだんて</t>
+        </is>
+      </c>
+      <c r="F810" t="n">
+        <v>5190</v>
+      </c>
+      <c r="G810" t="n">
+        <v>0</v>
+      </c>
+      <c r="H810" t="b">
+        <v>0</v>
+      </c>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J810" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167854617</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J809"/>
+  <autoFilter ref="A1:J810"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 5 own-file progress (반복 30)
</commit_message>
<xml_diff>
--- a/output/discovery_result_5.xlsx
+++ b/output/discovery_result_5.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$811</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$813</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J811"/>
+  <dimension ref="A1:J813"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33511,8 +33511,90 @@
         </is>
       </c>
     </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>1205722924</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>falami</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>目元パック 男性[10回分/20枚] 大判サイズ ニードル ヒアルロン酸 パッチ目元 メンズ ニードルパッチ メンズパック クマ 取り パッチ マイクロニードルパッチ 目元ケアと口元眉間も対応 女性</t>
+        </is>
+      </c>
+      <c r="E812" t="inlineStr">
+        <is>
+          <t>Azizam</t>
+        </is>
+      </c>
+      <c r="F812" t="n">
+        <v>4998</v>
+      </c>
+      <c r="G812" t="n">
+        <v>1</v>
+      </c>
+      <c r="H812" t="b">
+        <v>0</v>
+      </c>
+      <c r="I812" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J812" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205722924</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>1206841476</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>falami</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>ニードル パッチ 30回分 美容グッズ 目元 パック ヒアルロン酸 パッチ レディース アイマスク 女性用 男性用 クマ 取り パッチ マイクロニードルパッチ 目元 ヒアルロン酸 パ</t>
+        </is>
+      </c>
+      <c r="E813" t="inlineStr">
+        <is>
+          <t>Falami</t>
+        </is>
+      </c>
+      <c r="F813" t="n">
+        <v>7633</v>
+      </c>
+      <c r="G813" t="n">
+        <v>3</v>
+      </c>
+      <c r="H813" t="b">
+        <v>0</v>
+      </c>
+      <c r="I813" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J813" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206841476</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J811"/>
+  <autoFilter ref="A1:J813"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>